<commit_message>
Add eligibility/templates checklist and four-stage roadmap; fix essential criteria count to 14
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -63,7 +63,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2767" uniqueCount="556">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="2760" uniqueCount="556">
   <si>
     <t xml:space="preserve">خطة عمل لجنة الاعتماد البرامجي – المرحلة الأولى: التحقق من الأدلة وجودتها وتحديد الفجوات</t>
   </si>
@@ -206,7 +206,7 @@
     <t xml:space="preserve">عمود نتيجة المراجعة مكتمل</t>
   </si>
   <si>
-    <t xml:space="preserve">مراجعة رئيس اللجنة لأدلة المعايير الأساسية الـ15 في البرنامجين</t>
+    <t xml:space="preserve">مراجعة رئيس اللجنة لأدلة المعايير الأساسية الـ14 في البرنامجين</t>
   </si>
   <si>
     <t xml:space="preserve">اعتماد نتائج المعايير الأساسية</t>
@@ -269,7 +269,7 @@
     <t xml:space="preserve">• "الدليل غير الموجود في المستودع غير موجود": لا يُعتمد أي دليل لم يُرفع ويُربط برمزه في ورقة الفحص.</t>
   </si>
   <si>
-    <t xml:space="preserve">• التركيز أولاً على المعايير الأساسية الـ15، لأن عدم استيفاء أي منها يؤثر مباشرة في قرار الاعتماد.</t>
+    <t xml:space="preserve">• التركيز أولاً على المعايير الأساسية الـ14، لأن عدم استيفاء أي منها يؤثر مباشرة في قرار الاعتماد.</t>
   </si>
   <si>
     <t xml:space="preserve">• الفصل بين "غياب الدليل" و"ضعف جودته": كثير من الفجوات تكون في التطبيق وإغلاق الحلقة لا في وجود السياسة.</t>
@@ -338,7 +338,7 @@
     <t xml:space="preserve">البرنامجان</t>
   </si>
   <si>
-    <t xml:space="preserve">قيادة اللجنة واعتماد المخرجات، المتابعة الأسبوعية، فحص محور جودة التدريس وتقييم الطالب (2-3) في البرنامجين، مراجعة المعايير الأساسية الـ15، والتواصل مع عمادة الجودة والإدارة العليا</t>
+    <t xml:space="preserve">قيادة اللجنة واعتماد المخرجات، المتابعة الأسبوعية، فحص محور جودة التدريس وتقييم الطالب (2-3) في البرنامجين، مراجعة المعايير الأساسية الـ14، والتواصل مع عمادة الجودة والإدارة العليا</t>
   </si>
   <si>
     <t xml:space="preserve">عضو 2</t>
@@ -455,7 +455,7 @@
     <t xml:space="preserve">• يفحص كل عضو أدلة برنامجه، ثم يراجعها زميله من البرنامج الآخر (مراجعة متقاطعة) لضمان الموضوعية وتوحيد الحكم بين البرنامجين.</t>
   </si>
   <si>
-    <t xml:space="preserve">• يراجع رئيس اللجنة جميع أدلة المعايير الأساسية الـ15 (المظللة بالأصفر) في البرنامجين قبل اعتماد نتائج الفحص.</t>
+    <t xml:space="preserve">• يراجع رئيس اللجنة جميع أدلة المعايير الأساسية الـ14 (المظللة بالأصفر) في البرنامجين قبل اعتماد نتائج الفحص.</t>
   </si>
   <si>
     <t xml:space="preserve">• يمكن تعديل الأسماء في عمود "مسؤول الفحص" أو "المراجع" باختيار عضو آخر – تأكد من مطابقة الاسم لجدول الأعضاء أعلاه.</t>
@@ -509,7 +509,7 @@
     <t xml:space="preserve">5. مصادر التعلم والمرافق والتجهيزات</t>
   </si>
   <si>
-    <t xml:space="preserve">المعايير الأساسية (15 معياراً)</t>
+    <t xml:space="preserve">المعايير الأساسية (14 معياراً)</t>
   </si>
   <si>
     <t xml:space="preserve">الإجمالي</t>
@@ -5198,7 +5198,7 @@
       </c>
       <c r="B19" s="20" t="n">
         <f aca="false">COUNTIFS('فحص-البرنامج1'!$E:$E,"نعم")</f>
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C19" s="20" t="n">
         <f aca="false">COUNTIFS('فحص-البرنامج1'!$E:$E,"نعم",'فحص-البرنامج1'!$I:$I,"&lt;&gt;")</f>
@@ -5860,7 +5860,7 @@
       </c>
       <c r="B37" s="20" t="n">
         <f aca="false">COUNTIFS('فحص-البرنامج2'!$E:$E,"نعم")</f>
-        <v>66</v>
+        <v>63</v>
       </c>
       <c r="C37" s="20" t="n">
         <f aca="false">COUNTIFS('فحص-البرنامج2'!$E:$E,"نعم",'فحص-البرنامج2'!$I:$I,"&lt;&gt;")</f>
@@ -5957,7 +5957,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{3411FFE9-80F8-4866-83C4-DDA32B46E089}</x14:id>
+          <x14:id>{DB32ECA1-C8B3-4F75-9D15-AD19277E62FC}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5971,7 +5971,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{365881EA-91ED-48DC-BDFF-82A7BB86653A}</x14:id>
+          <x14:id>{75D220ED-B6BD-40A7-A74D-60F3B44020F0}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5985,7 +5985,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{8650EE63-CA60-4B78-B25E-A1D87E4E213E}</x14:id>
+          <x14:id>{DADDFE67-8AD2-46B7-8AAF-E0DD4078DA91}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5999,7 +5999,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{AD83876B-1824-46A6-8DE9-6D26F1B03E23}</x14:id>
+          <x14:id>{67EA376F-84FC-4E96-9FE9-DB1A3077E097}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -6015,7 +6015,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{3411FFE9-80F8-4866-83C4-DDA32B46E089}">
+          <x14:cfRule type="dataBar" id="{DB32ECA1-C8B3-4F75-9D15-AD19277E62FC}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6030,7 +6030,7 @@
           <xm:sqref>D6:D20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{365881EA-91ED-48DC-BDFF-82A7BB86653A}">
+          <x14:cfRule type="dataBar" id="{75D220ED-B6BD-40A7-A74D-60F3B44020F0}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6045,7 +6045,7 @@
           <xm:sqref>H6:H20</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{8650EE63-CA60-4B78-B25E-A1D87E4E213E}">
+          <x14:cfRule type="dataBar" id="{DADDFE67-8AD2-46B7-8AAF-E0DD4078DA91}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -6060,7 +6060,7 @@
           <xm:sqref>D24:D38</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{AD83876B-1824-46A6-8DE9-6D26F1B03E23}">
+          <x14:cfRule type="dataBar" id="{67EA376F-84FC-4E96-9FE9-DB1A3077E097}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -13995,25 +13995,23 @@
       <c r="W136" s="30"/>
     </row>
     <row r="137" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="31" t="s">
+      <c r="A137" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B137" s="32" t="s">
+      <c r="B137" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C137" s="32" t="s">
+      <c r="C137" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D137" s="32" t="s">
+      <c r="D137" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E137" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F137" s="31" t="n">
+      <c r="E137" s="27"/>
+      <c r="F137" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G137" s="32" t="s">
+      <c r="G137" s="28" t="s">
         <v>434</v>
       </c>
       <c r="H137" s="27" t="str">
@@ -14052,25 +14050,23 @@
       <c r="W137" s="30"/>
     </row>
     <row r="138" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="31" t="s">
+      <c r="A138" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B138" s="32" t="s">
+      <c r="B138" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C138" s="32" t="s">
+      <c r="C138" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D138" s="32" t="s">
+      <c r="D138" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E138" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F138" s="31" t="n">
+      <c r="E138" s="27"/>
+      <c r="F138" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="G138" s="32" t="s">
+      <c r="G138" s="28" t="s">
         <v>435</v>
       </c>
       <c r="H138" s="27" t="str">
@@ -14109,25 +14105,23 @@
       <c r="W138" s="30"/>
     </row>
     <row r="139" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="31" t="s">
+      <c r="A139" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B139" s="32" t="s">
+      <c r="B139" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C139" s="32" t="s">
+      <c r="C139" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D139" s="32" t="s">
+      <c r="D139" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E139" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F139" s="31" t="n">
+      <c r="E139" s="27"/>
+      <c r="F139" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="G139" s="32" t="s">
+      <c r="G139" s="28" t="s">
         <v>436</v>
       </c>
       <c r="H139" s="27" t="str">
@@ -25531,25 +25525,23 @@
       <c r="W136" s="30"/>
     </row>
     <row r="137" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A137" s="31" t="s">
+      <c r="A137" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B137" s="32" t="s">
+      <c r="B137" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C137" s="32" t="s">
+      <c r="C137" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D137" s="32" t="s">
+      <c r="D137" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E137" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F137" s="31" t="n">
+      <c r="E137" s="27"/>
+      <c r="F137" s="27" t="n">
         <v>1</v>
       </c>
-      <c r="G137" s="32" t="s">
+      <c r="G137" s="28" t="s">
         <v>434</v>
       </c>
       <c r="H137" s="27" t="str">
@@ -25588,25 +25580,23 @@
       <c r="W137" s="30"/>
     </row>
     <row r="138" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A138" s="31" t="s">
+      <c r="A138" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B138" s="32" t="s">
+      <c r="B138" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C138" s="32" t="s">
+      <c r="C138" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D138" s="32" t="s">
+      <c r="D138" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E138" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F138" s="31" t="n">
+      <c r="E138" s="27"/>
+      <c r="F138" s="27" t="n">
         <v>2</v>
       </c>
-      <c r="G138" s="32" t="s">
+      <c r="G138" s="28" t="s">
         <v>435</v>
       </c>
       <c r="H138" s="27" t="str">
@@ -25645,25 +25635,23 @@
       <c r="W138" s="30"/>
     </row>
     <row r="139" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A139" s="31" t="s">
+      <c r="A139" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B139" s="32" t="s">
+      <c r="B139" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C139" s="32" t="s">
+      <c r="C139" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D139" s="32" t="s">
+      <c r="D139" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E139" s="31" t="s">
-        <v>185</v>
-      </c>
-      <c r="F139" s="31" t="n">
+      <c r="E139" s="27"/>
+      <c r="F139" s="27" t="n">
         <v>3</v>
       </c>
-      <c r="G139" s="32" t="s">
+      <c r="G139" s="28" t="s">
         <v>436</v>
       </c>
       <c r="H139" s="27" t="str">
@@ -31567,21 +31555,19 @@
       </c>
     </row>
     <row r="36" customFormat="false" ht="22.35" hidden="false" customHeight="false" outlineLevel="0" collapsed="false">
-      <c r="A36" s="31" t="s">
+      <c r="A36" s="27" t="s">
         <v>432</v>
       </c>
-      <c r="B36" s="32" t="s">
+      <c r="B36" s="28" t="s">
         <v>145</v>
       </c>
-      <c r="C36" s="32" t="s">
+      <c r="C36" s="28" t="s">
         <v>125</v>
       </c>
-      <c r="D36" s="32" t="s">
+      <c r="D36" s="28" t="s">
         <v>433</v>
       </c>
-      <c r="E36" s="31" t="s">
-        <v>185</v>
-      </c>
+      <c r="E36" s="27"/>
       <c r="F36" s="27" t="n">
         <f aca="false">COUNTIFS('فحص-البرنامج1'!$A:$A,A36,'فحص-البرنامج1'!$I:$I,"&lt;&gt;")</f>
         <v>0</v>
@@ -32623,7 +32609,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{922BDDB1-4797-4E65-8CCA-B0C170DA1626}</x14:id>
+          <x14:id>{59BAD8C7-5C00-41A8-9FA0-FF7E70A38CEE}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -32637,7 +32623,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{295D2BC7-9EFA-4EE2-A139-B55C4EF01D2B}</x14:id>
+          <x14:id>{6AA0E8BF-7DA3-4F34-ADE4-7E4053DA5CFB}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -32654,7 +32640,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{922BDDB1-4797-4E65-8CCA-B0C170DA1626}">
+          <x14:cfRule type="dataBar" id="{59BAD8C7-5C00-41A8-9FA0-FF7E70A38CEE}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -32669,7 +32655,7 @@
           <xm:sqref>I5:I52</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{295D2BC7-9EFA-4EE2-A139-B55C4EF01D2B}">
+          <x14:cfRule type="dataBar" id="{6AA0E8BF-7DA3-4F34-ADE4-7E4053DA5CFB}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>

</xml_diff>

<commit_message>
Requirements: no documents to fetch for graduates and institutional status
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -32,7 +32,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3335" uniqueCount="645">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="3337" uniqueCount="645">
   <si>
     <t xml:space="preserve">خطة المرحلة الأولى للاعتماد البرامجي: جمع الأدلة وتحديد الفجوات</t>
   </si>
@@ -592,10 +592,13 @@
     <t xml:space="preserve">تخرّج دفعة واحدة على الأقل من البرنامج</t>
   </si>
   <si>
-    <t xml:space="preserve">محقق – يُجلب الدليل</t>
-  </si>
-  <si>
-    <t xml:space="preserve">إحصاء الخريجين لكل برنامج مع سنة تخرج أول دفعة</t>
+    <t xml:space="preserve">محقق</t>
+  </si>
+  <si>
+    <t xml:space="preserve">—</t>
+  </si>
+  <si>
+    <t xml:space="preserve">تخرّجت دفعات من البرامج الثلاثة</t>
   </si>
   <si>
     <t xml:space="preserve">متطلبات التقدم</t>
@@ -646,9 +649,6 @@
     <t xml:space="preserve">المرحلة التالية بعد الخطة</t>
   </si>
   <si>
-    <t xml:space="preserve">—</t>
-  </si>
-  <si>
     <t xml:space="preserve">تُكتب بعد جمع الأدلة ومعالجة الفجوات</t>
   </si>
   <si>
@@ -694,7 +694,7 @@
     <t xml:space="preserve">المؤسسة معتمدة أو مؤهلة مؤسسياً</t>
   </si>
   <si>
-    <t xml:space="preserve">الجامعة حاصلة على الاعتماد المؤسسي الكامل – يُجلب قرار الاعتماد مع تاريخ صلاحيته</t>
+    <t xml:space="preserve">الجامعة حاصلة على الاعتماد المؤسسي الكامل</t>
   </si>
   <si>
     <t xml:space="preserve">نموذج مقترح: مراجعة رسالة البرنامج وأهدافه (للنقاش في اللجنة)</t>
@@ -5333,7 +5333,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{E1E33025-2DCB-47B1-8F4D-5E2541228D92}</x14:id>
+          <x14:id>{3385169E-CA70-4B7D-8470-29DC1E962E10}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5347,7 +5347,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{2AA22E18-42A8-4EE3-BED2-DFBF8F14E14B}</x14:id>
+          <x14:id>{BFE9761E-F0C6-40F7-997F-A4177A875D6C}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5361,7 +5361,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{5A73AB9B-1768-4BF1-8797-E000335B7390}</x14:id>
+          <x14:id>{89BBA577-6837-4B9C-B61B-62FF5024EAF4}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5375,7 +5375,7 @@
       </dataBar>
       <extLst>
         <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{B025F937-C7B1-47D3-B67F-A62EFF666E3E}">
-          <x14:id>{6F954580-B19D-4EB6-A51F-F169E0C100BA}</x14:id>
+          <x14:id>{5FB871AB-4E2D-48DD-9AE0-C8FD87A9AD7D}</x14:id>
         </ext>
       </extLst>
     </cfRule>
@@ -5391,7 +5391,7 @@
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{78C0D931-6437-407d-A8EE-F0AAD7539E65}">
       <x14:conditionalFormattings>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{E1E33025-2DCB-47B1-8F4D-5E2541228D92}">
+          <x14:cfRule type="dataBar" id="{3385169E-CA70-4B7D-8470-29DC1E962E10}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5406,7 +5406,7 @@
           <xm:sqref>G6:G12</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{2AA22E18-42A8-4EE3-BED2-DFBF8F14E14B}">
+          <x14:cfRule type="dataBar" id="{BFE9761E-F0C6-40F7-997F-A4177A875D6C}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5421,7 +5421,7 @@
           <xm:sqref>G16:G22</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{5A73AB9B-1768-4BF1-8797-E000335B7390}">
+          <x14:cfRule type="dataBar" id="{89BBA577-6837-4B9C-B61B-62FF5024EAF4}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5436,7 +5436,7 @@
           <xm:sqref>G26:G33</xm:sqref>
         </x14:conditionalFormatting>
         <x14:conditionalFormatting xmlns:xm="http://schemas.microsoft.com/office/excel/2006/main">
-          <x14:cfRule type="dataBar" id="{6F954580-B19D-4EB6-A51F-F169E0C100BA}">
+          <x14:cfRule type="dataBar" id="{5FB871AB-4E2D-48DD-9AE0-C8FD87A9AD7D}">
             <x14:dataBar minLength="10" maxLength="90" axisPosition="none" gradient="true">
               <x14:cfvo type="num">
                 <xm:f>0</xm:f>
@@ -5556,17 +5556,16 @@
       <c r="D7" s="11" t="s">
         <v>186</v>
       </c>
-      <c r="E7" s="7" t="str">
-        <f aca="false">'الإعدادات واللجنة'!$B$12</f>
-        <v>د. نهلة بنت سعد القثامي</v>
+      <c r="E7" s="7" t="s">
+        <v>187</v>
       </c>
       <c r="F7" s="6" t="s">
-        <v>187</v>
+        <v>188</v>
       </c>
     </row>
     <row r="8" customFormat="false" ht="15" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
       <c r="A8" s="13" t="s">
-        <v>188</v>
+        <v>189</v>
       </c>
       <c r="B8" s="13"/>
       <c r="C8" s="13"/>
@@ -5579,20 +5578,20 @@
         <v>3</v>
       </c>
       <c r="B9" s="18" t="s">
-        <v>189</v>
+        <v>190</v>
       </c>
       <c r="C9" s="6" t="s">
-        <v>190</v>
+        <v>191</v>
       </c>
       <c r="D9" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E9" s="7" t="str">
         <f aca="false">'الإعدادات واللجنة'!$B$13</f>
         <v>د. عبير بنت عبدالله راجحي</v>
       </c>
       <c r="F9" s="6" t="s">
-        <v>192</v>
+        <v>193</v>
       </c>
     </row>
     <row r="10" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5600,20 +5599,20 @@
         <v>4</v>
       </c>
       <c r="B10" s="18" t="s">
-        <v>193</v>
+        <v>194</v>
       </c>
       <c r="C10" s="6" t="s">
-        <v>194</v>
+        <v>195</v>
       </c>
       <c r="D10" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E10" s="7" t="str">
         <f aca="false">'الإعدادات واللجنة'!$B$13</f>
         <v>د. عبير بنت عبدالله راجحي</v>
       </c>
       <c r="F10" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="11" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5621,20 +5620,20 @@
         <v>5</v>
       </c>
       <c r="B11" s="18" t="s">
-        <v>196</v>
+        <v>197</v>
       </c>
       <c r="C11" s="6" t="s">
-        <v>197</v>
+        <v>198</v>
       </c>
       <c r="D11" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E11" s="7" t="str">
         <f aca="false">'الإعدادات واللجنة'!$B$13</f>
         <v>د. عبير بنت عبدالله راجحي</v>
       </c>
       <c r="F11" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="12" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5645,17 +5644,17 @@
         <v>129</v>
       </c>
       <c r="C12" s="6" t="s">
-        <v>198</v>
+        <v>199</v>
       </c>
       <c r="D12" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E12" s="7" t="str">
         <f aca="false">'الإعدادات واللجنة'!$B$13</f>
         <v>د. عبير بنت عبدالله راجحي</v>
       </c>
       <c r="F12" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="13" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5663,20 +5662,20 @@
         <v>7</v>
       </c>
       <c r="B13" s="18" t="s">
-        <v>199</v>
+        <v>200</v>
       </c>
       <c r="C13" s="6" t="s">
-        <v>200</v>
+        <v>201</v>
       </c>
       <c r="D13" s="12" t="s">
-        <v>191</v>
+        <v>192</v>
       </c>
       <c r="E13" s="7" t="str">
         <f aca="false">'الإعدادات واللجنة'!$B$13</f>
         <v>د. عبير بنت عبدالله راجحي</v>
       </c>
       <c r="F13" s="6" t="s">
-        <v>195</v>
+        <v>196</v>
       </c>
     </row>
     <row r="14" customFormat="false" ht="31.5" hidden="false" customHeight="true" outlineLevel="0" collapsed="false">
@@ -5684,16 +5683,16 @@
         <v>8</v>
       </c>
       <c r="B14" s="18" t="s">
-        <v>201</v>
+        <v>202</v>
       </c>
       <c r="C14" s="6" t="s">
-        <v>202</v>
+        <v>203</v>
       </c>
       <c r="D14" s="5" t="s">
-        <v>203</v>
+        <v>204</v>
       </c>
       <c r="E14" s="7" t="s">
-        <v>204</v>
+        <v>187</v>
       </c>
       <c r="F14" s="6" t="s">
         <v>205</v>
@@ -5778,11 +5777,10 @@
         <v>219</v>
       </c>
       <c r="D19" s="11" t="s">
-        <v>182</v>
-      </c>
-      <c r="E19" s="7" t="str">
-        <f aca="false">'الإعدادات واللجنة'!$B$12</f>
-        <v>د. نهلة بنت سعد القثامي</v>
+        <v>186</v>
+      </c>
+      <c r="E19" s="7" t="s">
+        <v>187</v>
       </c>
       <c r="F19" s="6" t="s">
         <v>220</v>

</xml_diff>

<commit_message>
Std-6 proposed evidence approved by Dr. Hassan instead of quality head
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -278,7 +278,7 @@
     <t>ملاحظة عن الماجستير</t>
   </si>
   <si>
-    <t>• يُقيَّم وفق معايير الدراسات العليا 2022 (56 محكاً منها 16 أساسياً، ومعيار سادس للبحث والمشاريع). أدلة المحكات المشتركة مأخوذة من دليل البكالوريوس، وأدلة المعيار 6 مقترحة ومعلّمة باللون الأحمر وتعتمدها رئيسة الجودة. ترقيم المحكات موحّد بالترتيب المعتاد (مثل 1-1-2).</t>
+    <t>• يُقيَّم وفق معايير الدراسات العليا 2022 (56 محكاً منها 16 أساسياً، ومعيار سادس للبحث والمشاريع). أدلة المحكات المشتركة مأخوذة من دليل البكالوريوس، وأدلة المعيار 6 مقترحة ومعلّمة باللون الأحمر ويعتمدها د. حسن القحطاني. ترقيم المحكات موحّد بالترتيب المعتاد (مثل 1-1-2).</t>
   </si>
   <si>
     <t>الإعدادات وتشكيل لجنة الاعتماد البرامجي</t>
@@ -344,7 +344,7 @@
     <t>رئيسة الجودة</t>
   </si>
   <si>
-    <t>متطلبات التقدم مع لجنة الجودة (التوصيفات، والتقارير السنوية، والإطار الوطني، ونواتج التعلم، ومؤشرات الأداء) وعرض حالتها في الأسبوعين 4 و7؛ واعتماد الأدلة المقترحة لمعيار البحث في الماجستير</t>
+    <t>متطلبات التقدم مع لجنة الجودة (التوصيفات، والتقارير السنوية، والإطار الوطني، ونواتج التعلم، ومؤشرات الأداء) وعرض حالتها في الأسبوعين 4 و7</t>
   </si>
   <si>
     <t>أ. فاطمة بنت سلمان الخزعل</t>
@@ -395,7 +395,7 @@
     <t>د. حسن بن سعد القحطاني</t>
   </si>
   <si>
-    <t>المعيار 5: مصادر التعلم والمرافق، ومحور ضمان الجودة (1-2) للبرامج الثلاثة</t>
+    <t>المعيار 5: مصادر التعلم والمرافق، ومحور ضمان الجودة (1-2) للبرامج الثلاثة، واعتماد الأدلة المقترحة لمعيار البحث (6) في الماجستير</t>
   </si>
   <si>
     <t>توزيع المحاور (المسؤول عن المحور للبرامج الثلاثة) – يمكن تغيير المسؤول من القائمة المنسدلة</t>
@@ -1817,7 +1817,7 @@
     <t>خطة البحث العلمي للبرنامج مرتبطة بالخطة البحثية للمؤسسة.</t>
   </si>
   <si>
-    <t>مقترح – يعتمده رئيسة الجودة</t>
+    <t>مقترح – يعتمده د. حسن القحطاني</t>
   </si>
   <si>
     <t>تقرير سنوي عن النشاط البحثي ومؤشراته (KPI-PG-9 إلى KPI-PG-13) مع المقارنة المرجعية.</t>
@@ -2964,15 +2964,15 @@
       <c r="A9" s="11" t="s">
         <v>21</v>
       </c>
-      <c r="B9" s="19" t="s">
-        <v>22</v>
+      <c r="B9" s="17" t="s">
+        <v>12</v>
       </c>
       <c r="C9" s="13" t="s">
         <v>23</v>
       </c>
       <c r="D9" s="14" t="str">
-        <f>'الإعدادات واللجنة'!$B$13</f>
-        <v>د. عبير بنت عبدالله راجحي</v>
+        <f>'الإعدادات واللجنة'!$B$20</f>
+        <v>د. حسن بن سعد القحطاني</v>
       </c>
       <c r="E9" s="13" t="s">
         <v>24</v>

</xml_diff>

<commit_message>
Explain the Thursday status message in the plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -233,7 +233,12 @@
     <t>• ملف مشترك (OneDrive / Google Drive): يعبّئ كل عضو ورقته مباشرة، ولوحة المتابعة تتحدث تلقائياً.</t>
   </si>
   <si>
-    <t>• رسالة الخميس: ترسل أمينة اللجنة 3 أسطر في قروب اللجنة: نسبة الإنجاز لكل برنامج، ومن تأخر، وما يحتاج قراراً.</t>
+    <t xml:space="preserve">• رسالة الخميس (بديل الاجتماع الأسبوعي): ترسلها أمينة اللجنة كل خميس في قروب اللجنة، وتأخذ أرقامها من ورقة "لوحة المتابعة" دون حساب يدوي. وتتضمن:
+   ① نسبة الإنجاز لكل برنامج: نسبة الأدلة المقيَّمة ونسبة المكتمل منها.
+   ② ما يحتاج متابعة: العضو المتأخر في إنجازه، وعدد الأدلة التي تحتاج تعديلاً بعد المراجعة.
+   ③ ما يحتاج قراراً من الرئيسة أو اللجنة.
+   ④ مهام الأسبوع القادم حسب الخطة.
+   الهدف: أن تعرف الرئيسة الوضع أسبوعياً وتتدخل عند الحاجة فقط، وألا تتراكم القرارات المعلّقة.</t>
   </si>
   <si>
     <t>• 3 اجتماعات للجنة عند المحطات: الانطلاق (الأسبوع 1)، ومنتصف الخطة (الأسبوع 4)، ومناقشة الفجوات (الأسبوع 7).</t>
@@ -3285,7 +3290,7 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" ht="15" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="118" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>

</xml_diff>

<commit_message>
Weekly message: progress and handling challenges
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -233,12 +233,7 @@
     <t>• ملف مشترك (OneDrive / Google Drive): يعبّئ كل عضو ورقته مباشرة، ولوحة المتابعة تتحدث تلقائياً.</t>
   </si>
   <si>
-    <t xml:space="preserve">• رسالة الخميس (بديل الاجتماع الأسبوعي): ترسلها أمينة اللجنة كل خميس في قروب اللجنة، وتأخذ أرقامها من ورقة "لوحة المتابعة" دون حساب يدوي. وتتضمن:
-   ① نسبة الإنجاز لكل برنامج: نسبة الأدلة المقيَّمة ونسبة المكتمل منها.
-   ② ما يحتاج متابعة: العضو المتأخر في إنجازه، وعدد الأدلة التي تحتاج تعديلاً بعد المراجعة.
-   ③ ما يحتاج قراراً من الرئيسة أو اللجنة.
-   ④ مهام الأسبوع القادم حسب الخطة.
-   الهدف: أن تعرف الرئيسة الوضع أسبوعياً وتتدخل عند الحاجة فقط، وألا تتراكم القرارات المعلّقة.</t>
+    <t xml:space="preserve">• الرسالة الأسبوعية (كل خميس): ترسلها أمينة اللجنة في قروب اللجنة، وتوضح فيها نسبة الإنجاز لكل برنامج (من ورقة "لوحة المتابعة") ومعالجة أي تحديات تواجه الأعضاء، ومن لديه استفسار أو تردد في أي دليل يتواصل مع الرئيسة أو الأمينة.</t>
   </si>
   <si>
     <t>• 3 اجتماعات للجنة عند المحطات: الانطلاق (الأسبوع 1)، ومنتصف الخطة (الأسبوع 4)، ومناقشة الفجوات (الأسبوع 7).</t>
@@ -3290,7 +3285,7 @@
       <c r="F25" s="6"/>
       <c r="G25" s="6"/>
     </row>
-    <row r="26" spans="1:7" ht="118" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="26" spans="1:7" ht="34" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A26" s="6" t="s">
         <v>61</v>
       </c>

</xml_diff>

<commit_message>
Plan: evidence examination mechanism in committee's wording plus sheet workflow steps
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -3580,7 +3580,7 @@
     <row r="32" spans="1:7" ht="42.75" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A32" s="66" t="inlineStr">
         <is>
-          <t xml:space="preserve">آلية تقييم الدليل (في ورقة فحص كل برنامج)</t>
+          <t xml:space="preserve">آلية فحص الأدلة</t>
         </is>
       </c>
       <c r="B32" s="66"/>
@@ -3590,14 +3590,15 @@
       <c r="F32" s="66"/>
       <c r="G32" s="66"/>
     </row>
-    <row r="33" spans="1:7" ht="112" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="33" spans="1:7" ht="125" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A33" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">1. يصفّي العضو عمود "المسؤول" على اسمه، فتظهر أدلته فقط.
-2. يرفع الدليل للمستودع بالترميز المعتمد، ويضع رابطه في عمود "رابط الدليل".
-3. يختار "حالة الدليل": متوفر ومكتمل • متوفر ويحتاج تحسين • غير متوفر.
-4. إذا لم يكن مكتملاً يختار "سبب النقص" الرئيسي: غير معتمد • غير محدّث • لا يغطي المحك كاملاً • لا يثبت التطبيق الفعلي • لا توجد نتائج وتحسين.
-5. تظهر "الأولوية" تلقائياً: عالية إذا كان الدليل غير متوفر أو المحك أساسياً ★، ومتوسطة لغير ذلك.</t>
+          <t xml:space="preserve">يقوم كل عضو بمراجعة الأدلة المرتبطة بالمعيار المسند إليه، والتحقق من مدى كفايتها لإثبات استيفاء المحك، وذلك وفق الآتي:
+1. توفر الدليل: التحقق من وجود الدليل المطلوب.
+2. الاعتماد: التحقق من أن الدليل معتمد من الجهة المختصة، متى ما كان الاعتماد مطلوبًا.
+3. الحداثة: التحقق من أن الدليل محدث ويعكس الوضع الحالي للبرنامج والفترة المطلوبة.
+4. الارتباط بالمحك: التأكد من أن الدليل يغطي متطلبات المحك بصورة مباشرة وكافية.
+5. إثبات التطبيق: التحقق من أن الدليل يثبت التطبيق الفعلي، ولا يقتصر على وجود سياسة أو نموذج فقط، وأن نتائج القياس استُخدمت في التحسين، متى ما كان المحك يتطلب ذلك.</t>
         </is>
       </c>
       <c r="B33" s="67"/>
@@ -3607,13 +3608,14 @@
       <c r="F33" s="67"/>
       <c r="G33" s="67"/>
     </row>
-    <row r="34" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="34" spans="1:7" ht="90" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A34" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">6. يكتب في الوقت نفسه "الإجراء المطلوب" مع الجهة التي ستستكمل الدليل، ويختار "الموعد" (أسبوع من الخطة أو "بعد الخطة")، وتُراجع خطة الاستكمال وتُعتمد في اجتماع الأسبوع 7.
-7. تراجع أمينة اللجنة الأدلة أسبوعياً وتختار في عمود "مراجعة أ. فاطمة": تمت • تحتاج تعديل، مع ملاحظتها، ويعالج العضو ما يحتاج تعديلاً.
-8. تراجع رئيسة اللجنة كفاية أدلة المحكات الأساسية ★ في الأسبوع 6.
-9. تتحدث "لوحة المتابعة" تلقائياً مع كل إدخال.</t>
+          <t xml:space="preserve">تصنيف حالة الدليل:
+• متوفر ومكتمل: مستوفٍ لمتطلبات الفحص أعلاه.
+• متوفر ويحتاج تحسين: الدليل موجود، إلا أنه يحتاج إلى استكمال أو تحديث أو اعتماد أو تعزيز بما يثبت التطبيق.
+• غير متوفر: لم يتم العثور على دليل يثبت استيفاء المتطلب.
+وعند وجود نقص، يتم توضيح سبب النقص والإجراء المطلوب لاستكمال الدليل ضمن ورقة الفحص.</t>
         </is>
       </c>
       <c r="B34" s="67"/>
@@ -3623,10 +3625,14 @@
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
     </row>
-    <row r="35" spans="1:7" ht="24" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="67" t="inlineStr">
         <is>
-          <t xml:space="preserve">• الدليل المكتمل: معتمد، ومحدّث، ويغطي المحك كاملاً، ويثبت التطبيق الفعلي، وفيه نتائج وتحسين.</t>
+          <t xml:space="preserve">خطوات العمل في ورقة الفحص:
+1. يصفّي العضو عمود "المسؤول" على اسمه، ويرفع كل دليل للمستودع بالترميز المعتمد ويضع رابطه.
+2. يختار "حالة الدليل"، وإن لم يكن مكتملاً يختار "سبب النقص" ويكتب "الإجراء المطلوب" والجهة التي ستستكمله ويختار "الموعد". وتظهر "الأولوية" تلقائياً.
+3. تراجع أمينة اللجنة الأدلة أسبوعياً (تمت • تحتاج تعديل)، وتراجع رئيسة اللجنة كفاية أدلة المحكات الأساسية ★ في الأسبوع 6.
+4. تُراجع خطة الاستكمال وتُعتمد في اجتماع الأسبوع 7، وتتحدث "لوحة المتابعة" تلقائياً مع كل إدخال.</t>
         </is>
       </c>
       <c r="B35" s="67"/>

</xml_diff>

<commit_message>
Gap reasons: 6 options grouped by documentation/implementation gap; dashboard and plan updated
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -3664,9 +3664,12 @@
       <c r="F37" s="69"/>
       <c r="G37" s="69"/>
     </row>
-    <row r="38" spans="1:7" ht="49.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A38" s="70" t="s">
-        <v>65</v>
+    <row r="38" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A38" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• فجوة تطبيق: يوجد متطلب أو إجراء، لكن التطبيق الفعلي غير مكتمل أو غير منتظم أو لا توجد نتائج كافية تثبته.
+   (سبب النقص في ورقة الفحص: الممارسة غير مطبقة أو مطبقة جزئياً • لا توجد نتائج وتحسين)</t>
+        </is>
       </c>
       <c r="B38" s="70"/>
       <c r="C38" s="70"/>
@@ -3675,9 +3678,12 @@
       <c r="F38" s="70"/>
       <c r="G38" s="70"/>
     </row>
-    <row r="39" spans="1:7" ht="49.75" customHeight="1" x14ac:dyDescent="0.2">
-      <c r="A39" s="70" t="s">
-        <v>66</v>
+    <row r="39" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+      <c r="A39" s="70" t="inlineStr">
+        <is>
+          <t xml:space="preserve">• فجوة توثيق/دليل: الممارسة موجودة، لكن الدليل مفقود أو قديم أو غير معتمد أو لا يثبت التنفيذ بشكل كافٍ.
+   (سبب النقص في ورقة الفحص: الدليل مفقود رغم وجود الممارسة • غير معتمد • غير محدّث • لا يغطي المحك كاملاً)</t>
+        </is>
       </c>
       <c r="B39" s="70"/>
       <c r="C39" s="70"/>
@@ -4386,7 +4392,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:I50"/>
+  <dimension ref="A1:I51"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -5588,87 +5594,116 @@
         <v>ماجستير علوم البيانات</v>
       </c>
     </row>
-    <row r="46" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A46" s="13" t="s">
-        <v>151</v>
+    <row r="46" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A46" s="13" t="inlineStr">
+        <is>
+          <t>الدليل مفقود رغم وجود الممارسة</t>
+        </is>
       </c>
       <c r="B46" s="6">
+        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"الدليل مفقود رغم وجود الممارسة")</f>
+        <v>0</v>
+      </c>
+      <c r="C46" s="6">
+        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"الدليل مفقود رغم وجود الممارسة")</f>
+        <v>0</v>
+      </c>
+      <c r="D46" s="6">
+        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"الدليل مفقود رغم وجود الممارسة")</f>
+        <v>0</v>
+      </c>
+    </row>
+    <row r="47" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A47" s="13" t="inlineStr">
+        <is>
+          <t>غير معتمد</t>
+        </is>
+      </c>
+      <c r="B47" s="6">
         <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"غير معتمد")</f>
         <v>0</v>
       </c>
-      <c r="C46" s="6">
+      <c r="C47" s="6">
         <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"غير معتمد")</f>
         <v>0</v>
       </c>
-      <c r="D46" s="6">
+      <c r="D47" s="6">
         <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"غير معتمد")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="47" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A47" s="13" t="s">
-        <v>152</v>
-      </c>
-      <c r="B47" s="6">
+    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A48" s="13" t="inlineStr">
+        <is>
+          <t>غير محدّث</t>
+        </is>
+      </c>
+      <c r="B48" s="6">
         <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"غير محدّث")</f>
         <v>0</v>
       </c>
-      <c r="C47" s="6">
+      <c r="C48" s="6">
         <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"غير محدّث")</f>
         <v>0</v>
       </c>
-      <c r="D47" s="6">
+      <c r="D48" s="6">
         <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"غير محدّث")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="48" spans="1:9" x14ac:dyDescent="0.2">
-      <c r="A48" s="13" t="s">
-        <v>153</v>
-      </c>
-      <c r="B48" s="6">
+    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A49" s="13" t="inlineStr">
+        <is>
+          <t>لا يغطي المحك كاملاً</t>
+        </is>
+      </c>
+      <c r="B49" s="6">
         <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"لا يغطي المحك كاملاً")</f>
         <v>0</v>
       </c>
-      <c r="C48" s="6">
+      <c r="C49" s="6">
         <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"لا يغطي المحك كاملاً")</f>
         <v>0</v>
       </c>
-      <c r="D48" s="6">
+      <c r="D49" s="6">
         <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"لا يغطي المحك كاملاً")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="13" t="s">
-        <v>154</v>
-      </c>
-      <c r="B49" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"لا يثبت التطبيق الفعلي")</f>
+    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A50" s="13" t="inlineStr">
+        <is>
+          <t>الممارسة غير مطبقة أو مطبقة جزئياً</t>
+        </is>
+      </c>
+      <c r="B50" s="6">
+        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
         <v>0</v>
       </c>
-      <c r="C49" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"لا يثبت التطبيق الفعلي")</f>
+      <c r="C50" s="6">
+        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
         <v>0</v>
       </c>
-      <c r="D49" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"لا يثبت التطبيق الفعلي")</f>
+      <c r="D50" s="6">
+        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
         <v>0</v>
       </c>
     </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="s">
-        <v>155</v>
-      </c>
-      <c r="B50" s="6">
+    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
+      <c r="A51" s="13" t="inlineStr">
+        <is>
+          <t>لا توجد نتائج وتحسين</t>
+        </is>
+      </c>
+      <c r="B51" s="6">
         <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"لا توجد نتائج وتحسين")</f>
         <v>0</v>
       </c>
-      <c r="C50" s="6">
+      <c r="C51" s="6">
         <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"لا توجد نتائج وتحسين")</f>
         <v>0</v>
       </c>
-      <c r="D50" s="6">
+      <c r="D51" s="6">
         <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"لا توجد نتائج وتحسين")</f>
         <v>0</v>
       </c>
@@ -14361,7 +14396,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J208" xr:uid="{00000000-0002-0000-0500-000001000000}">
-      <formula1>"غير معتمد,غير محدّث,لا يغطي المحك كاملاً,لا يثبت التطبيق الفعلي,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0500-000002000000}">
@@ -21891,7 +21926,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J208" xr:uid="{00000000-0002-0000-0600-000001000000}">
-      <formula1>"غير معتمد,غير محدّث,لا يغطي المحك كاملاً,لا يثبت التطبيق الفعلي,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0600-000002000000}">
@@ -30219,7 +30254,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J230" xr:uid="{00000000-0002-0000-0700-000001000000}">
-      <formula1>"غير معتمد,غير محدّث,لا يغطي المحك كاملاً,لا يثبت التطبيق الفعلي,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M230" xr:uid="{00000000-0002-0000-0700-000002000000}">

</xml_diff>

<commit_message>
Replace deficiency reasons with gap type (documentation/implementation) in sheets, dashboard and plan
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -489,10 +489,10 @@
     <t>تحتاج تعديل</t>
   </si>
   <si>
-    <t>أكثر أسباب النقص</t>
-  </si>
-  <si>
-    <t>سبب النقص</t>
+    <t xml:space="preserve">نوع الفجوات</t>
+  </si>
+  <si>
+    <t xml:space="preserve">نوع الفجوة</t>
   </si>
   <si>
     <t>غير معتمد</t>
@@ -810,7 +810,7 @@
     <t>سؤال مفتوح: ما مقترحك لتحسين الرسالة أو الأهداف؟</t>
   </si>
   <si>
-    <t>عبّئ الخلايا الصفراء: حالة الدليل، وإن كان ناقصاً: السبب والإجراء والموعد، ثم رابط الدليل. الأعمدة P–Q لأ. فاطمة. الصفوف المظللة = محكات أساسية ★</t>
+    <t xml:space="preserve">عبّئ الخلايا الصفراء: حالة الدليل، وإن كان ناقصاً: نوع الفجوة (توثيق أو تطبيق) والإجراء والموعد، ثم رابط الدليل. الأعمدة P–Q لأ. فاطمة. الصفوف المظللة = محكات أساسية ★</t>
   </si>
   <si>
     <t>نص المحك</t>
@@ -3615,7 +3615,7 @@
 • متوفر ومكتمل: مستوفٍ لمتطلبات الفحص أعلاه.
 • متوفر ويحتاج تحسين: الدليل موجود، إلا أنه يحتاج إلى استكمال أو تحديث أو اعتماد أو تعزيز بما يثبت التطبيق.
 • غير متوفر: لم يتم العثور على دليل يثبت استيفاء المتطلب.
-وعند وجود نقص، يتم توضيح سبب النقص والإجراء المطلوب لاستكمال الدليل ضمن ورقة الفحص.</t>
+وعند وجود نقص، يتم تحديد نوع الفجوة (توثيق أو تطبيق) والإجراء المطلوب لاستكمال الدليل ضمن ورقة الفحص.</t>
         </is>
       </c>
       <c r="B34" s="67"/>
@@ -3625,12 +3625,12 @@
       <c r="F34" s="67"/>
       <c r="G34" s="67"/>
     </row>
-    <row r="35" spans="1:7" ht="98" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="35" spans="1:7" ht="110" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A35" s="67" t="inlineStr">
         <is>
           <t xml:space="preserve">خطوات العمل في ورقة الفحص:
 1. يصفّي العضو عمود "المسؤول" على اسمه، ويرفع كل دليل للمستودع بالترميز المعتمد ويضع رابطه.
-2. يختار "حالة الدليل"، وإن لم يكن مكتملاً يختار "سبب النقص" ويكتب "الإجراء المطلوب" والجهة التي ستستكمله ويختار "الموعد". وتظهر "الأولوية" تلقائياً.
+2. يختار "حالة الدليل"، وإن لم يكن مكتملاً يختار "نوع الفجوة" بسؤال: هل العمل يتم فعلاً؟ (نعم = فجوة توثيق • لا أو جزئياً = فجوة تطبيق)، ويكتب "الإجراء المطلوب" والجهة التي ستستكمله ويختار "الموعد". وتظهر "الأولوية" تلقائياً.
 3. تراجع أمينة اللجنة الأدلة أسبوعياً (تمت • تحتاج تعديل)، وتراجع رئيسة اللجنة كفاية أدلة المحكات الأساسية ★ في الأسبوع 6.
 4. تُراجع خطة الاستكمال وتُعتمد في اجتماع الأسبوع 7، وتتحدث "لوحة المتابعة" تلقائياً مع كل إدخال.</t>
         </is>
@@ -3667,8 +3667,7 @@
     <row r="38" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A38" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">• فجوة تطبيق: يوجد متطلب أو إجراء، لكن التطبيق الفعلي غير مكتمل أو غير منتظم أو لا توجد نتائج كافية تثبته.
-   (سبب النقص في ورقة الفحص: الممارسة غير مطبقة أو مطبقة جزئياً • لا توجد نتائج وتحسين)</t>
+          <t xml:space="preserve">• فجوة تطبيق: يوجد متطلب أو إجراء، لكن التطبيق الفعلي غير مكتمل أو غير منتظم أو لا توجد نتائج كافية تثبته. وإذا كان العمل لا يتم ولا يوجد دليل عليه، تُصنّف فجوة تطبيق.</t>
         </is>
       </c>
       <c r="B38" s="70"/>
@@ -3678,11 +3677,10 @@
       <c r="F38" s="70"/>
       <c r="G38" s="70"/>
     </row>
-    <row r="39" spans="1:7" ht="48" customHeight="1" x14ac:dyDescent="0.2">
+    <row r="39" spans="1:7" ht="30" customHeight="1" x14ac:dyDescent="0.2">
       <c r="A39" s="70" t="inlineStr">
         <is>
-          <t xml:space="preserve">• فجوة توثيق/دليل: الممارسة موجودة، لكن الدليل مفقود أو قديم أو غير معتمد أو لا يثبت التنفيذ بشكل كافٍ.
-   (سبب النقص في ورقة الفحص: الدليل مفقود رغم وجود الممارسة • غير معتمد • غير محدّث • لا يغطي المحك كاملاً)</t>
+          <t xml:space="preserve">• فجوة توثيق/دليل: الممارسة موجودة، لكن الدليل مفقود أو قديم أو غير معتمد أو لا يثبت التنفيذ بشكل كافٍ.</t>
         </is>
       </c>
       <c r="B39" s="70"/>
@@ -4392,7 +4390,7 @@
   <sheetPr>
     <tabColor rgb="FF2E75B6"/>
   </sheetPr>
-  <dimension ref="A1:I51"/>
+  <dimension ref="A1:I47"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="8.6640625" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
     <col min="1" max="1" width="42" customWidth="1"/>
@@ -5597,114 +5595,38 @@
     <row r="46" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A46" s="13" t="inlineStr">
         <is>
-          <t>الدليل مفقود رغم وجود الممارسة</t>
+          <t>فجوة توثيق</t>
         </is>
       </c>
       <c r="B46" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"الدليل مفقود رغم وجود الممارسة")</f>
+        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"فجوة توثيق")</f>
         <v>0</v>
       </c>
       <c r="C46" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"الدليل مفقود رغم وجود الممارسة")</f>
+        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"فجوة توثيق")</f>
         <v>0</v>
       </c>
       <c r="D46" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"الدليل مفقود رغم وجود الممارسة")</f>
+        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"فجوة توثيق")</f>
         <v>0</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.2">
       <c r="A47" s="13" t="inlineStr">
         <is>
-          <t>غير معتمد</t>
+          <t>فجوة تطبيق</t>
         </is>
       </c>
       <c r="B47" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"غير معتمد")</f>
+        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"فجوة تطبيق")</f>
         <v>0</v>
       </c>
       <c r="C47" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"غير معتمد")</f>
+        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"فجوة تطبيق")</f>
         <v>0</v>
       </c>
       <c r="D47" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"غير معتمد")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="48" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A48" s="13" t="inlineStr">
-        <is>
-          <t>غير محدّث</t>
-        </is>
-      </c>
-      <c r="B48" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"غير محدّث")</f>
-        <v>0</v>
-      </c>
-      <c r="C48" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"غير محدّث")</f>
-        <v>0</v>
-      </c>
-      <c r="D48" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"غير محدّث")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="49" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A49" s="13" t="inlineStr">
-        <is>
-          <t>لا يغطي المحك كاملاً</t>
-        </is>
-      </c>
-      <c r="B49" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"لا يغطي المحك كاملاً")</f>
-        <v>0</v>
-      </c>
-      <c r="C49" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"لا يغطي المحك كاملاً")</f>
-        <v>0</v>
-      </c>
-      <c r="D49" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"لا يغطي المحك كاملاً")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="50" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A50" s="13" t="inlineStr">
-        <is>
-          <t>الممارسة غير مطبقة أو مطبقة جزئياً</t>
-        </is>
-      </c>
-      <c r="B50" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
-        <v>0</v>
-      </c>
-      <c r="C50" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
-        <v>0</v>
-      </c>
-      <c r="D50" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"الممارسة غير مطبقة أو مطبقة جزئياً")</f>
-        <v>0</v>
-      </c>
-    </row>
-    <row r="51" spans="1:4" x14ac:dyDescent="0.2">
-      <c r="A51" s="13" t="inlineStr">
-        <is>
-          <t>لا توجد نتائج وتحسين</t>
-        </is>
-      </c>
-      <c r="B51" s="6">
-        <f>COUNTIF('فحص-حاسب-بكالوريوس'!$J$5:$J$208,"لا توجد نتائج وتحسين")</f>
-        <v>0</v>
-      </c>
-      <c r="C51" s="6">
-        <f>COUNTIF('فحص-بيانات-بكالوريوس'!$J$5:$J$208,"لا توجد نتائج وتحسين")</f>
-        <v>0</v>
-      </c>
-      <c r="D51" s="6">
-        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"لا توجد نتائج وتحسين")</f>
+        <f>COUNTIF('فحص-بيانات-ماجستير'!$J$5:$J$230,"فجوة تطبيق")</f>
         <v>0</v>
       </c>
     </row>
@@ -14396,7 +14318,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J208" xr:uid="{00000000-0002-0000-0500-000001000000}">
-      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"فجوة توثيق,فجوة تطبيق"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0500-000002000000}">
@@ -21926,7 +21848,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J208" xr:uid="{00000000-0002-0000-0600-000001000000}">
-      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"فجوة توثيق,فجوة تطبيق"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0600-000002000000}">
@@ -30254,7 +30176,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="J5:J230" xr:uid="{00000000-0002-0000-0700-000001000000}">
-      <formula1>"الدليل مفقود رغم وجود الممارسة,غير معتمد,غير محدّث,لا يغطي المحك كاملاً,الممارسة غير مطبقة أو مطبقة جزئياً,لا توجد نتائج وتحسين"</formula1>
+      <formula1>"فجوة توثيق,فجوة تطبيق"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M230" xr:uid="{00000000-0002-0000-0700-000002000000}">

</xml_diff>

<commit_message>
Check sheets: grey/red guard for complete evidence, yellow reminder for gap type; deadline options by remediation horizon
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -2596,7 +2596,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="23">
+  <dxfs count="26">
     <dxf>
       <fill>
         <patternFill>
@@ -2794,6 +2794,33 @@
       <fill>
         <patternFill>
           <bgColor rgb="FFC6EFCE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFD9D9D9"/>
+          <bgColor rgb="FFD9D9D9"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <font>
+        <color rgb="FF9C0006"/>
+      </font>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFC7CE"/>
+          <bgColor rgb="FFFFC7CE"/>
+        </patternFill>
+      </fill>
+    </dxf>
+    <dxf>
+      <fill>
+        <patternFill patternType="solid">
+          <fgColor rgb="FFFFD966"/>
+          <bgColor rgb="FFFFD966"/>
         </patternFill>
       </fill>
     </dxf>
@@ -14312,6 +14339,19 @@
       <formula>"تحتاج تعديل"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J208 L5:M208">
+    <cfRule type="expression" dxfId="24" priority="101">
+      <formula>AND($I5="متوفر ومكتمل",J5&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="102">
+      <formula>$I5="متوفر ومكتمل"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J208">
+    <cfRule type="expression" dxfId="25" priority="103">
+      <formula>AND(OR($I5="متوفر ويحتاج تحسين",$I5="غير متوفر"),J5="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="I5:I208" xr:uid="{00000000-0002-0000-0500-000000000000}">
       <formula1>"متوفر ومكتمل,متوفر ويحتاج تحسين,غير متوفر"</formula1>
@@ -14322,7 +14362,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0500-000002000000}">
-      <formula1>"الأسبوع 1,الأسبوع 2,الأسبوع 3,الأسبوع 4,الأسبوع 5,الأسبوع 6,الأسبوع 7,الأسبوع 8,بعد الخطة"</formula1>
+      <formula1>"خلال المرحلة الأولى,خلال فصل دراسي,خلال سنة دراسية"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="P5:P208" xr:uid="{00000000-0002-0000-0500-000003000000}">
@@ -21842,6 +21882,19 @@
       <formula>"تحتاج تعديل"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J208 L5:M208">
+    <cfRule type="expression" dxfId="24" priority="101">
+      <formula>AND($I5="متوفر ومكتمل",J5&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="102">
+      <formula>$I5="متوفر ومكتمل"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J208">
+    <cfRule type="expression" dxfId="25" priority="103">
+      <formula>AND(OR($I5="متوفر ويحتاج تحسين",$I5="غير متوفر"),J5="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="I5:I208" xr:uid="{00000000-0002-0000-0600-000000000000}">
       <formula1>"متوفر ومكتمل,متوفر ويحتاج تحسين,غير متوفر"</formula1>
@@ -21852,7 +21905,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M208" xr:uid="{00000000-0002-0000-0600-000002000000}">
-      <formula1>"الأسبوع 1,الأسبوع 2,الأسبوع 3,الأسبوع 4,الأسبوع 5,الأسبوع 6,الأسبوع 7,الأسبوع 8,بعد الخطة"</formula1>
+      <formula1>"خلال المرحلة الأولى,خلال فصل دراسي,خلال سنة دراسية"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="P5:P208" xr:uid="{00000000-0002-0000-0600-000003000000}">
@@ -30170,6 +30223,19 @@
       <formula>"تحتاج تعديل"</formula>
     </cfRule>
   </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J230 L5:M230">
+    <cfRule type="expression" dxfId="24" priority="101">
+      <formula>AND($I5="متوفر ومكتمل",J5&lt;&gt;"")</formula>
+    </cfRule>
+    <cfRule type="expression" dxfId="23" priority="102">
+      <formula>$I5="متوفر ومكتمل"</formula>
+    </cfRule>
+  </conditionalFormatting>
+  <conditionalFormatting sqref="J5:J230">
+    <cfRule type="expression" dxfId="25" priority="103">
+      <formula>AND(OR($I5="متوفر ويحتاج تحسين",$I5="غير متوفر"),J5="")</formula>
+    </cfRule>
+  </conditionalFormatting>
   <dataValidations count="4">
     <dataValidation type="list" allowBlank="1" sqref="I5:I230" xr:uid="{00000000-0002-0000-0700-000000000000}">
       <formula1>"متوفر ومكتمل,متوفر ويحتاج تحسين,غير متوفر"</formula1>
@@ -30180,7 +30246,7 @@
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="M5:M230" xr:uid="{00000000-0002-0000-0700-000002000000}">
-      <formula1>"الأسبوع 1,الأسبوع 2,الأسبوع 3,الأسبوع 4,الأسبوع 5,الأسبوع 6,الأسبوع 7,الأسبوع 8,بعد الخطة"</formula1>
+      <formula1>"خلال المرحلة الأولى,خلال فصل دراسي,خلال سنة دراسية"</formula1>
       <formula2>0</formula2>
     </dataValidation>
     <dataValidation type="list" allowBlank="1" sqref="P5:P230" xr:uid="{00000000-0002-0000-0700-000003000000}">

</xml_diff>

<commit_message>
Add classification examples sheet linked to guide criteria
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -18,6 +18,7 @@
     <sheet name="لوحة المتابعة" sheetId="3" r:id="rId3"/>
     <sheet name="متطلبات التقدم للاعتماد" sheetId="4" r:id="rId4"/>
     <sheet name="مراجعة الرسالة (مقترح)" sheetId="5" r:id="rId5"/>
+    <sheet name="أمثلة التصنيف" sheetId="9" r:id="rId99"/>
     <sheet name="فحص-حاسب-بكالوريوس" sheetId="6" r:id="rId6"/>
     <sheet name="فحص-بيانات-بكالوريوس" sheetId="7" r:id="rId7"/>
     <sheet name="فحص-بيانات-ماجستير" sheetId="8" r:id="rId8"/>
@@ -30259,4 +30260,549 @@
     <oddFooter xml:space="preserve">&amp;L_x000D_&amp;1#&amp;"Aptos"&amp;10&amp;K000000 Restricted - مقيد </oddFooter>
   </headerFooter>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet9.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+  </sheetPr>
+  <dimension ref="A1:H15"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="18" customWidth="1"/>
+    <col min="2" max="2" width="26" customWidth="1"/>
+    <col min="3" max="3" width="38" customWidth="1"/>
+    <col min="4" max="4" width="40" customWidth="1"/>
+    <col min="5" max="5" width="13" customWidth="1"/>
+    <col min="6" max="6" width="38" customWidth="1"/>
+    <col min="7" max="7" width="17" customWidth="1"/>
+    <col min="8" max="8" width="10" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:8" ht="30" customHeight="1">
+      <c r="A1" s="63" t="inlineStr">
+        <is>
+          <t xml:space="preserve">أمثلة تصنيف الأدلة (لاجتماع الانطلاق وجلسة توحيد الحكم)</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:8" ht="46" customHeight="1">
+      <c r="A2" s="64" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الأدلة من الدليل الاسترشادي، ووضعها افتراضي للتوضيح.  القاعدة: حالة الدليل ← بنود الفحص الخمسة • نوع الفجوة ← هل العمل يتم فعلاً؟ (نعم = فجوة توثيق • لا أو جزئياً = فجوة تطبيق) • الأولوية تلقائية: عالية إذا كان الدليل غير متوفر أو المحك أساسياً ★.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:8" ht="30" customHeight="1">
+      <c r="A4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">حالة الدليل</t>
+        </is>
+      </c>
+      <c r="B4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">المحك</t>
+        </is>
+      </c>
+      <c r="C4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الدليل</t>
+        </is>
+      </c>
+      <c r="D4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الوضع</t>
+        </is>
+      </c>
+      <c r="E4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">نوع الفجوة</t>
+        </is>
+      </c>
+      <c r="F4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الإجراء المطلوب</t>
+        </is>
+      </c>
+      <c r="G4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الموعد</t>
+        </is>
+      </c>
+      <c r="H4" s="55" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الأولوية</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:8" ht="48" customHeight="1">
+      <c r="A5" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ومكتمل</t>
+        </is>
+      </c>
+      <c r="B5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-1-1 اتساق الرسالة والأهداف</t>
+        </is>
+      </c>
+      <c r="C5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">إعلان رسالة البرنامج وأهدافه على الموقع الإلكتروني</t>
+        </is>
+      </c>
+      <c r="D5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">منشورة، وهي الصيغة المعتمدة الحالية</t>
+        </is>
+      </c>
+      <c r="E5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="G5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H5" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+    </row>
+    <row r="6" spans="1:8" ht="48" customHeight="1">
+      <c r="A6" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ومكتمل</t>
+        </is>
+      </c>
+      <c r="B6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">5-0-3 ★ السلامة</t>
+        </is>
+      </c>
+      <c r="C6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عقد الشركة المسؤولة عن التخلص من النفايات الخطرة</t>
+        </is>
+      </c>
+      <c r="D6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">العقد ساري ومعتمد</t>
+        </is>
+      </c>
+      <c r="E6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="G6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H6" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+    </row>
+    <row r="7" spans="1:8" ht="48" customHeight="1">
+      <c r="A7" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ويحتاج تحسين</t>
+        </is>
+      </c>
+      <c r="B7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-1-1 اتساق الرسالة والأهداف</t>
+        </is>
+      </c>
+      <c r="C7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مصفوفة اتساق رسالة البرنامج وأهدافه مع رسالة الجامعة والكلية</t>
+        </is>
+      </c>
+      <c r="D7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">موجودة، لكنها على رسالة الكلية القديمة (غير محدّثة)</t>
+        </is>
+      </c>
+      <c r="E7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة توثيق</t>
+        </is>
+      </c>
+      <c r="F7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تحديثها واعتمادها من مجلس القسم</t>
+        </is>
+      </c>
+      <c r="G7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال المرحلة الأولى</t>
+        </is>
+      </c>
+      <c r="H7" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="8" spans="1:8" ht="48" customHeight="1">
+      <c r="A8" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ويحتاج تحسين</t>
+        </is>
+      </c>
+      <c r="B8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2-2-4 ربط نواتج المقررات بالبرنامج</t>
+        </is>
+      </c>
+      <c r="C8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">توصيف البرنامج مع مصفوفة ربط نواتج المقررات بنواتج البرنامج</t>
+        </is>
+      </c>
+      <c r="D8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">موجود، لكنه غير معتمد من مجلس الكلية</t>
+        </is>
+      </c>
+      <c r="E8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة توثيق</t>
+        </is>
+      </c>
+      <c r="F8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رفعه لمجلس الكلية لاعتماده</t>
+        </is>
+      </c>
+      <c r="G8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال المرحلة الأولى</t>
+        </is>
+      </c>
+      <c r="H8" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوسطة</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" spans="1:8" ht="48" customHeight="1">
+      <c r="A9" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ويحتاج تحسين</t>
+        </is>
+      </c>
+      <c r="B9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3-0-3 ★ الإرشاد الأكاديمي</t>
+        </is>
+      </c>
+      <c r="C9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">دليل الإرشاد والتوجيه الأكاديمي للطالب</t>
+        </is>
+      </c>
+      <c r="D9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">الدليل موجود، لكن الإرشاد لا يُطبّق بانتظام ولا توجد سجلات جلسات</t>
+        </is>
+      </c>
+      <c r="E9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة تطبيق</t>
+        </is>
+      </c>
+      <c r="F9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تفعيل الساعات الإرشادية وتوثيق الجلسات (القسم)</t>
+        </is>
+      </c>
+      <c r="G9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال فصل دراسي</t>
+        </is>
+      </c>
+      <c r="H9" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="10" spans="1:8" ht="48" customHeight="1">
+      <c r="A10" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">متوفر ويحتاج تحسين</t>
+        </is>
+      </c>
+      <c r="B10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-2-2 ★ تحليل مؤشرات الأداء</t>
+        </is>
+      </c>
+      <c r="C10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير قياس مؤشرات الأداء الرئيسة</t>
+        </is>
+      </c>
+      <c r="D10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">التقارير موجودة، لكن لم تُناقش ولم تُبنَ عليها خطة تحسين</t>
+        </is>
+      </c>
+      <c r="E10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة تطبيق</t>
+        </is>
+      </c>
+      <c r="F10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مناقشتها في مجلس القسم وإعداد خطة تحسين</t>
+        </is>
+      </c>
+      <c r="G10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال فصل دراسي</t>
+        </is>
+      </c>
+      <c r="H10" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" spans="1:8" ht="48" customHeight="1">
+      <c r="A11" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">غير متوفر</t>
+        </is>
+      </c>
+      <c r="B11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">3-0-7 ★ رضا الطلاب عن الخدمات</t>
+        </is>
+      </c>
+      <c r="C11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير استطلاعات رأي الطلبة حول جودة الخدمات</t>
+        </is>
+      </c>
+      <c r="D11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عمادة الجودة طبّقت الاستطلاع، لكن لا يوجد تقرير خاص بالبرنامج</t>
+        </is>
+      </c>
+      <c r="E11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة توثيق</t>
+        </is>
+      </c>
+      <c r="F11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">طلب النتائج من عمادة الجودة وإعداد تقرير للبرنامج</t>
+        </is>
+      </c>
+      <c r="G11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال المرحلة الأولى</t>
+        </is>
+      </c>
+      <c r="H11" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" spans="1:8" ht="48" customHeight="1">
+      <c r="A12" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">غير متوفر</t>
+        </is>
+      </c>
+      <c r="B12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4-0-6 تقييم أداء هيئة التدريس</t>
+        </is>
+      </c>
+      <c r="C12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">نماذج من التغذية الراجعة المقدمة عن أداء أعضاء هيئة التدريس</t>
+        </is>
+      </c>
+      <c r="D12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">التغذية الراجعة تُقدَّم شفهياً أو بالبريد، لكن لا تُحفظ</t>
+        </is>
+      </c>
+      <c r="E12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة توثيق</t>
+        </is>
+      </c>
+      <c r="F12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">جمع نماذج منها وحفظها في المستودع</t>
+        </is>
+      </c>
+      <c r="G12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال المرحلة الأولى</t>
+        </is>
+      </c>
+      <c r="H12" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" spans="1:8" ht="48" customHeight="1">
+      <c r="A13" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">غير متوفر</t>
+        </is>
+      </c>
+      <c r="B13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">4-0-6 تقييم أداء هيئة التدريس</t>
+        </is>
+      </c>
+      <c r="C13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">استطلاع رأي أعضاء هيئة التدريس عن رضاهم عن طرق تقييم أدائهم</t>
+        </is>
+      </c>
+      <c r="D13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">لم يُطبَّق أصلاً</t>
+        </is>
+      </c>
+      <c r="E13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة تطبيق</t>
+        </is>
+      </c>
+      <c r="F13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تصميم الاستطلاع وتطبيقه وإعداد تقريره</t>
+        </is>
+      </c>
+      <c r="G13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال فصل دراسي</t>
+        </is>
+      </c>
+      <c r="H13" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="14" spans="1:8" ht="48" customHeight="1">
+      <c r="A14" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">غير متوفر</t>
+        </is>
+      </c>
+      <c r="B14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">6-0-8 كفاءة الإشراف العلمي (ماجستير)</t>
+        </is>
+      </c>
+      <c r="C14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">نتائج تقييم الطلاب لجودة الإشراف العلمي</t>
+        </is>
+      </c>
+      <c r="D14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">لا يوجد تقييم للإشراف</t>
+        </is>
+      </c>
+      <c r="E14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">فجوة تطبيق</t>
+        </is>
+      </c>
+      <c r="F14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تطبيق تقييم سنوي للإشراف ثم تحليله والتحسين</t>
+        </is>
+      </c>
+      <c r="G14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خلال سنة دراسية</t>
+        </is>
+      </c>
+      <c r="H14" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">عالية</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" spans="1:8" ht="48" customHeight="1">
+      <c r="A15" s="46" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خطأ شائع 🔴</t>
+        </is>
+      </c>
+      <c r="B15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">1-1-1 اتساق الرسالة والأهداف</t>
+        </is>
+      </c>
+      <c r="C15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مصفوفة اتساق رسالة البرنامج وأهدافه</t>
+        </is>
+      </c>
+      <c r="D15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">اختار العضو "متوفر ومكتمل" ثم كتب في الإجراء: "تحديث المصفوفة"</t>
+        </is>
+      </c>
+      <c r="E15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="F15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تتلون الخانة بالأحمر: ما دام يحتاج تحديثاً فهو "متوفر ويحتاج تحسين" وليس "مكتملاً"</t>
+        </is>
+      </c>
+      <c r="G15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+      <c r="H15" s="47" t="inlineStr">
+        <is>
+          <t xml:space="preserve">—</t>
+        </is>
+      </c>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:H1"/>
+    <mergeCell ref="A2:H2"/>
+  </mergeCells>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Add evidence register sheet (search first, add new evidence, coding by Dr. Barakati)
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -20,12 +20,13 @@
     <sheet name="متطلبات التقدم للاعتماد" sheetId="4" r:id="rId5"/>
     <sheet name="وثائق الجودة" sheetId="11" r:id="rId100"/>
     <sheet name="أمثلة التصنيف" sheetId="9" r:id="rId6"/>
+    <sheet name="سجل الأدلة" sheetId="12" r:id="rId101"/>
     <sheet name="فحص-حاسب-بكالوريوس" sheetId="6" r:id="rId7"/>
     <sheet name="فحص-بيانات-بكالوريوس" sheetId="7" r:id="rId8"/>
     <sheet name="فحص-بيانات-ماجستير" sheetId="8" r:id="rId9"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'فحص-حاسب-بكالوريوس'!$A$4:$R$208</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="8" hidden="1">'فحص-حاسب-بكالوريوس'!$A$4:$R$208</definedName>
   </definedNames>
   <calcPr calcId="191029" calcMode="auto" fullCalcOnLoad="1"/>
   <extLst>
@@ -5541,6 +5542,4006 @@
 </worksheet>
 </file>
 
+<file path=xl/worksheets/sheet11.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+  <sheetPr>
+    <tabColor rgb="FF548235"/>
+  </sheetPr>
+  <dimension ref="A1:I304"/>
+  <sheetFormatPr defaultRowHeight="15"/>
+  <cols>
+    <col min="1" max="1" width="5" customWidth="1"/>
+    <col min="2" max="2" width="42" customWidth="1"/>
+    <col min="3" max="3" width="36" customWidth="1"/>
+    <col min="4" max="4" width="24" customWidth="1"/>
+    <col min="5" max="5" width="18" customWidth="1"/>
+    <col min="6" max="6" width="40" customWidth="1"/>
+    <col min="7" max="7" width="24" customWidth="1"/>
+    <col min="8" max="8" width="13" customWidth="1"/>
+    <col min="9" max="9" width="20" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" ht="30" customHeight="1">
+      <c r="A1" s="98" t="inlineStr">
+        <is>
+          <t xml:space="preserve">سجل الأدلة – ابحث هنا أولاً قبل البحث عن أي دليل</t>
+        </is>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="46" customHeight="1">
+      <c r="A2" s="99" t="inlineStr">
+        <is>
+          <t xml:space="preserve">ابحث بكلمة من اسم الدليل (Cmd + F أو Ctrl + F). إذا وجدته فانسخ رابطه إلى ورقة الفحص. وإذا رفعت دليلاً جديداً فأضفه في أول سطر فارغ. عمود «رمز الدليل» يعبّئه د. عبدالله البركاتي فقط.</t>
+        </is>
+      </c>
+    </row>
+    <row r="4" spans="1:9" ht="30" customHeight="1">
+      <c r="A4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">م</t>
+        </is>
+      </c>
+      <c r="B4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">اسم الدليل</t>
+        </is>
+      </c>
+      <c r="C4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">وصف مختصر</t>
+        </is>
+      </c>
+      <c r="D4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">البرنامج</t>
+        </is>
+      </c>
+      <c r="E4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">المعيار / المحكات</t>
+        </is>
+      </c>
+      <c r="F4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رابط الدليل</t>
+        </is>
+      </c>
+      <c r="G4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رفعه</t>
+        </is>
+      </c>
+      <c r="H4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تاريخ الرفع</t>
+        </is>
+      </c>
+      <c r="I4" s="29" t="inlineStr">
+        <is>
+          <t xml:space="preserve">رمز الدليل (د. البركاتي)</t>
+        </is>
+      </c>
+    </row>
+    <row r="5" spans="1:9">
+      <c r="A5" s="30">
+        <v>1</v>
+      </c>
+      <c r="B5" s="38"/>
+      <c r="C5" s="38"/>
+      <c r="D5" s="38"/>
+      <c r="E5" s="38"/>
+      <c r="F5" s="38"/>
+      <c r="G5" s="38"/>
+      <c r="H5" s="38"/>
+      <c r="I5" s="38"/>
+    </row>
+    <row r="6" spans="1:9">
+      <c r="A6" s="30">
+        <v>2</v>
+      </c>
+      <c r="B6" s="38"/>
+      <c r="C6" s="38"/>
+      <c r="D6" s="38"/>
+      <c r="E6" s="38"/>
+      <c r="F6" s="38"/>
+      <c r="G6" s="38"/>
+      <c r="H6" s="38"/>
+      <c r="I6" s="38"/>
+    </row>
+    <row r="7" spans="1:9">
+      <c r="A7" s="30">
+        <v>3</v>
+      </c>
+      <c r="B7" s="38"/>
+      <c r="C7" s="38"/>
+      <c r="D7" s="38"/>
+      <c r="E7" s="38"/>
+      <c r="F7" s="38"/>
+      <c r="G7" s="38"/>
+      <c r="H7" s="38"/>
+      <c r="I7" s="38"/>
+    </row>
+    <row r="8" spans="1:9">
+      <c r="A8" s="30">
+        <v>4</v>
+      </c>
+      <c r="B8" s="38"/>
+      <c r="C8" s="38"/>
+      <c r="D8" s="38"/>
+      <c r="E8" s="38"/>
+      <c r="F8" s="38"/>
+      <c r="G8" s="38"/>
+      <c r="H8" s="38"/>
+      <c r="I8" s="38"/>
+    </row>
+    <row r="9" spans="1:9">
+      <c r="A9" s="30">
+        <v>5</v>
+      </c>
+      <c r="B9" s="38"/>
+      <c r="C9" s="38"/>
+      <c r="D9" s="38"/>
+      <c r="E9" s="38"/>
+      <c r="F9" s="38"/>
+      <c r="G9" s="38"/>
+      <c r="H9" s="38"/>
+      <c r="I9" s="38"/>
+    </row>
+    <row r="10" spans="1:9">
+      <c r="A10" s="30">
+        <v>6</v>
+      </c>
+      <c r="B10" s="38"/>
+      <c r="C10" s="38"/>
+      <c r="D10" s="38"/>
+      <c r="E10" s="38"/>
+      <c r="F10" s="38"/>
+      <c r="G10" s="38"/>
+      <c r="H10" s="38"/>
+      <c r="I10" s="38"/>
+    </row>
+    <row r="11" spans="1:9">
+      <c r="A11" s="30">
+        <v>7</v>
+      </c>
+      <c r="B11" s="38"/>
+      <c r="C11" s="38"/>
+      <c r="D11" s="38"/>
+      <c r="E11" s="38"/>
+      <c r="F11" s="38"/>
+      <c r="G11" s="38"/>
+      <c r="H11" s="38"/>
+      <c r="I11" s="38"/>
+    </row>
+    <row r="12" spans="1:9">
+      <c r="A12" s="30">
+        <v>8</v>
+      </c>
+      <c r="B12" s="38"/>
+      <c r="C12" s="38"/>
+      <c r="D12" s="38"/>
+      <c r="E12" s="38"/>
+      <c r="F12" s="38"/>
+      <c r="G12" s="38"/>
+      <c r="H12" s="38"/>
+      <c r="I12" s="38"/>
+    </row>
+    <row r="13" spans="1:9">
+      <c r="A13" s="30">
+        <v>9</v>
+      </c>
+      <c r="B13" s="38"/>
+      <c r="C13" s="38"/>
+      <c r="D13" s="38"/>
+      <c r="E13" s="38"/>
+      <c r="F13" s="38"/>
+      <c r="G13" s="38"/>
+      <c r="H13" s="38"/>
+      <c r="I13" s="38"/>
+    </row>
+    <row r="14" spans="1:9">
+      <c r="A14" s="30">
+        <v>10</v>
+      </c>
+      <c r="B14" s="38"/>
+      <c r="C14" s="38"/>
+      <c r="D14" s="38"/>
+      <c r="E14" s="38"/>
+      <c r="F14" s="38"/>
+      <c r="G14" s="38"/>
+      <c r="H14" s="38"/>
+      <c r="I14" s="38"/>
+    </row>
+    <row r="15" spans="1:9">
+      <c r="A15" s="30">
+        <v>11</v>
+      </c>
+      <c r="B15" s="38"/>
+      <c r="C15" s="38"/>
+      <c r="D15" s="38"/>
+      <c r="E15" s="38"/>
+      <c r="F15" s="38"/>
+      <c r="G15" s="38"/>
+      <c r="H15" s="38"/>
+      <c r="I15" s="38"/>
+    </row>
+    <row r="16" spans="1:9">
+      <c r="A16" s="30">
+        <v>12</v>
+      </c>
+      <c r="B16" s="38"/>
+      <c r="C16" s="38"/>
+      <c r="D16" s="38"/>
+      <c r="E16" s="38"/>
+      <c r="F16" s="38"/>
+      <c r="G16" s="38"/>
+      <c r="H16" s="38"/>
+      <c r="I16" s="38"/>
+    </row>
+    <row r="17" spans="1:9">
+      <c r="A17" s="30">
+        <v>13</v>
+      </c>
+      <c r="B17" s="38"/>
+      <c r="C17" s="38"/>
+      <c r="D17" s="38"/>
+      <c r="E17" s="38"/>
+      <c r="F17" s="38"/>
+      <c r="G17" s="38"/>
+      <c r="H17" s="38"/>
+      <c r="I17" s="38"/>
+    </row>
+    <row r="18" spans="1:9">
+      <c r="A18" s="30">
+        <v>14</v>
+      </c>
+      <c r="B18" s="38"/>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="38"/>
+      <c r="F18" s="38"/>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+      <c r="I18" s="38"/>
+    </row>
+    <row r="19" spans="1:9">
+      <c r="A19" s="30">
+        <v>15</v>
+      </c>
+      <c r="B19" s="38"/>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="38"/>
+      <c r="F19" s="38"/>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+      <c r="I19" s="38"/>
+    </row>
+    <row r="20" spans="1:9">
+      <c r="A20" s="30">
+        <v>16</v>
+      </c>
+      <c r="B20" s="38"/>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="38"/>
+      <c r="F20" s="38"/>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+      <c r="I20" s="38"/>
+    </row>
+    <row r="21" spans="1:9">
+      <c r="A21" s="30">
+        <v>17</v>
+      </c>
+      <c r="B21" s="38"/>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="38"/>
+      <c r="F21" s="38"/>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+      <c r="I21" s="38"/>
+    </row>
+    <row r="22" spans="1:9">
+      <c r="A22" s="30">
+        <v>18</v>
+      </c>
+      <c r="B22" s="38"/>
+      <c r="C22" s="38"/>
+      <c r="D22" s="38"/>
+      <c r="E22" s="38"/>
+      <c r="F22" s="38"/>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+      <c r="I22" s="38"/>
+    </row>
+    <row r="23" spans="1:9">
+      <c r="A23" s="30">
+        <v>19</v>
+      </c>
+      <c r="B23" s="38"/>
+      <c r="C23" s="38"/>
+      <c r="D23" s="38"/>
+      <c r="E23" s="38"/>
+      <c r="F23" s="38"/>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+      <c r="I23" s="38"/>
+    </row>
+    <row r="24" spans="1:9">
+      <c r="A24" s="30">
+        <v>20</v>
+      </c>
+      <c r="B24" s="38"/>
+      <c r="C24" s="38"/>
+      <c r="D24" s="38"/>
+      <c r="E24" s="38"/>
+      <c r="F24" s="38"/>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
+      <c r="I24" s="38"/>
+    </row>
+    <row r="25" spans="1:9">
+      <c r="A25" s="30">
+        <v>21</v>
+      </c>
+      <c r="B25" s="38"/>
+      <c r="C25" s="38"/>
+      <c r="D25" s="38"/>
+      <c r="E25" s="38"/>
+      <c r="F25" s="38"/>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+      <c r="I25" s="38"/>
+    </row>
+    <row r="26" spans="1:9">
+      <c r="A26" s="30">
+        <v>22</v>
+      </c>
+      <c r="B26" s="38"/>
+      <c r="C26" s="38"/>
+      <c r="D26" s="38"/>
+      <c r="E26" s="38"/>
+      <c r="F26" s="38"/>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+      <c r="I26" s="38"/>
+    </row>
+    <row r="27" spans="1:9">
+      <c r="A27" s="30">
+        <v>23</v>
+      </c>
+      <c r="B27" s="38"/>
+      <c r="C27" s="38"/>
+      <c r="D27" s="38"/>
+      <c r="E27" s="38"/>
+      <c r="F27" s="38"/>
+      <c r="G27" s="38"/>
+      <c r="H27" s="38"/>
+      <c r="I27" s="38"/>
+    </row>
+    <row r="28" spans="1:9">
+      <c r="A28" s="30">
+        <v>24</v>
+      </c>
+      <c r="B28" s="38"/>
+      <c r="C28" s="38"/>
+      <c r="D28" s="38"/>
+      <c r="E28" s="38"/>
+      <c r="F28" s="38"/>
+      <c r="G28" s="38"/>
+      <c r="H28" s="38"/>
+      <c r="I28" s="38"/>
+    </row>
+    <row r="29" spans="1:9">
+      <c r="A29" s="30">
+        <v>25</v>
+      </c>
+      <c r="B29" s="38"/>
+      <c r="C29" s="38"/>
+      <c r="D29" s="38"/>
+      <c r="E29" s="38"/>
+      <c r="F29" s="38"/>
+      <c r="G29" s="38"/>
+      <c r="H29" s="38"/>
+      <c r="I29" s="38"/>
+    </row>
+    <row r="30" spans="1:9">
+      <c r="A30" s="30">
+        <v>26</v>
+      </c>
+      <c r="B30" s="38"/>
+      <c r="C30" s="38"/>
+      <c r="D30" s="38"/>
+      <c r="E30" s="38"/>
+      <c r="F30" s="38"/>
+      <c r="G30" s="38"/>
+      <c r="H30" s="38"/>
+      <c r="I30" s="38"/>
+    </row>
+    <row r="31" spans="1:9">
+      <c r="A31" s="30">
+        <v>27</v>
+      </c>
+      <c r="B31" s="38"/>
+      <c r="C31" s="38"/>
+      <c r="D31" s="38"/>
+      <c r="E31" s="38"/>
+      <c r="F31" s="38"/>
+      <c r="G31" s="38"/>
+      <c r="H31" s="38"/>
+      <c r="I31" s="38"/>
+    </row>
+    <row r="32" spans="1:9">
+      <c r="A32" s="30">
+        <v>28</v>
+      </c>
+      <c r="B32" s="38"/>
+      <c r="C32" s="38"/>
+      <c r="D32" s="38"/>
+      <c r="E32" s="38"/>
+      <c r="F32" s="38"/>
+      <c r="G32" s="38"/>
+      <c r="H32" s="38"/>
+      <c r="I32" s="38"/>
+    </row>
+    <row r="33" spans="1:9">
+      <c r="A33" s="30">
+        <v>29</v>
+      </c>
+      <c r="B33" s="38"/>
+      <c r="C33" s="38"/>
+      <c r="D33" s="38"/>
+      <c r="E33" s="38"/>
+      <c r="F33" s="38"/>
+      <c r="G33" s="38"/>
+      <c r="H33" s="38"/>
+      <c r="I33" s="38"/>
+    </row>
+    <row r="34" spans="1:9">
+      <c r="A34" s="30">
+        <v>30</v>
+      </c>
+      <c r="B34" s="38"/>
+      <c r="C34" s="38"/>
+      <c r="D34" s="38"/>
+      <c r="E34" s="38"/>
+      <c r="F34" s="38"/>
+      <c r="G34" s="38"/>
+      <c r="H34" s="38"/>
+      <c r="I34" s="38"/>
+    </row>
+    <row r="35" spans="1:9">
+      <c r="A35" s="30">
+        <v>31</v>
+      </c>
+      <c r="B35" s="38"/>
+      <c r="C35" s="38"/>
+      <c r="D35" s="38"/>
+      <c r="E35" s="38"/>
+      <c r="F35" s="38"/>
+      <c r="G35" s="38"/>
+      <c r="H35" s="38"/>
+      <c r="I35" s="38"/>
+    </row>
+    <row r="36" spans="1:9">
+      <c r="A36" s="30">
+        <v>32</v>
+      </c>
+      <c r="B36" s="38"/>
+      <c r="C36" s="38"/>
+      <c r="D36" s="38"/>
+      <c r="E36" s="38"/>
+      <c r="F36" s="38"/>
+      <c r="G36" s="38"/>
+      <c r="H36" s="38"/>
+      <c r="I36" s="38"/>
+    </row>
+    <row r="37" spans="1:9">
+      <c r="A37" s="30">
+        <v>33</v>
+      </c>
+      <c r="B37" s="38"/>
+      <c r="C37" s="38"/>
+      <c r="D37" s="38"/>
+      <c r="E37" s="38"/>
+      <c r="F37" s="38"/>
+      <c r="G37" s="38"/>
+      <c r="H37" s="38"/>
+      <c r="I37" s="38"/>
+    </row>
+    <row r="38" spans="1:9">
+      <c r="A38" s="30">
+        <v>34</v>
+      </c>
+      <c r="B38" s="38"/>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="38"/>
+      <c r="F38" s="38"/>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+      <c r="I38" s="38"/>
+    </row>
+    <row r="39" spans="1:9">
+      <c r="A39" s="30">
+        <v>35</v>
+      </c>
+      <c r="B39" s="38"/>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="38"/>
+      <c r="F39" s="38"/>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+      <c r="I39" s="38"/>
+    </row>
+    <row r="40" spans="1:9">
+      <c r="A40" s="30">
+        <v>36</v>
+      </c>
+      <c r="B40" s="38"/>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="38"/>
+      <c r="F40" s="38"/>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+      <c r="I40" s="38"/>
+    </row>
+    <row r="41" spans="1:9">
+      <c r="A41" s="30">
+        <v>37</v>
+      </c>
+      <c r="B41" s="38"/>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="38"/>
+      <c r="F41" s="38"/>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+      <c r="I41" s="38"/>
+    </row>
+    <row r="42" spans="1:9">
+      <c r="A42" s="30">
+        <v>38</v>
+      </c>
+      <c r="B42" s="38"/>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="38"/>
+      <c r="F42" s="38"/>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+      <c r="I42" s="38"/>
+    </row>
+    <row r="43" spans="1:9">
+      <c r="A43" s="30">
+        <v>39</v>
+      </c>
+      <c r="B43" s="38"/>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="38"/>
+      <c r="F43" s="38"/>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+      <c r="I43" s="38"/>
+    </row>
+    <row r="44" spans="1:9">
+      <c r="A44" s="30">
+        <v>40</v>
+      </c>
+      <c r="B44" s="38"/>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="38"/>
+      <c r="F44" s="38"/>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+      <c r="I44" s="38"/>
+    </row>
+    <row r="45" spans="1:9">
+      <c r="A45" s="30">
+        <v>41</v>
+      </c>
+      <c r="B45" s="38"/>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="38"/>
+      <c r="F45" s="38"/>
+      <c r="G45" s="38"/>
+      <c r="H45" s="38"/>
+      <c r="I45" s="38"/>
+    </row>
+    <row r="46" spans="1:9">
+      <c r="A46" s="30">
+        <v>42</v>
+      </c>
+      <c r="B46" s="38"/>
+      <c r="C46" s="38"/>
+      <c r="D46" s="38"/>
+      <c r="E46" s="38"/>
+      <c r="F46" s="38"/>
+      <c r="G46" s="38"/>
+      <c r="H46" s="38"/>
+      <c r="I46" s="38"/>
+    </row>
+    <row r="47" spans="1:9">
+      <c r="A47" s="30">
+        <v>43</v>
+      </c>
+      <c r="B47" s="38"/>
+      <c r="C47" s="38"/>
+      <c r="D47" s="38"/>
+      <c r="E47" s="38"/>
+      <c r="F47" s="38"/>
+      <c r="G47" s="38"/>
+      <c r="H47" s="38"/>
+      <c r="I47" s="38"/>
+    </row>
+    <row r="48" spans="1:9">
+      <c r="A48" s="30">
+        <v>44</v>
+      </c>
+      <c r="B48" s="38"/>
+      <c r="C48" s="38"/>
+      <c r="D48" s="38"/>
+      <c r="E48" s="38"/>
+      <c r="F48" s="38"/>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+      <c r="I48" s="38"/>
+    </row>
+    <row r="49" spans="1:9">
+      <c r="A49" s="30">
+        <v>45</v>
+      </c>
+      <c r="B49" s="38"/>
+      <c r="C49" s="38"/>
+      <c r="D49" s="38"/>
+      <c r="E49" s="38"/>
+      <c r="F49" s="38"/>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+      <c r="I49" s="38"/>
+    </row>
+    <row r="50" spans="1:9">
+      <c r="A50" s="30">
+        <v>46</v>
+      </c>
+      <c r="B50" s="38"/>
+      <c r="C50" s="38"/>
+      <c r="D50" s="38"/>
+      <c r="E50" s="38"/>
+      <c r="F50" s="38"/>
+      <c r="G50" s="38"/>
+      <c r="H50" s="38"/>
+      <c r="I50" s="38"/>
+    </row>
+    <row r="51" spans="1:9">
+      <c r="A51" s="30">
+        <v>47</v>
+      </c>
+      <c r="B51" s="38"/>
+      <c r="C51" s="38"/>
+      <c r="D51" s="38"/>
+      <c r="E51" s="38"/>
+      <c r="F51" s="38"/>
+      <c r="G51" s="38"/>
+      <c r="H51" s="38"/>
+      <c r="I51" s="38"/>
+    </row>
+    <row r="52" spans="1:9">
+      <c r="A52" s="30">
+        <v>48</v>
+      </c>
+      <c r="B52" s="38"/>
+      <c r="C52" s="38"/>
+      <c r="D52" s="38"/>
+      <c r="E52" s="38"/>
+      <c r="F52" s="38"/>
+      <c r="G52" s="38"/>
+      <c r="H52" s="38"/>
+      <c r="I52" s="38"/>
+    </row>
+    <row r="53" spans="1:9">
+      <c r="A53" s="30">
+        <v>49</v>
+      </c>
+      <c r="B53" s="38"/>
+      <c r="C53" s="38"/>
+      <c r="D53" s="38"/>
+      <c r="E53" s="38"/>
+      <c r="F53" s="38"/>
+      <c r="G53" s="38"/>
+      <c r="H53" s="38"/>
+      <c r="I53" s="38"/>
+    </row>
+    <row r="54" spans="1:9">
+      <c r="A54" s="30">
+        <v>50</v>
+      </c>
+      <c r="B54" s="38"/>
+      <c r="C54" s="38"/>
+      <c r="D54" s="38"/>
+      <c r="E54" s="38"/>
+      <c r="F54" s="38"/>
+      <c r="G54" s="38"/>
+      <c r="H54" s="38"/>
+      <c r="I54" s="38"/>
+    </row>
+    <row r="55" spans="1:9">
+      <c r="A55" s="30">
+        <v>51</v>
+      </c>
+      <c r="B55" s="38"/>
+      <c r="C55" s="38"/>
+      <c r="D55" s="38"/>
+      <c r="E55" s="38"/>
+      <c r="F55" s="38"/>
+      <c r="G55" s="38"/>
+      <c r="H55" s="38"/>
+      <c r="I55" s="38"/>
+    </row>
+    <row r="56" spans="1:9">
+      <c r="A56" s="30">
+        <v>52</v>
+      </c>
+      <c r="B56" s="38"/>
+      <c r="C56" s="38"/>
+      <c r="D56" s="38"/>
+      <c r="E56" s="38"/>
+      <c r="F56" s="38"/>
+      <c r="G56" s="38"/>
+      <c r="H56" s="38"/>
+      <c r="I56" s="38"/>
+    </row>
+    <row r="57" spans="1:9">
+      <c r="A57" s="30">
+        <v>53</v>
+      </c>
+      <c r="B57" s="38"/>
+      <c r="C57" s="38"/>
+      <c r="D57" s="38"/>
+      <c r="E57" s="38"/>
+      <c r="F57" s="38"/>
+      <c r="G57" s="38"/>
+      <c r="H57" s="38"/>
+      <c r="I57" s="38"/>
+    </row>
+    <row r="58" spans="1:9">
+      <c r="A58" s="30">
+        <v>54</v>
+      </c>
+      <c r="B58" s="38"/>
+      <c r="C58" s="38"/>
+      <c r="D58" s="38"/>
+      <c r="E58" s="38"/>
+      <c r="F58" s="38"/>
+      <c r="G58" s="38"/>
+      <c r="H58" s="38"/>
+      <c r="I58" s="38"/>
+    </row>
+    <row r="59" spans="1:9">
+      <c r="A59" s="30">
+        <v>55</v>
+      </c>
+      <c r="B59" s="38"/>
+      <c r="C59" s="38"/>
+      <c r="D59" s="38"/>
+      <c r="E59" s="38"/>
+      <c r="F59" s="38"/>
+      <c r="G59" s="38"/>
+      <c r="H59" s="38"/>
+      <c r="I59" s="38"/>
+    </row>
+    <row r="60" spans="1:9">
+      <c r="A60" s="30">
+        <v>56</v>
+      </c>
+      <c r="B60" s="38"/>
+      <c r="C60" s="38"/>
+      <c r="D60" s="38"/>
+      <c r="E60" s="38"/>
+      <c r="F60" s="38"/>
+      <c r="G60" s="38"/>
+      <c r="H60" s="38"/>
+      <c r="I60" s="38"/>
+    </row>
+    <row r="61" spans="1:9">
+      <c r="A61" s="30">
+        <v>57</v>
+      </c>
+      <c r="B61" s="38"/>
+      <c r="C61" s="38"/>
+      <c r="D61" s="38"/>
+      <c r="E61" s="38"/>
+      <c r="F61" s="38"/>
+      <c r="G61" s="38"/>
+      <c r="H61" s="38"/>
+      <c r="I61" s="38"/>
+    </row>
+    <row r="62" spans="1:9">
+      <c r="A62" s="30">
+        <v>58</v>
+      </c>
+      <c r="B62" s="38"/>
+      <c r="C62" s="38"/>
+      <c r="D62" s="38"/>
+      <c r="E62" s="38"/>
+      <c r="F62" s="38"/>
+      <c r="G62" s="38"/>
+      <c r="H62" s="38"/>
+      <c r="I62" s="38"/>
+    </row>
+    <row r="63" spans="1:9">
+      <c r="A63" s="30">
+        <v>59</v>
+      </c>
+      <c r="B63" s="38"/>
+      <c r="C63" s="38"/>
+      <c r="D63" s="38"/>
+      <c r="E63" s="38"/>
+      <c r="F63" s="38"/>
+      <c r="G63" s="38"/>
+      <c r="H63" s="38"/>
+      <c r="I63" s="38"/>
+    </row>
+    <row r="64" spans="1:9">
+      <c r="A64" s="30">
+        <v>60</v>
+      </c>
+      <c r="B64" s="38"/>
+      <c r="C64" s="38"/>
+      <c r="D64" s="38"/>
+      <c r="E64" s="38"/>
+      <c r="F64" s="38"/>
+      <c r="G64" s="38"/>
+      <c r="H64" s="38"/>
+      <c r="I64" s="38"/>
+    </row>
+    <row r="65" spans="1:9">
+      <c r="A65" s="30">
+        <v>61</v>
+      </c>
+      <c r="B65" s="38"/>
+      <c r="C65" s="38"/>
+      <c r="D65" s="38"/>
+      <c r="E65" s="38"/>
+      <c r="F65" s="38"/>
+      <c r="G65" s="38"/>
+      <c r="H65" s="38"/>
+      <c r="I65" s="38"/>
+    </row>
+    <row r="66" spans="1:9">
+      <c r="A66" s="30">
+        <v>62</v>
+      </c>
+      <c r="B66" s="38"/>
+      <c r="C66" s="38"/>
+      <c r="D66" s="38"/>
+      <c r="E66" s="38"/>
+      <c r="F66" s="38"/>
+      <c r="G66" s="38"/>
+      <c r="H66" s="38"/>
+      <c r="I66" s="38"/>
+    </row>
+    <row r="67" spans="1:9">
+      <c r="A67" s="30">
+        <v>63</v>
+      </c>
+      <c r="B67" s="38"/>
+      <c r="C67" s="38"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="38"/>
+      <c r="F67" s="38"/>
+      <c r="G67" s="38"/>
+      <c r="H67" s="38"/>
+      <c r="I67" s="38"/>
+    </row>
+    <row r="68" spans="1:9">
+      <c r="A68" s="30">
+        <v>64</v>
+      </c>
+      <c r="B68" s="38"/>
+      <c r="C68" s="38"/>
+      <c r="D68" s="38"/>
+      <c r="E68" s="38"/>
+      <c r="F68" s="38"/>
+      <c r="G68" s="38"/>
+      <c r="H68" s="38"/>
+      <c r="I68" s="38"/>
+    </row>
+    <row r="69" spans="1:9">
+      <c r="A69" s="30">
+        <v>65</v>
+      </c>
+      <c r="B69" s="38"/>
+      <c r="C69" s="38"/>
+      <c r="D69" s="38"/>
+      <c r="E69" s="38"/>
+      <c r="F69" s="38"/>
+      <c r="G69" s="38"/>
+      <c r="H69" s="38"/>
+      <c r="I69" s="38"/>
+    </row>
+    <row r="70" spans="1:9">
+      <c r="A70" s="30">
+        <v>66</v>
+      </c>
+      <c r="B70" s="38"/>
+      <c r="C70" s="38"/>
+      <c r="D70" s="38"/>
+      <c r="E70" s="38"/>
+      <c r="F70" s="38"/>
+      <c r="G70" s="38"/>
+      <c r="H70" s="38"/>
+      <c r="I70" s="38"/>
+    </row>
+    <row r="71" spans="1:9">
+      <c r="A71" s="30">
+        <v>67</v>
+      </c>
+      <c r="B71" s="38"/>
+      <c r="C71" s="38"/>
+      <c r="D71" s="38"/>
+      <c r="E71" s="38"/>
+      <c r="F71" s="38"/>
+      <c r="G71" s="38"/>
+      <c r="H71" s="38"/>
+      <c r="I71" s="38"/>
+    </row>
+    <row r="72" spans="1:9">
+      <c r="A72" s="30">
+        <v>68</v>
+      </c>
+      <c r="B72" s="38"/>
+      <c r="C72" s="38"/>
+      <c r="D72" s="38"/>
+      <c r="E72" s="38"/>
+      <c r="F72" s="38"/>
+      <c r="G72" s="38"/>
+      <c r="H72" s="38"/>
+      <c r="I72" s="38"/>
+    </row>
+    <row r="73" spans="1:9">
+      <c r="A73" s="30">
+        <v>69</v>
+      </c>
+      <c r="B73" s="38"/>
+      <c r="C73" s="38"/>
+      <c r="D73" s="38"/>
+      <c r="E73" s="38"/>
+      <c r="F73" s="38"/>
+      <c r="G73" s="38"/>
+      <c r="H73" s="38"/>
+      <c r="I73" s="38"/>
+    </row>
+    <row r="74" spans="1:9">
+      <c r="A74" s="30">
+        <v>70</v>
+      </c>
+      <c r="B74" s="38"/>
+      <c r="C74" s="38"/>
+      <c r="D74" s="38"/>
+      <c r="E74" s="38"/>
+      <c r="F74" s="38"/>
+      <c r="G74" s="38"/>
+      <c r="H74" s="38"/>
+      <c r="I74" s="38"/>
+    </row>
+    <row r="75" spans="1:9">
+      <c r="A75" s="30">
+        <v>71</v>
+      </c>
+      <c r="B75" s="38"/>
+      <c r="C75" s="38"/>
+      <c r="D75" s="38"/>
+      <c r="E75" s="38"/>
+      <c r="F75" s="38"/>
+      <c r="G75" s="38"/>
+      <c r="H75" s="38"/>
+      <c r="I75" s="38"/>
+    </row>
+    <row r="76" spans="1:9">
+      <c r="A76" s="30">
+        <v>72</v>
+      </c>
+      <c r="B76" s="38"/>
+      <c r="C76" s="38"/>
+      <c r="D76" s="38"/>
+      <c r="E76" s="38"/>
+      <c r="F76" s="38"/>
+      <c r="G76" s="38"/>
+      <c r="H76" s="38"/>
+      <c r="I76" s="38"/>
+    </row>
+    <row r="77" spans="1:9">
+      <c r="A77" s="30">
+        <v>73</v>
+      </c>
+      <c r="B77" s="38"/>
+      <c r="C77" s="38"/>
+      <c r="D77" s="38"/>
+      <c r="E77" s="38"/>
+      <c r="F77" s="38"/>
+      <c r="G77" s="38"/>
+      <c r="H77" s="38"/>
+      <c r="I77" s="38"/>
+    </row>
+    <row r="78" spans="1:9">
+      <c r="A78" s="30">
+        <v>74</v>
+      </c>
+      <c r="B78" s="38"/>
+      <c r="C78" s="38"/>
+      <c r="D78" s="38"/>
+      <c r="E78" s="38"/>
+      <c r="F78" s="38"/>
+      <c r="G78" s="38"/>
+      <c r="H78" s="38"/>
+      <c r="I78" s="38"/>
+    </row>
+    <row r="79" spans="1:9">
+      <c r="A79" s="30">
+        <v>75</v>
+      </c>
+      <c r="B79" s="38"/>
+      <c r="C79" s="38"/>
+      <c r="D79" s="38"/>
+      <c r="E79" s="38"/>
+      <c r="F79" s="38"/>
+      <c r="G79" s="38"/>
+      <c r="H79" s="38"/>
+      <c r="I79" s="38"/>
+    </row>
+    <row r="80" spans="1:9">
+      <c r="A80" s="30">
+        <v>76</v>
+      </c>
+      <c r="B80" s="38"/>
+      <c r="C80" s="38"/>
+      <c r="D80" s="38"/>
+      <c r="E80" s="38"/>
+      <c r="F80" s="38"/>
+      <c r="G80" s="38"/>
+      <c r="H80" s="38"/>
+      <c r="I80" s="38"/>
+    </row>
+    <row r="81" spans="1:9">
+      <c r="A81" s="30">
+        <v>77</v>
+      </c>
+      <c r="B81" s="38"/>
+      <c r="C81" s="38"/>
+      <c r="D81" s="38"/>
+      <c r="E81" s="38"/>
+      <c r="F81" s="38"/>
+      <c r="G81" s="38"/>
+      <c r="H81" s="38"/>
+      <c r="I81" s="38"/>
+    </row>
+    <row r="82" spans="1:9">
+      <c r="A82" s="30">
+        <v>78</v>
+      </c>
+      <c r="B82" s="38"/>
+      <c r="C82" s="38"/>
+      <c r="D82" s="38"/>
+      <c r="E82" s="38"/>
+      <c r="F82" s="38"/>
+      <c r="G82" s="38"/>
+      <c r="H82" s="38"/>
+      <c r="I82" s="38"/>
+    </row>
+    <row r="83" spans="1:9">
+      <c r="A83" s="30">
+        <v>79</v>
+      </c>
+      <c r="B83" s="38"/>
+      <c r="C83" s="38"/>
+      <c r="D83" s="38"/>
+      <c r="E83" s="38"/>
+      <c r="F83" s="38"/>
+      <c r="G83" s="38"/>
+      <c r="H83" s="38"/>
+      <c r="I83" s="38"/>
+    </row>
+    <row r="84" spans="1:9">
+      <c r="A84" s="30">
+        <v>80</v>
+      </c>
+      <c r="B84" s="38"/>
+      <c r="C84" s="38"/>
+      <c r="D84" s="38"/>
+      <c r="E84" s="38"/>
+      <c r="F84" s="38"/>
+      <c r="G84" s="38"/>
+      <c r="H84" s="38"/>
+      <c r="I84" s="38"/>
+    </row>
+    <row r="85" spans="1:9">
+      <c r="A85" s="30">
+        <v>81</v>
+      </c>
+      <c r="B85" s="38"/>
+      <c r="C85" s="38"/>
+      <c r="D85" s="38"/>
+      <c r="E85" s="38"/>
+      <c r="F85" s="38"/>
+      <c r="G85" s="38"/>
+      <c r="H85" s="38"/>
+      <c r="I85" s="38"/>
+    </row>
+    <row r="86" spans="1:9">
+      <c r="A86" s="30">
+        <v>82</v>
+      </c>
+      <c r="B86" s="38"/>
+      <c r="C86" s="38"/>
+      <c r="D86" s="38"/>
+      <c r="E86" s="38"/>
+      <c r="F86" s="38"/>
+      <c r="G86" s="38"/>
+      <c r="H86" s="38"/>
+      <c r="I86" s="38"/>
+    </row>
+    <row r="87" spans="1:9">
+      <c r="A87" s="30">
+        <v>83</v>
+      </c>
+      <c r="B87" s="38"/>
+      <c r="C87" s="38"/>
+      <c r="D87" s="38"/>
+      <c r="E87" s="38"/>
+      <c r="F87" s="38"/>
+      <c r="G87" s="38"/>
+      <c r="H87" s="38"/>
+      <c r="I87" s="38"/>
+    </row>
+    <row r="88" spans="1:9">
+      <c r="A88" s="30">
+        <v>84</v>
+      </c>
+      <c r="B88" s="38"/>
+      <c r="C88" s="38"/>
+      <c r="D88" s="38"/>
+      <c r="E88" s="38"/>
+      <c r="F88" s="38"/>
+      <c r="G88" s="38"/>
+      <c r="H88" s="38"/>
+      <c r="I88" s="38"/>
+    </row>
+    <row r="89" spans="1:9">
+      <c r="A89" s="30">
+        <v>85</v>
+      </c>
+      <c r="B89" s="38"/>
+      <c r="C89" s="38"/>
+      <c r="D89" s="38"/>
+      <c r="E89" s="38"/>
+      <c r="F89" s="38"/>
+      <c r="G89" s="38"/>
+      <c r="H89" s="38"/>
+      <c r="I89" s="38"/>
+    </row>
+    <row r="90" spans="1:9">
+      <c r="A90" s="30">
+        <v>86</v>
+      </c>
+      <c r="B90" s="38"/>
+      <c r="C90" s="38"/>
+      <c r="D90" s="38"/>
+      <c r="E90" s="38"/>
+      <c r="F90" s="38"/>
+      <c r="G90" s="38"/>
+      <c r="H90" s="38"/>
+      <c r="I90" s="38"/>
+    </row>
+    <row r="91" spans="1:9">
+      <c r="A91" s="30">
+        <v>87</v>
+      </c>
+      <c r="B91" s="38"/>
+      <c r="C91" s="38"/>
+      <c r="D91" s="38"/>
+      <c r="E91" s="38"/>
+      <c r="F91" s="38"/>
+      <c r="G91" s="38"/>
+      <c r="H91" s="38"/>
+      <c r="I91" s="38"/>
+    </row>
+    <row r="92" spans="1:9">
+      <c r="A92" s="30">
+        <v>88</v>
+      </c>
+      <c r="B92" s="38"/>
+      <c r="C92" s="38"/>
+      <c r="D92" s="38"/>
+      <c r="E92" s="38"/>
+      <c r="F92" s="38"/>
+      <c r="G92" s="38"/>
+      <c r="H92" s="38"/>
+      <c r="I92" s="38"/>
+    </row>
+    <row r="93" spans="1:9">
+      <c r="A93" s="30">
+        <v>89</v>
+      </c>
+      <c r="B93" s="38"/>
+      <c r="C93" s="38"/>
+      <c r="D93" s="38"/>
+      <c r="E93" s="38"/>
+      <c r="F93" s="38"/>
+      <c r="G93" s="38"/>
+      <c r="H93" s="38"/>
+      <c r="I93" s="38"/>
+    </row>
+    <row r="94" spans="1:9">
+      <c r="A94" s="30">
+        <v>90</v>
+      </c>
+      <c r="B94" s="38"/>
+      <c r="C94" s="38"/>
+      <c r="D94" s="38"/>
+      <c r="E94" s="38"/>
+      <c r="F94" s="38"/>
+      <c r="G94" s="38"/>
+      <c r="H94" s="38"/>
+      <c r="I94" s="38"/>
+    </row>
+    <row r="95" spans="1:9">
+      <c r="A95" s="30">
+        <v>91</v>
+      </c>
+      <c r="B95" s="38"/>
+      <c r="C95" s="38"/>
+      <c r="D95" s="38"/>
+      <c r="E95" s="38"/>
+      <c r="F95" s="38"/>
+      <c r="G95" s="38"/>
+      <c r="H95" s="38"/>
+      <c r="I95" s="38"/>
+    </row>
+    <row r="96" spans="1:9">
+      <c r="A96" s="30">
+        <v>92</v>
+      </c>
+      <c r="B96" s="38"/>
+      <c r="C96" s="38"/>
+      <c r="D96" s="38"/>
+      <c r="E96" s="38"/>
+      <c r="F96" s="38"/>
+      <c r="G96" s="38"/>
+      <c r="H96" s="38"/>
+      <c r="I96" s="38"/>
+    </row>
+    <row r="97" spans="1:9">
+      <c r="A97" s="30">
+        <v>93</v>
+      </c>
+      <c r="B97" s="38"/>
+      <c r="C97" s="38"/>
+      <c r="D97" s="38"/>
+      <c r="E97" s="38"/>
+      <c r="F97" s="38"/>
+      <c r="G97" s="38"/>
+      <c r="H97" s="38"/>
+      <c r="I97" s="38"/>
+    </row>
+    <row r="98" spans="1:9">
+      <c r="A98" s="30">
+        <v>94</v>
+      </c>
+      <c r="B98" s="38"/>
+      <c r="C98" s="38"/>
+      <c r="D98" s="38"/>
+      <c r="E98" s="38"/>
+      <c r="F98" s="38"/>
+      <c r="G98" s="38"/>
+      <c r="H98" s="38"/>
+      <c r="I98" s="38"/>
+    </row>
+    <row r="99" spans="1:9">
+      <c r="A99" s="30">
+        <v>95</v>
+      </c>
+      <c r="B99" s="38"/>
+      <c r="C99" s="38"/>
+      <c r="D99" s="38"/>
+      <c r="E99" s="38"/>
+      <c r="F99" s="38"/>
+      <c r="G99" s="38"/>
+      <c r="H99" s="38"/>
+      <c r="I99" s="38"/>
+    </row>
+    <row r="100" spans="1:9">
+      <c r="A100" s="30">
+        <v>96</v>
+      </c>
+      <c r="B100" s="38"/>
+      <c r="C100" s="38"/>
+      <c r="D100" s="38"/>
+      <c r="E100" s="38"/>
+      <c r="F100" s="38"/>
+      <c r="G100" s="38"/>
+      <c r="H100" s="38"/>
+      <c r="I100" s="38"/>
+    </row>
+    <row r="101" spans="1:9">
+      <c r="A101" s="30">
+        <v>97</v>
+      </c>
+      <c r="B101" s="38"/>
+      <c r="C101" s="38"/>
+      <c r="D101" s="38"/>
+      <c r="E101" s="38"/>
+      <c r="F101" s="38"/>
+      <c r="G101" s="38"/>
+      <c r="H101" s="38"/>
+      <c r="I101" s="38"/>
+    </row>
+    <row r="102" spans="1:9">
+      <c r="A102" s="30">
+        <v>98</v>
+      </c>
+      <c r="B102" s="38"/>
+      <c r="C102" s="38"/>
+      <c r="D102" s="38"/>
+      <c r="E102" s="38"/>
+      <c r="F102" s="38"/>
+      <c r="G102" s="38"/>
+      <c r="H102" s="38"/>
+      <c r="I102" s="38"/>
+    </row>
+    <row r="103" spans="1:9">
+      <c r="A103" s="30">
+        <v>99</v>
+      </c>
+      <c r="B103" s="38"/>
+      <c r="C103" s="38"/>
+      <c r="D103" s="38"/>
+      <c r="E103" s="38"/>
+      <c r="F103" s="38"/>
+      <c r="G103" s="38"/>
+      <c r="H103" s="38"/>
+      <c r="I103" s="38"/>
+    </row>
+    <row r="104" spans="1:9">
+      <c r="A104" s="30">
+        <v>100</v>
+      </c>
+      <c r="B104" s="38"/>
+      <c r="C104" s="38"/>
+      <c r="D104" s="38"/>
+      <c r="E104" s="38"/>
+      <c r="F104" s="38"/>
+      <c r="G104" s="38"/>
+      <c r="H104" s="38"/>
+      <c r="I104" s="38"/>
+    </row>
+    <row r="105" spans="1:9">
+      <c r="A105" s="30">
+        <v>101</v>
+      </c>
+      <c r="B105" s="38"/>
+      <c r="C105" s="38"/>
+      <c r="D105" s="38"/>
+      <c r="E105" s="38"/>
+      <c r="F105" s="38"/>
+      <c r="G105" s="38"/>
+      <c r="H105" s="38"/>
+      <c r="I105" s="38"/>
+    </row>
+    <row r="106" spans="1:9">
+      <c r="A106" s="30">
+        <v>102</v>
+      </c>
+      <c r="B106" s="38"/>
+      <c r="C106" s="38"/>
+      <c r="D106" s="38"/>
+      <c r="E106" s="38"/>
+      <c r="F106" s="38"/>
+      <c r="G106" s="38"/>
+      <c r="H106" s="38"/>
+      <c r="I106" s="38"/>
+    </row>
+    <row r="107" spans="1:9">
+      <c r="A107" s="30">
+        <v>103</v>
+      </c>
+      <c r="B107" s="38"/>
+      <c r="C107" s="38"/>
+      <c r="D107" s="38"/>
+      <c r="E107" s="38"/>
+      <c r="F107" s="38"/>
+      <c r="G107" s="38"/>
+      <c r="H107" s="38"/>
+      <c r="I107" s="38"/>
+    </row>
+    <row r="108" spans="1:9">
+      <c r="A108" s="30">
+        <v>104</v>
+      </c>
+      <c r="B108" s="38"/>
+      <c r="C108" s="38"/>
+      <c r="D108" s="38"/>
+      <c r="E108" s="38"/>
+      <c r="F108" s="38"/>
+      <c r="G108" s="38"/>
+      <c r="H108" s="38"/>
+      <c r="I108" s="38"/>
+    </row>
+    <row r="109" spans="1:9">
+      <c r="A109" s="30">
+        <v>105</v>
+      </c>
+      <c r="B109" s="38"/>
+      <c r="C109" s="38"/>
+      <c r="D109" s="38"/>
+      <c r="E109" s="38"/>
+      <c r="F109" s="38"/>
+      <c r="G109" s="38"/>
+      <c r="H109" s="38"/>
+      <c r="I109" s="38"/>
+    </row>
+    <row r="110" spans="1:9">
+      <c r="A110" s="30">
+        <v>106</v>
+      </c>
+      <c r="B110" s="38"/>
+      <c r="C110" s="38"/>
+      <c r="D110" s="38"/>
+      <c r="E110" s="38"/>
+      <c r="F110" s="38"/>
+      <c r="G110" s="38"/>
+      <c r="H110" s="38"/>
+      <c r="I110" s="38"/>
+    </row>
+    <row r="111" spans="1:9">
+      <c r="A111" s="30">
+        <v>107</v>
+      </c>
+      <c r="B111" s="38"/>
+      <c r="C111" s="38"/>
+      <c r="D111" s="38"/>
+      <c r="E111" s="38"/>
+      <c r="F111" s="38"/>
+      <c r="G111" s="38"/>
+      <c r="H111" s="38"/>
+      <c r="I111" s="38"/>
+    </row>
+    <row r="112" spans="1:9">
+      <c r="A112" s="30">
+        <v>108</v>
+      </c>
+      <c r="B112" s="38"/>
+      <c r="C112" s="38"/>
+      <c r="D112" s="38"/>
+      <c r="E112" s="38"/>
+      <c r="F112" s="38"/>
+      <c r="G112" s="38"/>
+      <c r="H112" s="38"/>
+      <c r="I112" s="38"/>
+    </row>
+    <row r="113" spans="1:9">
+      <c r="A113" s="30">
+        <v>109</v>
+      </c>
+      <c r="B113" s="38"/>
+      <c r="C113" s="38"/>
+      <c r="D113" s="38"/>
+      <c r="E113" s="38"/>
+      <c r="F113" s="38"/>
+      <c r="G113" s="38"/>
+      <c r="H113" s="38"/>
+      <c r="I113" s="38"/>
+    </row>
+    <row r="114" spans="1:9">
+      <c r="A114" s="30">
+        <v>110</v>
+      </c>
+      <c r="B114" s="38"/>
+      <c r="C114" s="38"/>
+      <c r="D114" s="38"/>
+      <c r="E114" s="38"/>
+      <c r="F114" s="38"/>
+      <c r="G114" s="38"/>
+      <c r="H114" s="38"/>
+      <c r="I114" s="38"/>
+    </row>
+    <row r="115" spans="1:9">
+      <c r="A115" s="30">
+        <v>111</v>
+      </c>
+      <c r="B115" s="38"/>
+      <c r="C115" s="38"/>
+      <c r="D115" s="38"/>
+      <c r="E115" s="38"/>
+      <c r="F115" s="38"/>
+      <c r="G115" s="38"/>
+      <c r="H115" s="38"/>
+      <c r="I115" s="38"/>
+    </row>
+    <row r="116" spans="1:9">
+      <c r="A116" s="30">
+        <v>112</v>
+      </c>
+      <c r="B116" s="38"/>
+      <c r="C116" s="38"/>
+      <c r="D116" s="38"/>
+      <c r="E116" s="38"/>
+      <c r="F116" s="38"/>
+      <c r="G116" s="38"/>
+      <c r="H116" s="38"/>
+      <c r="I116" s="38"/>
+    </row>
+    <row r="117" spans="1:9">
+      <c r="A117" s="30">
+        <v>113</v>
+      </c>
+      <c r="B117" s="38"/>
+      <c r="C117" s="38"/>
+      <c r="D117" s="38"/>
+      <c r="E117" s="38"/>
+      <c r="F117" s="38"/>
+      <c r="G117" s="38"/>
+      <c r="H117" s="38"/>
+      <c r="I117" s="38"/>
+    </row>
+    <row r="118" spans="1:9">
+      <c r="A118" s="30">
+        <v>114</v>
+      </c>
+      <c r="B118" s="38"/>
+      <c r="C118" s="38"/>
+      <c r="D118" s="38"/>
+      <c r="E118" s="38"/>
+      <c r="F118" s="38"/>
+      <c r="G118" s="38"/>
+      <c r="H118" s="38"/>
+      <c r="I118" s="38"/>
+    </row>
+    <row r="119" spans="1:9">
+      <c r="A119" s="30">
+        <v>115</v>
+      </c>
+      <c r="B119" s="38"/>
+      <c r="C119" s="38"/>
+      <c r="D119" s="38"/>
+      <c r="E119" s="38"/>
+      <c r="F119" s="38"/>
+      <c r="G119" s="38"/>
+      <c r="H119" s="38"/>
+      <c r="I119" s="38"/>
+    </row>
+    <row r="120" spans="1:9">
+      <c r="A120" s="30">
+        <v>116</v>
+      </c>
+      <c r="B120" s="38"/>
+      <c r="C120" s="38"/>
+      <c r="D120" s="38"/>
+      <c r="E120" s="38"/>
+      <c r="F120" s="38"/>
+      <c r="G120" s="38"/>
+      <c r="H120" s="38"/>
+      <c r="I120" s="38"/>
+    </row>
+    <row r="121" spans="1:9">
+      <c r="A121" s="30">
+        <v>117</v>
+      </c>
+      <c r="B121" s="38"/>
+      <c r="C121" s="38"/>
+      <c r="D121" s="38"/>
+      <c r="E121" s="38"/>
+      <c r="F121" s="38"/>
+      <c r="G121" s="38"/>
+      <c r="H121" s="38"/>
+      <c r="I121" s="38"/>
+    </row>
+    <row r="122" spans="1:9">
+      <c r="A122" s="30">
+        <v>118</v>
+      </c>
+      <c r="B122" s="38"/>
+      <c r="C122" s="38"/>
+      <c r="D122" s="38"/>
+      <c r="E122" s="38"/>
+      <c r="F122" s="38"/>
+      <c r="G122" s="38"/>
+      <c r="H122" s="38"/>
+      <c r="I122" s="38"/>
+    </row>
+    <row r="123" spans="1:9">
+      <c r="A123" s="30">
+        <v>119</v>
+      </c>
+      <c r="B123" s="38"/>
+      <c r="C123" s="38"/>
+      <c r="D123" s="38"/>
+      <c r="E123" s="38"/>
+      <c r="F123" s="38"/>
+      <c r="G123" s="38"/>
+      <c r="H123" s="38"/>
+      <c r="I123" s="38"/>
+    </row>
+    <row r="124" spans="1:9">
+      <c r="A124" s="30">
+        <v>120</v>
+      </c>
+      <c r="B124" s="38"/>
+      <c r="C124" s="38"/>
+      <c r="D124" s="38"/>
+      <c r="E124" s="38"/>
+      <c r="F124" s="38"/>
+      <c r="G124" s="38"/>
+      <c r="H124" s="38"/>
+      <c r="I124" s="38"/>
+    </row>
+    <row r="125" spans="1:9">
+      <c r="A125" s="30">
+        <v>121</v>
+      </c>
+      <c r="B125" s="38"/>
+      <c r="C125" s="38"/>
+      <c r="D125" s="38"/>
+      <c r="E125" s="38"/>
+      <c r="F125" s="38"/>
+      <c r="G125" s="38"/>
+      <c r="H125" s="38"/>
+      <c r="I125" s="38"/>
+    </row>
+    <row r="126" spans="1:9">
+      <c r="A126" s="30">
+        <v>122</v>
+      </c>
+      <c r="B126" s="38"/>
+      <c r="C126" s="38"/>
+      <c r="D126" s="38"/>
+      <c r="E126" s="38"/>
+      <c r="F126" s="38"/>
+      <c r="G126" s="38"/>
+      <c r="H126" s="38"/>
+      <c r="I126" s="38"/>
+    </row>
+    <row r="127" spans="1:9">
+      <c r="A127" s="30">
+        <v>123</v>
+      </c>
+      <c r="B127" s="38"/>
+      <c r="C127" s="38"/>
+      <c r="D127" s="38"/>
+      <c r="E127" s="38"/>
+      <c r="F127" s="38"/>
+      <c r="G127" s="38"/>
+      <c r="H127" s="38"/>
+      <c r="I127" s="38"/>
+    </row>
+    <row r="128" spans="1:9">
+      <c r="A128" s="30">
+        <v>124</v>
+      </c>
+      <c r="B128" s="38"/>
+      <c r="C128" s="38"/>
+      <c r="D128" s="38"/>
+      <c r="E128" s="38"/>
+      <c r="F128" s="38"/>
+      <c r="G128" s="38"/>
+      <c r="H128" s="38"/>
+      <c r="I128" s="38"/>
+    </row>
+    <row r="129" spans="1:9">
+      <c r="A129" s="30">
+        <v>125</v>
+      </c>
+      <c r="B129" s="38"/>
+      <c r="C129" s="38"/>
+      <c r="D129" s="38"/>
+      <c r="E129" s="38"/>
+      <c r="F129" s="38"/>
+      <c r="G129" s="38"/>
+      <c r="H129" s="38"/>
+      <c r="I129" s="38"/>
+    </row>
+    <row r="130" spans="1:9">
+      <c r="A130" s="30">
+        <v>126</v>
+      </c>
+      <c r="B130" s="38"/>
+      <c r="C130" s="38"/>
+      <c r="D130" s="38"/>
+      <c r="E130" s="38"/>
+      <c r="F130" s="38"/>
+      <c r="G130" s="38"/>
+      <c r="H130" s="38"/>
+      <c r="I130" s="38"/>
+    </row>
+    <row r="131" spans="1:9">
+      <c r="A131" s="30">
+        <v>127</v>
+      </c>
+      <c r="B131" s="38"/>
+      <c r="C131" s="38"/>
+      <c r="D131" s="38"/>
+      <c r="E131" s="38"/>
+      <c r="F131" s="38"/>
+      <c r="G131" s="38"/>
+      <c r="H131" s="38"/>
+      <c r="I131" s="38"/>
+    </row>
+    <row r="132" spans="1:9">
+      <c r="A132" s="30">
+        <v>128</v>
+      </c>
+      <c r="B132" s="38"/>
+      <c r="C132" s="38"/>
+      <c r="D132" s="38"/>
+      <c r="E132" s="38"/>
+      <c r="F132" s="38"/>
+      <c r="G132" s="38"/>
+      <c r="H132" s="38"/>
+      <c r="I132" s="38"/>
+    </row>
+    <row r="133" spans="1:9">
+      <c r="A133" s="30">
+        <v>129</v>
+      </c>
+      <c r="B133" s="38"/>
+      <c r="C133" s="38"/>
+      <c r="D133" s="38"/>
+      <c r="E133" s="38"/>
+      <c r="F133" s="38"/>
+      <c r="G133" s="38"/>
+      <c r="H133" s="38"/>
+      <c r="I133" s="38"/>
+    </row>
+    <row r="134" spans="1:9">
+      <c r="A134" s="30">
+        <v>130</v>
+      </c>
+      <c r="B134" s="38"/>
+      <c r="C134" s="38"/>
+      <c r="D134" s="38"/>
+      <c r="E134" s="38"/>
+      <c r="F134" s="38"/>
+      <c r="G134" s="38"/>
+      <c r="H134" s="38"/>
+      <c r="I134" s="38"/>
+    </row>
+    <row r="135" spans="1:9">
+      <c r="A135" s="30">
+        <v>131</v>
+      </c>
+      <c r="B135" s="38"/>
+      <c r="C135" s="38"/>
+      <c r="D135" s="38"/>
+      <c r="E135" s="38"/>
+      <c r="F135" s="38"/>
+      <c r="G135" s="38"/>
+      <c r="H135" s="38"/>
+      <c r="I135" s="38"/>
+    </row>
+    <row r="136" spans="1:9">
+      <c r="A136" s="30">
+        <v>132</v>
+      </c>
+      <c r="B136" s="38"/>
+      <c r="C136" s="38"/>
+      <c r="D136" s="38"/>
+      <c r="E136" s="38"/>
+      <c r="F136" s="38"/>
+      <c r="G136" s="38"/>
+      <c r="H136" s="38"/>
+      <c r="I136" s="38"/>
+    </row>
+    <row r="137" spans="1:9">
+      <c r="A137" s="30">
+        <v>133</v>
+      </c>
+      <c r="B137" s="38"/>
+      <c r="C137" s="38"/>
+      <c r="D137" s="38"/>
+      <c r="E137" s="38"/>
+      <c r="F137" s="38"/>
+      <c r="G137" s="38"/>
+      <c r="H137" s="38"/>
+      <c r="I137" s="38"/>
+    </row>
+    <row r="138" spans="1:9">
+      <c r="A138" s="30">
+        <v>134</v>
+      </c>
+      <c r="B138" s="38"/>
+      <c r="C138" s="38"/>
+      <c r="D138" s="38"/>
+      <c r="E138" s="38"/>
+      <c r="F138" s="38"/>
+      <c r="G138" s="38"/>
+      <c r="H138" s="38"/>
+      <c r="I138" s="38"/>
+    </row>
+    <row r="139" spans="1:9">
+      <c r="A139" s="30">
+        <v>135</v>
+      </c>
+      <c r="B139" s="38"/>
+      <c r="C139" s="38"/>
+      <c r="D139" s="38"/>
+      <c r="E139" s="38"/>
+      <c r="F139" s="38"/>
+      <c r="G139" s="38"/>
+      <c r="H139" s="38"/>
+      <c r="I139" s="38"/>
+    </row>
+    <row r="140" spans="1:9">
+      <c r="A140" s="30">
+        <v>136</v>
+      </c>
+      <c r="B140" s="38"/>
+      <c r="C140" s="38"/>
+      <c r="D140" s="38"/>
+      <c r="E140" s="38"/>
+      <c r="F140" s="38"/>
+      <c r="G140" s="38"/>
+      <c r="H140" s="38"/>
+      <c r="I140" s="38"/>
+    </row>
+    <row r="141" spans="1:9">
+      <c r="A141" s="30">
+        <v>137</v>
+      </c>
+      <c r="B141" s="38"/>
+      <c r="C141" s="38"/>
+      <c r="D141" s="38"/>
+      <c r="E141" s="38"/>
+      <c r="F141" s="38"/>
+      <c r="G141" s="38"/>
+      <c r="H141" s="38"/>
+      <c r="I141" s="38"/>
+    </row>
+    <row r="142" spans="1:9">
+      <c r="A142" s="30">
+        <v>138</v>
+      </c>
+      <c r="B142" s="38"/>
+      <c r="C142" s="38"/>
+      <c r="D142" s="38"/>
+      <c r="E142" s="38"/>
+      <c r="F142" s="38"/>
+      <c r="G142" s="38"/>
+      <c r="H142" s="38"/>
+      <c r="I142" s="38"/>
+    </row>
+    <row r="143" spans="1:9">
+      <c r="A143" s="30">
+        <v>139</v>
+      </c>
+      <c r="B143" s="38"/>
+      <c r="C143" s="38"/>
+      <c r="D143" s="38"/>
+      <c r="E143" s="38"/>
+      <c r="F143" s="38"/>
+      <c r="G143" s="38"/>
+      <c r="H143" s="38"/>
+      <c r="I143" s="38"/>
+    </row>
+    <row r="144" spans="1:9">
+      <c r="A144" s="30">
+        <v>140</v>
+      </c>
+      <c r="B144" s="38"/>
+      <c r="C144" s="38"/>
+      <c r="D144" s="38"/>
+      <c r="E144" s="38"/>
+      <c r="F144" s="38"/>
+      <c r="G144" s="38"/>
+      <c r="H144" s="38"/>
+      <c r="I144" s="38"/>
+    </row>
+    <row r="145" spans="1:9">
+      <c r="A145" s="30">
+        <v>141</v>
+      </c>
+      <c r="B145" s="38"/>
+      <c r="C145" s="38"/>
+      <c r="D145" s="38"/>
+      <c r="E145" s="38"/>
+      <c r="F145" s="38"/>
+      <c r="G145" s="38"/>
+      <c r="H145" s="38"/>
+      <c r="I145" s="38"/>
+    </row>
+    <row r="146" spans="1:9">
+      <c r="A146" s="30">
+        <v>142</v>
+      </c>
+      <c r="B146" s="38"/>
+      <c r="C146" s="38"/>
+      <c r="D146" s="38"/>
+      <c r="E146" s="38"/>
+      <c r="F146" s="38"/>
+      <c r="G146" s="38"/>
+      <c r="H146" s="38"/>
+      <c r="I146" s="38"/>
+    </row>
+    <row r="147" spans="1:9">
+      <c r="A147" s="30">
+        <v>143</v>
+      </c>
+      <c r="B147" s="38"/>
+      <c r="C147" s="38"/>
+      <c r="D147" s="38"/>
+      <c r="E147" s="38"/>
+      <c r="F147" s="38"/>
+      <c r="G147" s="38"/>
+      <c r="H147" s="38"/>
+      <c r="I147" s="38"/>
+    </row>
+    <row r="148" spans="1:9">
+      <c r="A148" s="30">
+        <v>144</v>
+      </c>
+      <c r="B148" s="38"/>
+      <c r="C148" s="38"/>
+      <c r="D148" s="38"/>
+      <c r="E148" s="38"/>
+      <c r="F148" s="38"/>
+      <c r="G148" s="38"/>
+      <c r="H148" s="38"/>
+      <c r="I148" s="38"/>
+    </row>
+    <row r="149" spans="1:9">
+      <c r="A149" s="30">
+        <v>145</v>
+      </c>
+      <c r="B149" s="38"/>
+      <c r="C149" s="38"/>
+      <c r="D149" s="38"/>
+      <c r="E149" s="38"/>
+      <c r="F149" s="38"/>
+      <c r="G149" s="38"/>
+      <c r="H149" s="38"/>
+      <c r="I149" s="38"/>
+    </row>
+    <row r="150" spans="1:9">
+      <c r="A150" s="30">
+        <v>146</v>
+      </c>
+      <c r="B150" s="38"/>
+      <c r="C150" s="38"/>
+      <c r="D150" s="38"/>
+      <c r="E150" s="38"/>
+      <c r="F150" s="38"/>
+      <c r="G150" s="38"/>
+      <c r="H150" s="38"/>
+      <c r="I150" s="38"/>
+    </row>
+    <row r="151" spans="1:9">
+      <c r="A151" s="30">
+        <v>147</v>
+      </c>
+      <c r="B151" s="38"/>
+      <c r="C151" s="38"/>
+      <c r="D151" s="38"/>
+      <c r="E151" s="38"/>
+      <c r="F151" s="38"/>
+      <c r="G151" s="38"/>
+      <c r="H151" s="38"/>
+      <c r="I151" s="38"/>
+    </row>
+    <row r="152" spans="1:9">
+      <c r="A152" s="30">
+        <v>148</v>
+      </c>
+      <c r="B152" s="38"/>
+      <c r="C152" s="38"/>
+      <c r="D152" s="38"/>
+      <c r="E152" s="38"/>
+      <c r="F152" s="38"/>
+      <c r="G152" s="38"/>
+      <c r="H152" s="38"/>
+      <c r="I152" s="38"/>
+    </row>
+    <row r="153" spans="1:9">
+      <c r="A153" s="30">
+        <v>149</v>
+      </c>
+      <c r="B153" s="38"/>
+      <c r="C153" s="38"/>
+      <c r="D153" s="38"/>
+      <c r="E153" s="38"/>
+      <c r="F153" s="38"/>
+      <c r="G153" s="38"/>
+      <c r="H153" s="38"/>
+      <c r="I153" s="38"/>
+    </row>
+    <row r="154" spans="1:9">
+      <c r="A154" s="30">
+        <v>150</v>
+      </c>
+      <c r="B154" s="38"/>
+      <c r="C154" s="38"/>
+      <c r="D154" s="38"/>
+      <c r="E154" s="38"/>
+      <c r="F154" s="38"/>
+      <c r="G154" s="38"/>
+      <c r="H154" s="38"/>
+      <c r="I154" s="38"/>
+    </row>
+    <row r="155" spans="1:9">
+      <c r="A155" s="30">
+        <v>151</v>
+      </c>
+      <c r="B155" s="38"/>
+      <c r="C155" s="38"/>
+      <c r="D155" s="38"/>
+      <c r="E155" s="38"/>
+      <c r="F155" s="38"/>
+      <c r="G155" s="38"/>
+      <c r="H155" s="38"/>
+      <c r="I155" s="38"/>
+    </row>
+    <row r="156" spans="1:9">
+      <c r="A156" s="30">
+        <v>152</v>
+      </c>
+      <c r="B156" s="38"/>
+      <c r="C156" s="38"/>
+      <c r="D156" s="38"/>
+      <c r="E156" s="38"/>
+      <c r="F156" s="38"/>
+      <c r="G156" s="38"/>
+      <c r="H156" s="38"/>
+      <c r="I156" s="38"/>
+    </row>
+    <row r="157" spans="1:9">
+      <c r="A157" s="30">
+        <v>153</v>
+      </c>
+      <c r="B157" s="38"/>
+      <c r="C157" s="38"/>
+      <c r="D157" s="38"/>
+      <c r="E157" s="38"/>
+      <c r="F157" s="38"/>
+      <c r="G157" s="38"/>
+      <c r="H157" s="38"/>
+      <c r="I157" s="38"/>
+    </row>
+    <row r="158" spans="1:9">
+      <c r="A158" s="30">
+        <v>154</v>
+      </c>
+      <c r="B158" s="38"/>
+      <c r="C158" s="38"/>
+      <c r="D158" s="38"/>
+      <c r="E158" s="38"/>
+      <c r="F158" s="38"/>
+      <c r="G158" s="38"/>
+      <c r="H158" s="38"/>
+      <c r="I158" s="38"/>
+    </row>
+    <row r="159" spans="1:9">
+      <c r="A159" s="30">
+        <v>155</v>
+      </c>
+      <c r="B159" s="38"/>
+      <c r="C159" s="38"/>
+      <c r="D159" s="38"/>
+      <c r="E159" s="38"/>
+      <c r="F159" s="38"/>
+      <c r="G159" s="38"/>
+      <c r="H159" s="38"/>
+      <c r="I159" s="38"/>
+    </row>
+    <row r="160" spans="1:9">
+      <c r="A160" s="30">
+        <v>156</v>
+      </c>
+      <c r="B160" s="38"/>
+      <c r="C160" s="38"/>
+      <c r="D160" s="38"/>
+      <c r="E160" s="38"/>
+      <c r="F160" s="38"/>
+      <c r="G160" s="38"/>
+      <c r="H160" s="38"/>
+      <c r="I160" s="38"/>
+    </row>
+    <row r="161" spans="1:9">
+      <c r="A161" s="30">
+        <v>157</v>
+      </c>
+      <c r="B161" s="38"/>
+      <c r="C161" s="38"/>
+      <c r="D161" s="38"/>
+      <c r="E161" s="38"/>
+      <c r="F161" s="38"/>
+      <c r="G161" s="38"/>
+      <c r="H161" s="38"/>
+      <c r="I161" s="38"/>
+    </row>
+    <row r="162" spans="1:9">
+      <c r="A162" s="30">
+        <v>158</v>
+      </c>
+      <c r="B162" s="38"/>
+      <c r="C162" s="38"/>
+      <c r="D162" s="38"/>
+      <c r="E162" s="38"/>
+      <c r="F162" s="38"/>
+      <c r="G162" s="38"/>
+      <c r="H162" s="38"/>
+      <c r="I162" s="38"/>
+    </row>
+    <row r="163" spans="1:9">
+      <c r="A163" s="30">
+        <v>159</v>
+      </c>
+      <c r="B163" s="38"/>
+      <c r="C163" s="38"/>
+      <c r="D163" s="38"/>
+      <c r="E163" s="38"/>
+      <c r="F163" s="38"/>
+      <c r="G163" s="38"/>
+      <c r="H163" s="38"/>
+      <c r="I163" s="38"/>
+    </row>
+    <row r="164" spans="1:9">
+      <c r="A164" s="30">
+        <v>160</v>
+      </c>
+      <c r="B164" s="38"/>
+      <c r="C164" s="38"/>
+      <c r="D164" s="38"/>
+      <c r="E164" s="38"/>
+      <c r="F164" s="38"/>
+      <c r="G164" s="38"/>
+      <c r="H164" s="38"/>
+      <c r="I164" s="38"/>
+    </row>
+    <row r="165" spans="1:9">
+      <c r="A165" s="30">
+        <v>161</v>
+      </c>
+      <c r="B165" s="38"/>
+      <c r="C165" s="38"/>
+      <c r="D165" s="38"/>
+      <c r="E165" s="38"/>
+      <c r="F165" s="38"/>
+      <c r="G165" s="38"/>
+      <c r="H165" s="38"/>
+      <c r="I165" s="38"/>
+    </row>
+    <row r="166" spans="1:9">
+      <c r="A166" s="30">
+        <v>162</v>
+      </c>
+      <c r="B166" s="38"/>
+      <c r="C166" s="38"/>
+      <c r="D166" s="38"/>
+      <c r="E166" s="38"/>
+      <c r="F166" s="38"/>
+      <c r="G166" s="38"/>
+      <c r="H166" s="38"/>
+      <c r="I166" s="38"/>
+    </row>
+    <row r="167" spans="1:9">
+      <c r="A167" s="30">
+        <v>163</v>
+      </c>
+      <c r="B167" s="38"/>
+      <c r="C167" s="38"/>
+      <c r="D167" s="38"/>
+      <c r="E167" s="38"/>
+      <c r="F167" s="38"/>
+      <c r="G167" s="38"/>
+      <c r="H167" s="38"/>
+      <c r="I167" s="38"/>
+    </row>
+    <row r="168" spans="1:9">
+      <c r="A168" s="30">
+        <v>164</v>
+      </c>
+      <c r="B168" s="38"/>
+      <c r="C168" s="38"/>
+      <c r="D168" s="38"/>
+      <c r="E168" s="38"/>
+      <c r="F168" s="38"/>
+      <c r="G168" s="38"/>
+      <c r="H168" s="38"/>
+      <c r="I168" s="38"/>
+    </row>
+    <row r="169" spans="1:9">
+      <c r="A169" s="30">
+        <v>165</v>
+      </c>
+      <c r="B169" s="38"/>
+      <c r="C169" s="38"/>
+      <c r="D169" s="38"/>
+      <c r="E169" s="38"/>
+      <c r="F169" s="38"/>
+      <c r="G169" s="38"/>
+      <c r="H169" s="38"/>
+      <c r="I169" s="38"/>
+    </row>
+    <row r="170" spans="1:9">
+      <c r="A170" s="30">
+        <v>166</v>
+      </c>
+      <c r="B170" s="38"/>
+      <c r="C170" s="38"/>
+      <c r="D170" s="38"/>
+      <c r="E170" s="38"/>
+      <c r="F170" s="38"/>
+      <c r="G170" s="38"/>
+      <c r="H170" s="38"/>
+      <c r="I170" s="38"/>
+    </row>
+    <row r="171" spans="1:9">
+      <c r="A171" s="30">
+        <v>167</v>
+      </c>
+      <c r="B171" s="38"/>
+      <c r="C171" s="38"/>
+      <c r="D171" s="38"/>
+      <c r="E171" s="38"/>
+      <c r="F171" s="38"/>
+      <c r="G171" s="38"/>
+      <c r="H171" s="38"/>
+      <c r="I171" s="38"/>
+    </row>
+    <row r="172" spans="1:9">
+      <c r="A172" s="30">
+        <v>168</v>
+      </c>
+      <c r="B172" s="38"/>
+      <c r="C172" s="38"/>
+      <c r="D172" s="38"/>
+      <c r="E172" s="38"/>
+      <c r="F172" s="38"/>
+      <c r="G172" s="38"/>
+      <c r="H172" s="38"/>
+      <c r="I172" s="38"/>
+    </row>
+    <row r="173" spans="1:9">
+      <c r="A173" s="30">
+        <v>169</v>
+      </c>
+      <c r="B173" s="38"/>
+      <c r="C173" s="38"/>
+      <c r="D173" s="38"/>
+      <c r="E173" s="38"/>
+      <c r="F173" s="38"/>
+      <c r="G173" s="38"/>
+      <c r="H173" s="38"/>
+      <c r="I173" s="38"/>
+    </row>
+    <row r="174" spans="1:9">
+      <c r="A174" s="30">
+        <v>170</v>
+      </c>
+      <c r="B174" s="38"/>
+      <c r="C174" s="38"/>
+      <c r="D174" s="38"/>
+      <c r="E174" s="38"/>
+      <c r="F174" s="38"/>
+      <c r="G174" s="38"/>
+      <c r="H174" s="38"/>
+      <c r="I174" s="38"/>
+    </row>
+    <row r="175" spans="1:9">
+      <c r="A175" s="30">
+        <v>171</v>
+      </c>
+      <c r="B175" s="38"/>
+      <c r="C175" s="38"/>
+      <c r="D175" s="38"/>
+      <c r="E175" s="38"/>
+      <c r="F175" s="38"/>
+      <c r="G175" s="38"/>
+      <c r="H175" s="38"/>
+      <c r="I175" s="38"/>
+    </row>
+    <row r="176" spans="1:9">
+      <c r="A176" s="30">
+        <v>172</v>
+      </c>
+      <c r="B176" s="38"/>
+      <c r="C176" s="38"/>
+      <c r="D176" s="38"/>
+      <c r="E176" s="38"/>
+      <c r="F176" s="38"/>
+      <c r="G176" s="38"/>
+      <c r="H176" s="38"/>
+      <c r="I176" s="38"/>
+    </row>
+    <row r="177" spans="1:9">
+      <c r="A177" s="30">
+        <v>173</v>
+      </c>
+      <c r="B177" s="38"/>
+      <c r="C177" s="38"/>
+      <c r="D177" s="38"/>
+      <c r="E177" s="38"/>
+      <c r="F177" s="38"/>
+      <c r="G177" s="38"/>
+      <c r="H177" s="38"/>
+      <c r="I177" s="38"/>
+    </row>
+    <row r="178" spans="1:9">
+      <c r="A178" s="30">
+        <v>174</v>
+      </c>
+      <c r="B178" s="38"/>
+      <c r="C178" s="38"/>
+      <c r="D178" s="38"/>
+      <c r="E178" s="38"/>
+      <c r="F178" s="38"/>
+      <c r="G178" s="38"/>
+      <c r="H178" s="38"/>
+      <c r="I178" s="38"/>
+    </row>
+    <row r="179" spans="1:9">
+      <c r="A179" s="30">
+        <v>175</v>
+      </c>
+      <c r="B179" s="38"/>
+      <c r="C179" s="38"/>
+      <c r="D179" s="38"/>
+      <c r="E179" s="38"/>
+      <c r="F179" s="38"/>
+      <c r="G179" s="38"/>
+      <c r="H179" s="38"/>
+      <c r="I179" s="38"/>
+    </row>
+    <row r="180" spans="1:9">
+      <c r="A180" s="30">
+        <v>176</v>
+      </c>
+      <c r="B180" s="38"/>
+      <c r="C180" s="38"/>
+      <c r="D180" s="38"/>
+      <c r="E180" s="38"/>
+      <c r="F180" s="38"/>
+      <c r="G180" s="38"/>
+      <c r="H180" s="38"/>
+      <c r="I180" s="38"/>
+    </row>
+    <row r="181" spans="1:9">
+      <c r="A181" s="30">
+        <v>177</v>
+      </c>
+      <c r="B181" s="38"/>
+      <c r="C181" s="38"/>
+      <c r="D181" s="38"/>
+      <c r="E181" s="38"/>
+      <c r="F181" s="38"/>
+      <c r="G181" s="38"/>
+      <c r="H181" s="38"/>
+      <c r="I181" s="38"/>
+    </row>
+    <row r="182" spans="1:9">
+      <c r="A182" s="30">
+        <v>178</v>
+      </c>
+      <c r="B182" s="38"/>
+      <c r="C182" s="38"/>
+      <c r="D182" s="38"/>
+      <c r="E182" s="38"/>
+      <c r="F182" s="38"/>
+      <c r="G182" s="38"/>
+      <c r="H182" s="38"/>
+      <c r="I182" s="38"/>
+    </row>
+    <row r="183" spans="1:9">
+      <c r="A183" s="30">
+        <v>179</v>
+      </c>
+      <c r="B183" s="38"/>
+      <c r="C183" s="38"/>
+      <c r="D183" s="38"/>
+      <c r="E183" s="38"/>
+      <c r="F183" s="38"/>
+      <c r="G183" s="38"/>
+      <c r="H183" s="38"/>
+      <c r="I183" s="38"/>
+    </row>
+    <row r="184" spans="1:9">
+      <c r="A184" s="30">
+        <v>180</v>
+      </c>
+      <c r="B184" s="38"/>
+      <c r="C184" s="38"/>
+      <c r="D184" s="38"/>
+      <c r="E184" s="38"/>
+      <c r="F184" s="38"/>
+      <c r="G184" s="38"/>
+      <c r="H184" s="38"/>
+      <c r="I184" s="38"/>
+    </row>
+    <row r="185" spans="1:9">
+      <c r="A185" s="30">
+        <v>181</v>
+      </c>
+      <c r="B185" s="38"/>
+      <c r="C185" s="38"/>
+      <c r="D185" s="38"/>
+      <c r="E185" s="38"/>
+      <c r="F185" s="38"/>
+      <c r="G185" s="38"/>
+      <c r="H185" s="38"/>
+      <c r="I185" s="38"/>
+    </row>
+    <row r="186" spans="1:9">
+      <c r="A186" s="30">
+        <v>182</v>
+      </c>
+      <c r="B186" s="38"/>
+      <c r="C186" s="38"/>
+      <c r="D186" s="38"/>
+      <c r="E186" s="38"/>
+      <c r="F186" s="38"/>
+      <c r="G186" s="38"/>
+      <c r="H186" s="38"/>
+      <c r="I186" s="38"/>
+    </row>
+    <row r="187" spans="1:9">
+      <c r="A187" s="30">
+        <v>183</v>
+      </c>
+      <c r="B187" s="38"/>
+      <c r="C187" s="38"/>
+      <c r="D187" s="38"/>
+      <c r="E187" s="38"/>
+      <c r="F187" s="38"/>
+      <c r="G187" s="38"/>
+      <c r="H187" s="38"/>
+      <c r="I187" s="38"/>
+    </row>
+    <row r="188" spans="1:9">
+      <c r="A188" s="30">
+        <v>184</v>
+      </c>
+      <c r="B188" s="38"/>
+      <c r="C188" s="38"/>
+      <c r="D188" s="38"/>
+      <c r="E188" s="38"/>
+      <c r="F188" s="38"/>
+      <c r="G188" s="38"/>
+      <c r="H188" s="38"/>
+      <c r="I188" s="38"/>
+    </row>
+    <row r="189" spans="1:9">
+      <c r="A189" s="30">
+        <v>185</v>
+      </c>
+      <c r="B189" s="38"/>
+      <c r="C189" s="38"/>
+      <c r="D189" s="38"/>
+      <c r="E189" s="38"/>
+      <c r="F189" s="38"/>
+      <c r="G189" s="38"/>
+      <c r="H189" s="38"/>
+      <c r="I189" s="38"/>
+    </row>
+    <row r="190" spans="1:9">
+      <c r="A190" s="30">
+        <v>186</v>
+      </c>
+      <c r="B190" s="38"/>
+      <c r="C190" s="38"/>
+      <c r="D190" s="38"/>
+      <c r="E190" s="38"/>
+      <c r="F190" s="38"/>
+      <c r="G190" s="38"/>
+      <c r="H190" s="38"/>
+      <c r="I190" s="38"/>
+    </row>
+    <row r="191" spans="1:9">
+      <c r="A191" s="30">
+        <v>187</v>
+      </c>
+      <c r="B191" s="38"/>
+      <c r="C191" s="38"/>
+      <c r="D191" s="38"/>
+      <c r="E191" s="38"/>
+      <c r="F191" s="38"/>
+      <c r="G191" s="38"/>
+      <c r="H191" s="38"/>
+      <c r="I191" s="38"/>
+    </row>
+    <row r="192" spans="1:9">
+      <c r="A192" s="30">
+        <v>188</v>
+      </c>
+      <c r="B192" s="38"/>
+      <c r="C192" s="38"/>
+      <c r="D192" s="38"/>
+      <c r="E192" s="38"/>
+      <c r="F192" s="38"/>
+      <c r="G192" s="38"/>
+      <c r="H192" s="38"/>
+      <c r="I192" s="38"/>
+    </row>
+    <row r="193" spans="1:9">
+      <c r="A193" s="30">
+        <v>189</v>
+      </c>
+      <c r="B193" s="38"/>
+      <c r="C193" s="38"/>
+      <c r="D193" s="38"/>
+      <c r="E193" s="38"/>
+      <c r="F193" s="38"/>
+      <c r="G193" s="38"/>
+      <c r="H193" s="38"/>
+      <c r="I193" s="38"/>
+    </row>
+    <row r="194" spans="1:9">
+      <c r="A194" s="30">
+        <v>190</v>
+      </c>
+      <c r="B194" s="38"/>
+      <c r="C194" s="38"/>
+      <c r="D194" s="38"/>
+      <c r="E194" s="38"/>
+      <c r="F194" s="38"/>
+      <c r="G194" s="38"/>
+      <c r="H194" s="38"/>
+      <c r="I194" s="38"/>
+    </row>
+    <row r="195" spans="1:9">
+      <c r="A195" s="30">
+        <v>191</v>
+      </c>
+      <c r="B195" s="38"/>
+      <c r="C195" s="38"/>
+      <c r="D195" s="38"/>
+      <c r="E195" s="38"/>
+      <c r="F195" s="38"/>
+      <c r="G195" s="38"/>
+      <c r="H195" s="38"/>
+      <c r="I195" s="38"/>
+    </row>
+    <row r="196" spans="1:9">
+      <c r="A196" s="30">
+        <v>192</v>
+      </c>
+      <c r="B196" s="38"/>
+      <c r="C196" s="38"/>
+      <c r="D196" s="38"/>
+      <c r="E196" s="38"/>
+      <c r="F196" s="38"/>
+      <c r="G196" s="38"/>
+      <c r="H196" s="38"/>
+      <c r="I196" s="38"/>
+    </row>
+    <row r="197" spans="1:9">
+      <c r="A197" s="30">
+        <v>193</v>
+      </c>
+      <c r="B197" s="38"/>
+      <c r="C197" s="38"/>
+      <c r="D197" s="38"/>
+      <c r="E197" s="38"/>
+      <c r="F197" s="38"/>
+      <c r="G197" s="38"/>
+      <c r="H197" s="38"/>
+      <c r="I197" s="38"/>
+    </row>
+    <row r="198" spans="1:9">
+      <c r="A198" s="30">
+        <v>194</v>
+      </c>
+      <c r="B198" s="38"/>
+      <c r="C198" s="38"/>
+      <c r="D198" s="38"/>
+      <c r="E198" s="38"/>
+      <c r="F198" s="38"/>
+      <c r="G198" s="38"/>
+      <c r="H198" s="38"/>
+      <c r="I198" s="38"/>
+    </row>
+    <row r="199" spans="1:9">
+      <c r="A199" s="30">
+        <v>195</v>
+      </c>
+      <c r="B199" s="38"/>
+      <c r="C199" s="38"/>
+      <c r="D199" s="38"/>
+      <c r="E199" s="38"/>
+      <c r="F199" s="38"/>
+      <c r="G199" s="38"/>
+      <c r="H199" s="38"/>
+      <c r="I199" s="38"/>
+    </row>
+    <row r="200" spans="1:9">
+      <c r="A200" s="30">
+        <v>196</v>
+      </c>
+      <c r="B200" s="38"/>
+      <c r="C200" s="38"/>
+      <c r="D200" s="38"/>
+      <c r="E200" s="38"/>
+      <c r="F200" s="38"/>
+      <c r="G200" s="38"/>
+      <c r="H200" s="38"/>
+      <c r="I200" s="38"/>
+    </row>
+    <row r="201" spans="1:9">
+      <c r="A201" s="30">
+        <v>197</v>
+      </c>
+      <c r="B201" s="38"/>
+      <c r="C201" s="38"/>
+      <c r="D201" s="38"/>
+      <c r="E201" s="38"/>
+      <c r="F201" s="38"/>
+      <c r="G201" s="38"/>
+      <c r="H201" s="38"/>
+      <c r="I201" s="38"/>
+    </row>
+    <row r="202" spans="1:9">
+      <c r="A202" s="30">
+        <v>198</v>
+      </c>
+      <c r="B202" s="38"/>
+      <c r="C202" s="38"/>
+      <c r="D202" s="38"/>
+      <c r="E202" s="38"/>
+      <c r="F202" s="38"/>
+      <c r="G202" s="38"/>
+      <c r="H202" s="38"/>
+      <c r="I202" s="38"/>
+    </row>
+    <row r="203" spans="1:9">
+      <c r="A203" s="30">
+        <v>199</v>
+      </c>
+      <c r="B203" s="38"/>
+      <c r="C203" s="38"/>
+      <c r="D203" s="38"/>
+      <c r="E203" s="38"/>
+      <c r="F203" s="38"/>
+      <c r="G203" s="38"/>
+      <c r="H203" s="38"/>
+      <c r="I203" s="38"/>
+    </row>
+    <row r="204" spans="1:9">
+      <c r="A204" s="30">
+        <v>200</v>
+      </c>
+      <c r="B204" s="38"/>
+      <c r="C204" s="38"/>
+      <c r="D204" s="38"/>
+      <c r="E204" s="38"/>
+      <c r="F204" s="38"/>
+      <c r="G204" s="38"/>
+      <c r="H204" s="38"/>
+      <c r="I204" s="38"/>
+    </row>
+    <row r="205" spans="1:9">
+      <c r="A205" s="30">
+        <v>201</v>
+      </c>
+      <c r="B205" s="38"/>
+      <c r="C205" s="38"/>
+      <c r="D205" s="38"/>
+      <c r="E205" s="38"/>
+      <c r="F205" s="38"/>
+      <c r="G205" s="38"/>
+      <c r="H205" s="38"/>
+      <c r="I205" s="38"/>
+    </row>
+    <row r="206" spans="1:9">
+      <c r="A206" s="30">
+        <v>202</v>
+      </c>
+      <c r="B206" s="38"/>
+      <c r="C206" s="38"/>
+      <c r="D206" s="38"/>
+      <c r="E206" s="38"/>
+      <c r="F206" s="38"/>
+      <c r="G206" s="38"/>
+      <c r="H206" s="38"/>
+      <c r="I206" s="38"/>
+    </row>
+    <row r="207" spans="1:9">
+      <c r="A207" s="30">
+        <v>203</v>
+      </c>
+      <c r="B207" s="38"/>
+      <c r="C207" s="38"/>
+      <c r="D207" s="38"/>
+      <c r="E207" s="38"/>
+      <c r="F207" s="38"/>
+      <c r="G207" s="38"/>
+      <c r="H207" s="38"/>
+      <c r="I207" s="38"/>
+    </row>
+    <row r="208" spans="1:9">
+      <c r="A208" s="30">
+        <v>204</v>
+      </c>
+      <c r="B208" s="38"/>
+      <c r="C208" s="38"/>
+      <c r="D208" s="38"/>
+      <c r="E208" s="38"/>
+      <c r="F208" s="38"/>
+      <c r="G208" s="38"/>
+      <c r="H208" s="38"/>
+      <c r="I208" s="38"/>
+    </row>
+    <row r="209" spans="1:9">
+      <c r="A209" s="30">
+        <v>205</v>
+      </c>
+      <c r="B209" s="38"/>
+      <c r="C209" s="38"/>
+      <c r="D209" s="38"/>
+      <c r="E209" s="38"/>
+      <c r="F209" s="38"/>
+      <c r="G209" s="38"/>
+      <c r="H209" s="38"/>
+      <c r="I209" s="38"/>
+    </row>
+    <row r="210" spans="1:9">
+      <c r="A210" s="30">
+        <v>206</v>
+      </c>
+      <c r="B210" s="38"/>
+      <c r="C210" s="38"/>
+      <c r="D210" s="38"/>
+      <c r="E210" s="38"/>
+      <c r="F210" s="38"/>
+      <c r="G210" s="38"/>
+      <c r="H210" s="38"/>
+      <c r="I210" s="38"/>
+    </row>
+    <row r="211" spans="1:9">
+      <c r="A211" s="30">
+        <v>207</v>
+      </c>
+      <c r="B211" s="38"/>
+      <c r="C211" s="38"/>
+      <c r="D211" s="38"/>
+      <c r="E211" s="38"/>
+      <c r="F211" s="38"/>
+      <c r="G211" s="38"/>
+      <c r="H211" s="38"/>
+      <c r="I211" s="38"/>
+    </row>
+    <row r="212" spans="1:9">
+      <c r="A212" s="30">
+        <v>208</v>
+      </c>
+      <c r="B212" s="38"/>
+      <c r="C212" s="38"/>
+      <c r="D212" s="38"/>
+      <c r="E212" s="38"/>
+      <c r="F212" s="38"/>
+      <c r="G212" s="38"/>
+      <c r="H212" s="38"/>
+      <c r="I212" s="38"/>
+    </row>
+    <row r="213" spans="1:9">
+      <c r="A213" s="30">
+        <v>209</v>
+      </c>
+      <c r="B213" s="38"/>
+      <c r="C213" s="38"/>
+      <c r="D213" s="38"/>
+      <c r="E213" s="38"/>
+      <c r="F213" s="38"/>
+      <c r="G213" s="38"/>
+      <c r="H213" s="38"/>
+      <c r="I213" s="38"/>
+    </row>
+    <row r="214" spans="1:9">
+      <c r="A214" s="30">
+        <v>210</v>
+      </c>
+      <c r="B214" s="38"/>
+      <c r="C214" s="38"/>
+      <c r="D214" s="38"/>
+      <c r="E214" s="38"/>
+      <c r="F214" s="38"/>
+      <c r="G214" s="38"/>
+      <c r="H214" s="38"/>
+      <c r="I214" s="38"/>
+    </row>
+    <row r="215" spans="1:9">
+      <c r="A215" s="30">
+        <v>211</v>
+      </c>
+      <c r="B215" s="38"/>
+      <c r="C215" s="38"/>
+      <c r="D215" s="38"/>
+      <c r="E215" s="38"/>
+      <c r="F215" s="38"/>
+      <c r="G215" s="38"/>
+      <c r="H215" s="38"/>
+      <c r="I215" s="38"/>
+    </row>
+    <row r="216" spans="1:9">
+      <c r="A216" s="30">
+        <v>212</v>
+      </c>
+      <c r="B216" s="38"/>
+      <c r="C216" s="38"/>
+      <c r="D216" s="38"/>
+      <c r="E216" s="38"/>
+      <c r="F216" s="38"/>
+      <c r="G216" s="38"/>
+      <c r="H216" s="38"/>
+      <c r="I216" s="38"/>
+    </row>
+    <row r="217" spans="1:9">
+      <c r="A217" s="30">
+        <v>213</v>
+      </c>
+      <c r="B217" s="38"/>
+      <c r="C217" s="38"/>
+      <c r="D217" s="38"/>
+      <c r="E217" s="38"/>
+      <c r="F217" s="38"/>
+      <c r="G217" s="38"/>
+      <c r="H217" s="38"/>
+      <c r="I217" s="38"/>
+    </row>
+    <row r="218" spans="1:9">
+      <c r="A218" s="30">
+        <v>214</v>
+      </c>
+      <c r="B218" s="38"/>
+      <c r="C218" s="38"/>
+      <c r="D218" s="38"/>
+      <c r="E218" s="38"/>
+      <c r="F218" s="38"/>
+      <c r="G218" s="38"/>
+      <c r="H218" s="38"/>
+      <c r="I218" s="38"/>
+    </row>
+    <row r="219" spans="1:9">
+      <c r="A219" s="30">
+        <v>215</v>
+      </c>
+      <c r="B219" s="38"/>
+      <c r="C219" s="38"/>
+      <c r="D219" s="38"/>
+      <c r="E219" s="38"/>
+      <c r="F219" s="38"/>
+      <c r="G219" s="38"/>
+      <c r="H219" s="38"/>
+      <c r="I219" s="38"/>
+    </row>
+    <row r="220" spans="1:9">
+      <c r="A220" s="30">
+        <v>216</v>
+      </c>
+      <c r="B220" s="38"/>
+      <c r="C220" s="38"/>
+      <c r="D220" s="38"/>
+      <c r="E220" s="38"/>
+      <c r="F220" s="38"/>
+      <c r="G220" s="38"/>
+      <c r="H220" s="38"/>
+      <c r="I220" s="38"/>
+    </row>
+    <row r="221" spans="1:9">
+      <c r="A221" s="30">
+        <v>217</v>
+      </c>
+      <c r="B221" s="38"/>
+      <c r="C221" s="38"/>
+      <c r="D221" s="38"/>
+      <c r="E221" s="38"/>
+      <c r="F221" s="38"/>
+      <c r="G221" s="38"/>
+      <c r="H221" s="38"/>
+      <c r="I221" s="38"/>
+    </row>
+    <row r="222" spans="1:9">
+      <c r="A222" s="30">
+        <v>218</v>
+      </c>
+      <c r="B222" s="38"/>
+      <c r="C222" s="38"/>
+      <c r="D222" s="38"/>
+      <c r="E222" s="38"/>
+      <c r="F222" s="38"/>
+      <c r="G222" s="38"/>
+      <c r="H222" s="38"/>
+      <c r="I222" s="38"/>
+    </row>
+    <row r="223" spans="1:9">
+      <c r="A223" s="30">
+        <v>219</v>
+      </c>
+      <c r="B223" s="38"/>
+      <c r="C223" s="38"/>
+      <c r="D223" s="38"/>
+      <c r="E223" s="38"/>
+      <c r="F223" s="38"/>
+      <c r="G223" s="38"/>
+      <c r="H223" s="38"/>
+      <c r="I223" s="38"/>
+    </row>
+    <row r="224" spans="1:9">
+      <c r="A224" s="30">
+        <v>220</v>
+      </c>
+      <c r="B224" s="38"/>
+      <c r="C224" s="38"/>
+      <c r="D224" s="38"/>
+      <c r="E224" s="38"/>
+      <c r="F224" s="38"/>
+      <c r="G224" s="38"/>
+      <c r="H224" s="38"/>
+      <c r="I224" s="38"/>
+    </row>
+    <row r="225" spans="1:9">
+      <c r="A225" s="30">
+        <v>221</v>
+      </c>
+      <c r="B225" s="38"/>
+      <c r="C225" s="38"/>
+      <c r="D225" s="38"/>
+      <c r="E225" s="38"/>
+      <c r="F225" s="38"/>
+      <c r="G225" s="38"/>
+      <c r="H225" s="38"/>
+      <c r="I225" s="38"/>
+    </row>
+    <row r="226" spans="1:9">
+      <c r="A226" s="30">
+        <v>222</v>
+      </c>
+      <c r="B226" s="38"/>
+      <c r="C226" s="38"/>
+      <c r="D226" s="38"/>
+      <c r="E226" s="38"/>
+      <c r="F226" s="38"/>
+      <c r="G226" s="38"/>
+      <c r="H226" s="38"/>
+      <c r="I226" s="38"/>
+    </row>
+    <row r="227" spans="1:9">
+      <c r="A227" s="30">
+        <v>223</v>
+      </c>
+      <c r="B227" s="38"/>
+      <c r="C227" s="38"/>
+      <c r="D227" s="38"/>
+      <c r="E227" s="38"/>
+      <c r="F227" s="38"/>
+      <c r="G227" s="38"/>
+      <c r="H227" s="38"/>
+      <c r="I227" s="38"/>
+    </row>
+    <row r="228" spans="1:9">
+      <c r="A228" s="30">
+        <v>224</v>
+      </c>
+      <c r="B228" s="38"/>
+      <c r="C228" s="38"/>
+      <c r="D228" s="38"/>
+      <c r="E228" s="38"/>
+      <c r="F228" s="38"/>
+      <c r="G228" s="38"/>
+      <c r="H228" s="38"/>
+      <c r="I228" s="38"/>
+    </row>
+    <row r="229" spans="1:9">
+      <c r="A229" s="30">
+        <v>225</v>
+      </c>
+      <c r="B229" s="38"/>
+      <c r="C229" s="38"/>
+      <c r="D229" s="38"/>
+      <c r="E229" s="38"/>
+      <c r="F229" s="38"/>
+      <c r="G229" s="38"/>
+      <c r="H229" s="38"/>
+      <c r="I229" s="38"/>
+    </row>
+    <row r="230" spans="1:9">
+      <c r="A230" s="30">
+        <v>226</v>
+      </c>
+      <c r="B230" s="38"/>
+      <c r="C230" s="38"/>
+      <c r="D230" s="38"/>
+      <c r="E230" s="38"/>
+      <c r="F230" s="38"/>
+      <c r="G230" s="38"/>
+      <c r="H230" s="38"/>
+      <c r="I230" s="38"/>
+    </row>
+    <row r="231" spans="1:9">
+      <c r="A231" s="30">
+        <v>227</v>
+      </c>
+      <c r="B231" s="38"/>
+      <c r="C231" s="38"/>
+      <c r="D231" s="38"/>
+      <c r="E231" s="38"/>
+      <c r="F231" s="38"/>
+      <c r="G231" s="38"/>
+      <c r="H231" s="38"/>
+      <c r="I231" s="38"/>
+    </row>
+    <row r="232" spans="1:9">
+      <c r="A232" s="30">
+        <v>228</v>
+      </c>
+      <c r="B232" s="38"/>
+      <c r="C232" s="38"/>
+      <c r="D232" s="38"/>
+      <c r="E232" s="38"/>
+      <c r="F232" s="38"/>
+      <c r="G232" s="38"/>
+      <c r="H232" s="38"/>
+      <c r="I232" s="38"/>
+    </row>
+    <row r="233" spans="1:9">
+      <c r="A233" s="30">
+        <v>229</v>
+      </c>
+      <c r="B233" s="38"/>
+      <c r="C233" s="38"/>
+      <c r="D233" s="38"/>
+      <c r="E233" s="38"/>
+      <c r="F233" s="38"/>
+      <c r="G233" s="38"/>
+      <c r="H233" s="38"/>
+      <c r="I233" s="38"/>
+    </row>
+    <row r="234" spans="1:9">
+      <c r="A234" s="30">
+        <v>230</v>
+      </c>
+      <c r="B234" s="38"/>
+      <c r="C234" s="38"/>
+      <c r="D234" s="38"/>
+      <c r="E234" s="38"/>
+      <c r="F234" s="38"/>
+      <c r="G234" s="38"/>
+      <c r="H234" s="38"/>
+      <c r="I234" s="38"/>
+    </row>
+    <row r="235" spans="1:9">
+      <c r="A235" s="30">
+        <v>231</v>
+      </c>
+      <c r="B235" s="38"/>
+      <c r="C235" s="38"/>
+      <c r="D235" s="38"/>
+      <c r="E235" s="38"/>
+      <c r="F235" s="38"/>
+      <c r="G235" s="38"/>
+      <c r="H235" s="38"/>
+      <c r="I235" s="38"/>
+    </row>
+    <row r="236" spans="1:9">
+      <c r="A236" s="30">
+        <v>232</v>
+      </c>
+      <c r="B236" s="38"/>
+      <c r="C236" s="38"/>
+      <c r="D236" s="38"/>
+      <c r="E236" s="38"/>
+      <c r="F236" s="38"/>
+      <c r="G236" s="38"/>
+      <c r="H236" s="38"/>
+      <c r="I236" s="38"/>
+    </row>
+    <row r="237" spans="1:9">
+      <c r="A237" s="30">
+        <v>233</v>
+      </c>
+      <c r="B237" s="38"/>
+      <c r="C237" s="38"/>
+      <c r="D237" s="38"/>
+      <c r="E237" s="38"/>
+      <c r="F237" s="38"/>
+      <c r="G237" s="38"/>
+      <c r="H237" s="38"/>
+      <c r="I237" s="38"/>
+    </row>
+    <row r="238" spans="1:9">
+      <c r="A238" s="30">
+        <v>234</v>
+      </c>
+      <c r="B238" s="38"/>
+      <c r="C238" s="38"/>
+      <c r="D238" s="38"/>
+      <c r="E238" s="38"/>
+      <c r="F238" s="38"/>
+      <c r="G238" s="38"/>
+      <c r="H238" s="38"/>
+      <c r="I238" s="38"/>
+    </row>
+    <row r="239" spans="1:9">
+      <c r="A239" s="30">
+        <v>235</v>
+      </c>
+      <c r="B239" s="38"/>
+      <c r="C239" s="38"/>
+      <c r="D239" s="38"/>
+      <c r="E239" s="38"/>
+      <c r="F239" s="38"/>
+      <c r="G239" s="38"/>
+      <c r="H239" s="38"/>
+      <c r="I239" s="38"/>
+    </row>
+    <row r="240" spans="1:9">
+      <c r="A240" s="30">
+        <v>236</v>
+      </c>
+      <c r="B240" s="38"/>
+      <c r="C240" s="38"/>
+      <c r="D240" s="38"/>
+      <c r="E240" s="38"/>
+      <c r="F240" s="38"/>
+      <c r="G240" s="38"/>
+      <c r="H240" s="38"/>
+      <c r="I240" s="38"/>
+    </row>
+    <row r="241" spans="1:9">
+      <c r="A241" s="30">
+        <v>237</v>
+      </c>
+      <c r="B241" s="38"/>
+      <c r="C241" s="38"/>
+      <c r="D241" s="38"/>
+      <c r="E241" s="38"/>
+      <c r="F241" s="38"/>
+      <c r="G241" s="38"/>
+      <c r="H241" s="38"/>
+      <c r="I241" s="38"/>
+    </row>
+    <row r="242" spans="1:9">
+      <c r="A242" s="30">
+        <v>238</v>
+      </c>
+      <c r="B242" s="38"/>
+      <c r="C242" s="38"/>
+      <c r="D242" s="38"/>
+      <c r="E242" s="38"/>
+      <c r="F242" s="38"/>
+      <c r="G242" s="38"/>
+      <c r="H242" s="38"/>
+      <c r="I242" s="38"/>
+    </row>
+    <row r="243" spans="1:9">
+      <c r="A243" s="30">
+        <v>239</v>
+      </c>
+      <c r="B243" s="38"/>
+      <c r="C243" s="38"/>
+      <c r="D243" s="38"/>
+      <c r="E243" s="38"/>
+      <c r="F243" s="38"/>
+      <c r="G243" s="38"/>
+      <c r="H243" s="38"/>
+      <c r="I243" s="38"/>
+    </row>
+    <row r="244" spans="1:9">
+      <c r="A244" s="30">
+        <v>240</v>
+      </c>
+      <c r="B244" s="38"/>
+      <c r="C244" s="38"/>
+      <c r="D244" s="38"/>
+      <c r="E244" s="38"/>
+      <c r="F244" s="38"/>
+      <c r="G244" s="38"/>
+      <c r="H244" s="38"/>
+      <c r="I244" s="38"/>
+    </row>
+    <row r="245" spans="1:9">
+      <c r="A245" s="30">
+        <v>241</v>
+      </c>
+      <c r="B245" s="38"/>
+      <c r="C245" s="38"/>
+      <c r="D245" s="38"/>
+      <c r="E245" s="38"/>
+      <c r="F245" s="38"/>
+      <c r="G245" s="38"/>
+      <c r="H245" s="38"/>
+      <c r="I245" s="38"/>
+    </row>
+    <row r="246" spans="1:9">
+      <c r="A246" s="30">
+        <v>242</v>
+      </c>
+      <c r="B246" s="38"/>
+      <c r="C246" s="38"/>
+      <c r="D246" s="38"/>
+      <c r="E246" s="38"/>
+      <c r="F246" s="38"/>
+      <c r="G246" s="38"/>
+      <c r="H246" s="38"/>
+      <c r="I246" s="38"/>
+    </row>
+    <row r="247" spans="1:9">
+      <c r="A247" s="30">
+        <v>243</v>
+      </c>
+      <c r="B247" s="38"/>
+      <c r="C247" s="38"/>
+      <c r="D247" s="38"/>
+      <c r="E247" s="38"/>
+      <c r="F247" s="38"/>
+      <c r="G247" s="38"/>
+      <c r="H247" s="38"/>
+      <c r="I247" s="38"/>
+    </row>
+    <row r="248" spans="1:9">
+      <c r="A248" s="30">
+        <v>244</v>
+      </c>
+      <c r="B248" s="38"/>
+      <c r="C248" s="38"/>
+      <c r="D248" s="38"/>
+      <c r="E248" s="38"/>
+      <c r="F248" s="38"/>
+      <c r="G248" s="38"/>
+      <c r="H248" s="38"/>
+      <c r="I248" s="38"/>
+    </row>
+    <row r="249" spans="1:9">
+      <c r="A249" s="30">
+        <v>245</v>
+      </c>
+      <c r="B249" s="38"/>
+      <c r="C249" s="38"/>
+      <c r="D249" s="38"/>
+      <c r="E249" s="38"/>
+      <c r="F249" s="38"/>
+      <c r="G249" s="38"/>
+      <c r="H249" s="38"/>
+      <c r="I249" s="38"/>
+    </row>
+    <row r="250" spans="1:9">
+      <c r="A250" s="30">
+        <v>246</v>
+      </c>
+      <c r="B250" s="38"/>
+      <c r="C250" s="38"/>
+      <c r="D250" s="38"/>
+      <c r="E250" s="38"/>
+      <c r="F250" s="38"/>
+      <c r="G250" s="38"/>
+      <c r="H250" s="38"/>
+      <c r="I250" s="38"/>
+    </row>
+    <row r="251" spans="1:9">
+      <c r="A251" s="30">
+        <v>247</v>
+      </c>
+      <c r="B251" s="38"/>
+      <c r="C251" s="38"/>
+      <c r="D251" s="38"/>
+      <c r="E251" s="38"/>
+      <c r="F251" s="38"/>
+      <c r="G251" s="38"/>
+      <c r="H251" s="38"/>
+      <c r="I251" s="38"/>
+    </row>
+    <row r="252" spans="1:9">
+      <c r="A252" s="30">
+        <v>248</v>
+      </c>
+      <c r="B252" s="38"/>
+      <c r="C252" s="38"/>
+      <c r="D252" s="38"/>
+      <c r="E252" s="38"/>
+      <c r="F252" s="38"/>
+      <c r="G252" s="38"/>
+      <c r="H252" s="38"/>
+      <c r="I252" s="38"/>
+    </row>
+    <row r="253" spans="1:9">
+      <c r="A253" s="30">
+        <v>249</v>
+      </c>
+      <c r="B253" s="38"/>
+      <c r="C253" s="38"/>
+      <c r="D253" s="38"/>
+      <c r="E253" s="38"/>
+      <c r="F253" s="38"/>
+      <c r="G253" s="38"/>
+      <c r="H253" s="38"/>
+      <c r="I253" s="38"/>
+    </row>
+    <row r="254" spans="1:9">
+      <c r="A254" s="30">
+        <v>250</v>
+      </c>
+      <c r="B254" s="38"/>
+      <c r="C254" s="38"/>
+      <c r="D254" s="38"/>
+      <c r="E254" s="38"/>
+      <c r="F254" s="38"/>
+      <c r="G254" s="38"/>
+      <c r="H254" s="38"/>
+      <c r="I254" s="38"/>
+    </row>
+    <row r="255" spans="1:9">
+      <c r="A255" s="30">
+        <v>251</v>
+      </c>
+      <c r="B255" s="38"/>
+      <c r="C255" s="38"/>
+      <c r="D255" s="38"/>
+      <c r="E255" s="38"/>
+      <c r="F255" s="38"/>
+      <c r="G255" s="38"/>
+      <c r="H255" s="38"/>
+      <c r="I255" s="38"/>
+    </row>
+    <row r="256" spans="1:9">
+      <c r="A256" s="30">
+        <v>252</v>
+      </c>
+      <c r="B256" s="38"/>
+      <c r="C256" s="38"/>
+      <c r="D256" s="38"/>
+      <c r="E256" s="38"/>
+      <c r="F256" s="38"/>
+      <c r="G256" s="38"/>
+      <c r="H256" s="38"/>
+      <c r="I256" s="38"/>
+    </row>
+    <row r="257" spans="1:9">
+      <c r="A257" s="30">
+        <v>253</v>
+      </c>
+      <c r="B257" s="38"/>
+      <c r="C257" s="38"/>
+      <c r="D257" s="38"/>
+      <c r="E257" s="38"/>
+      <c r="F257" s="38"/>
+      <c r="G257" s="38"/>
+      <c r="H257" s="38"/>
+      <c r="I257" s="38"/>
+    </row>
+    <row r="258" spans="1:9">
+      <c r="A258" s="30">
+        <v>254</v>
+      </c>
+      <c r="B258" s="38"/>
+      <c r="C258" s="38"/>
+      <c r="D258" s="38"/>
+      <c r="E258" s="38"/>
+      <c r="F258" s="38"/>
+      <c r="G258" s="38"/>
+      <c r="H258" s="38"/>
+      <c r="I258" s="38"/>
+    </row>
+    <row r="259" spans="1:9">
+      <c r="A259" s="30">
+        <v>255</v>
+      </c>
+      <c r="B259" s="38"/>
+      <c r="C259" s="38"/>
+      <c r="D259" s="38"/>
+      <c r="E259" s="38"/>
+      <c r="F259" s="38"/>
+      <c r="G259" s="38"/>
+      <c r="H259" s="38"/>
+      <c r="I259" s="38"/>
+    </row>
+    <row r="260" spans="1:9">
+      <c r="A260" s="30">
+        <v>256</v>
+      </c>
+      <c r="B260" s="38"/>
+      <c r="C260" s="38"/>
+      <c r="D260" s="38"/>
+      <c r="E260" s="38"/>
+      <c r="F260" s="38"/>
+      <c r="G260" s="38"/>
+      <c r="H260" s="38"/>
+      <c r="I260" s="38"/>
+    </row>
+    <row r="261" spans="1:9">
+      <c r="A261" s="30">
+        <v>257</v>
+      </c>
+      <c r="B261" s="38"/>
+      <c r="C261" s="38"/>
+      <c r="D261" s="38"/>
+      <c r="E261" s="38"/>
+      <c r="F261" s="38"/>
+      <c r="G261" s="38"/>
+      <c r="H261" s="38"/>
+      <c r="I261" s="38"/>
+    </row>
+    <row r="262" spans="1:9">
+      <c r="A262" s="30">
+        <v>258</v>
+      </c>
+      <c r="B262" s="38"/>
+      <c r="C262" s="38"/>
+      <c r="D262" s="38"/>
+      <c r="E262" s="38"/>
+      <c r="F262" s="38"/>
+      <c r="G262" s="38"/>
+      <c r="H262" s="38"/>
+      <c r="I262" s="38"/>
+    </row>
+    <row r="263" spans="1:9">
+      <c r="A263" s="30">
+        <v>259</v>
+      </c>
+      <c r="B263" s="38"/>
+      <c r="C263" s="38"/>
+      <c r="D263" s="38"/>
+      <c r="E263" s="38"/>
+      <c r="F263" s="38"/>
+      <c r="G263" s="38"/>
+      <c r="H263" s="38"/>
+      <c r="I263" s="38"/>
+    </row>
+    <row r="264" spans="1:9">
+      <c r="A264" s="30">
+        <v>260</v>
+      </c>
+      <c r="B264" s="38"/>
+      <c r="C264" s="38"/>
+      <c r="D264" s="38"/>
+      <c r="E264" s="38"/>
+      <c r="F264" s="38"/>
+      <c r="G264" s="38"/>
+      <c r="H264" s="38"/>
+      <c r="I264" s="38"/>
+    </row>
+    <row r="265" spans="1:9">
+      <c r="A265" s="30">
+        <v>261</v>
+      </c>
+      <c r="B265" s="38"/>
+      <c r="C265" s="38"/>
+      <c r="D265" s="38"/>
+      <c r="E265" s="38"/>
+      <c r="F265" s="38"/>
+      <c r="G265" s="38"/>
+      <c r="H265" s="38"/>
+      <c r="I265" s="38"/>
+    </row>
+    <row r="266" spans="1:9">
+      <c r="A266" s="30">
+        <v>262</v>
+      </c>
+      <c r="B266" s="38"/>
+      <c r="C266" s="38"/>
+      <c r="D266" s="38"/>
+      <c r="E266" s="38"/>
+      <c r="F266" s="38"/>
+      <c r="G266" s="38"/>
+      <c r="H266" s="38"/>
+      <c r="I266" s="38"/>
+    </row>
+    <row r="267" spans="1:9">
+      <c r="A267" s="30">
+        <v>263</v>
+      </c>
+      <c r="B267" s="38"/>
+      <c r="C267" s="38"/>
+      <c r="D267" s="38"/>
+      <c r="E267" s="38"/>
+      <c r="F267" s="38"/>
+      <c r="G267" s="38"/>
+      <c r="H267" s="38"/>
+      <c r="I267" s="38"/>
+    </row>
+    <row r="268" spans="1:9">
+      <c r="A268" s="30">
+        <v>264</v>
+      </c>
+      <c r="B268" s="38"/>
+      <c r="C268" s="38"/>
+      <c r="D268" s="38"/>
+      <c r="E268" s="38"/>
+      <c r="F268" s="38"/>
+      <c r="G268" s="38"/>
+      <c r="H268" s="38"/>
+      <c r="I268" s="38"/>
+    </row>
+    <row r="269" spans="1:9">
+      <c r="A269" s="30">
+        <v>265</v>
+      </c>
+      <c r="B269" s="38"/>
+      <c r="C269" s="38"/>
+      <c r="D269" s="38"/>
+      <c r="E269" s="38"/>
+      <c r="F269" s="38"/>
+      <c r="G269" s="38"/>
+      <c r="H269" s="38"/>
+      <c r="I269" s="38"/>
+    </row>
+    <row r="270" spans="1:9">
+      <c r="A270" s="30">
+        <v>266</v>
+      </c>
+      <c r="B270" s="38"/>
+      <c r="C270" s="38"/>
+      <c r="D270" s="38"/>
+      <c r="E270" s="38"/>
+      <c r="F270" s="38"/>
+      <c r="G270" s="38"/>
+      <c r="H270" s="38"/>
+      <c r="I270" s="38"/>
+    </row>
+    <row r="271" spans="1:9">
+      <c r="A271" s="30">
+        <v>267</v>
+      </c>
+      <c r="B271" s="38"/>
+      <c r="C271" s="38"/>
+      <c r="D271" s="38"/>
+      <c r="E271" s="38"/>
+      <c r="F271" s="38"/>
+      <c r="G271" s="38"/>
+      <c r="H271" s="38"/>
+      <c r="I271" s="38"/>
+    </row>
+    <row r="272" spans="1:9">
+      <c r="A272" s="30">
+        <v>268</v>
+      </c>
+      <c r="B272" s="38"/>
+      <c r="C272" s="38"/>
+      <c r="D272" s="38"/>
+      <c r="E272" s="38"/>
+      <c r="F272" s="38"/>
+      <c r="G272" s="38"/>
+      <c r="H272" s="38"/>
+      <c r="I272" s="38"/>
+    </row>
+    <row r="273" spans="1:9">
+      <c r="A273" s="30">
+        <v>269</v>
+      </c>
+      <c r="B273" s="38"/>
+      <c r="C273" s="38"/>
+      <c r="D273" s="38"/>
+      <c r="E273" s="38"/>
+      <c r="F273" s="38"/>
+      <c r="G273" s="38"/>
+      <c r="H273" s="38"/>
+      <c r="I273" s="38"/>
+    </row>
+    <row r="274" spans="1:9">
+      <c r="A274" s="30">
+        <v>270</v>
+      </c>
+      <c r="B274" s="38"/>
+      <c r="C274" s="38"/>
+      <c r="D274" s="38"/>
+      <c r="E274" s="38"/>
+      <c r="F274" s="38"/>
+      <c r="G274" s="38"/>
+      <c r="H274" s="38"/>
+      <c r="I274" s="38"/>
+    </row>
+    <row r="275" spans="1:9">
+      <c r="A275" s="30">
+        <v>271</v>
+      </c>
+      <c r="B275" s="38"/>
+      <c r="C275" s="38"/>
+      <c r="D275" s="38"/>
+      <c r="E275" s="38"/>
+      <c r="F275" s="38"/>
+      <c r="G275" s="38"/>
+      <c r="H275" s="38"/>
+      <c r="I275" s="38"/>
+    </row>
+    <row r="276" spans="1:9">
+      <c r="A276" s="30">
+        <v>272</v>
+      </c>
+      <c r="B276" s="38"/>
+      <c r="C276" s="38"/>
+      <c r="D276" s="38"/>
+      <c r="E276" s="38"/>
+      <c r="F276" s="38"/>
+      <c r="G276" s="38"/>
+      <c r="H276" s="38"/>
+      <c r="I276" s="38"/>
+    </row>
+    <row r="277" spans="1:9">
+      <c r="A277" s="30">
+        <v>273</v>
+      </c>
+      <c r="B277" s="38"/>
+      <c r="C277" s="38"/>
+      <c r="D277" s="38"/>
+      <c r="E277" s="38"/>
+      <c r="F277" s="38"/>
+      <c r="G277" s="38"/>
+      <c r="H277" s="38"/>
+      <c r="I277" s="38"/>
+    </row>
+    <row r="278" spans="1:9">
+      <c r="A278" s="30">
+        <v>274</v>
+      </c>
+      <c r="B278" s="38"/>
+      <c r="C278" s="38"/>
+      <c r="D278" s="38"/>
+      <c r="E278" s="38"/>
+      <c r="F278" s="38"/>
+      <c r="G278" s="38"/>
+      <c r="H278" s="38"/>
+      <c r="I278" s="38"/>
+    </row>
+    <row r="279" spans="1:9">
+      <c r="A279" s="30">
+        <v>275</v>
+      </c>
+      <c r="B279" s="38"/>
+      <c r="C279" s="38"/>
+      <c r="D279" s="38"/>
+      <c r="E279" s="38"/>
+      <c r="F279" s="38"/>
+      <c r="G279" s="38"/>
+      <c r="H279" s="38"/>
+      <c r="I279" s="38"/>
+    </row>
+    <row r="280" spans="1:9">
+      <c r="A280" s="30">
+        <v>276</v>
+      </c>
+      <c r="B280" s="38"/>
+      <c r="C280" s="38"/>
+      <c r="D280" s="38"/>
+      <c r="E280" s="38"/>
+      <c r="F280" s="38"/>
+      <c r="G280" s="38"/>
+      <c r="H280" s="38"/>
+      <c r="I280" s="38"/>
+    </row>
+    <row r="281" spans="1:9">
+      <c r="A281" s="30">
+        <v>277</v>
+      </c>
+      <c r="B281" s="38"/>
+      <c r="C281" s="38"/>
+      <c r="D281" s="38"/>
+      <c r="E281" s="38"/>
+      <c r="F281" s="38"/>
+      <c r="G281" s="38"/>
+      <c r="H281" s="38"/>
+      <c r="I281" s="38"/>
+    </row>
+    <row r="282" spans="1:9">
+      <c r="A282" s="30">
+        <v>278</v>
+      </c>
+      <c r="B282" s="38"/>
+      <c r="C282" s="38"/>
+      <c r="D282" s="38"/>
+      <c r="E282" s="38"/>
+      <c r="F282" s="38"/>
+      <c r="G282" s="38"/>
+      <c r="H282" s="38"/>
+      <c r="I282" s="38"/>
+    </row>
+    <row r="283" spans="1:9">
+      <c r="A283" s="30">
+        <v>279</v>
+      </c>
+      <c r="B283" s="38"/>
+      <c r="C283" s="38"/>
+      <c r="D283" s="38"/>
+      <c r="E283" s="38"/>
+      <c r="F283" s="38"/>
+      <c r="G283" s="38"/>
+      <c r="H283" s="38"/>
+      <c r="I283" s="38"/>
+    </row>
+    <row r="284" spans="1:9">
+      <c r="A284" s="30">
+        <v>280</v>
+      </c>
+      <c r="B284" s="38"/>
+      <c r="C284" s="38"/>
+      <c r="D284" s="38"/>
+      <c r="E284" s="38"/>
+      <c r="F284" s="38"/>
+      <c r="G284" s="38"/>
+      <c r="H284" s="38"/>
+      <c r="I284" s="38"/>
+    </row>
+    <row r="285" spans="1:9">
+      <c r="A285" s="30">
+        <v>281</v>
+      </c>
+      <c r="B285" s="38"/>
+      <c r="C285" s="38"/>
+      <c r="D285" s="38"/>
+      <c r="E285" s="38"/>
+      <c r="F285" s="38"/>
+      <c r="G285" s="38"/>
+      <c r="H285" s="38"/>
+      <c r="I285" s="38"/>
+    </row>
+    <row r="286" spans="1:9">
+      <c r="A286" s="30">
+        <v>282</v>
+      </c>
+      <c r="B286" s="38"/>
+      <c r="C286" s="38"/>
+      <c r="D286" s="38"/>
+      <c r="E286" s="38"/>
+      <c r="F286" s="38"/>
+      <c r="G286" s="38"/>
+      <c r="H286" s="38"/>
+      <c r="I286" s="38"/>
+    </row>
+    <row r="287" spans="1:9">
+      <c r="A287" s="30">
+        <v>283</v>
+      </c>
+      <c r="B287" s="38"/>
+      <c r="C287" s="38"/>
+      <c r="D287" s="38"/>
+      <c r="E287" s="38"/>
+      <c r="F287" s="38"/>
+      <c r="G287" s="38"/>
+      <c r="H287" s="38"/>
+      <c r="I287" s="38"/>
+    </row>
+    <row r="288" spans="1:9">
+      <c r="A288" s="30">
+        <v>284</v>
+      </c>
+      <c r="B288" s="38"/>
+      <c r="C288" s="38"/>
+      <c r="D288" s="38"/>
+      <c r="E288" s="38"/>
+      <c r="F288" s="38"/>
+      <c r="G288" s="38"/>
+      <c r="H288" s="38"/>
+      <c r="I288" s="38"/>
+    </row>
+    <row r="289" spans="1:9">
+      <c r="A289" s="30">
+        <v>285</v>
+      </c>
+      <c r="B289" s="38"/>
+      <c r="C289" s="38"/>
+      <c r="D289" s="38"/>
+      <c r="E289" s="38"/>
+      <c r="F289" s="38"/>
+      <c r="G289" s="38"/>
+      <c r="H289" s="38"/>
+      <c r="I289" s="38"/>
+    </row>
+    <row r="290" spans="1:9">
+      <c r="A290" s="30">
+        <v>286</v>
+      </c>
+      <c r="B290" s="38"/>
+      <c r="C290" s="38"/>
+      <c r="D290" s="38"/>
+      <c r="E290" s="38"/>
+      <c r="F290" s="38"/>
+      <c r="G290" s="38"/>
+      <c r="H290" s="38"/>
+      <c r="I290" s="38"/>
+    </row>
+    <row r="291" spans="1:9">
+      <c r="A291" s="30">
+        <v>287</v>
+      </c>
+      <c r="B291" s="38"/>
+      <c r="C291" s="38"/>
+      <c r="D291" s="38"/>
+      <c r="E291" s="38"/>
+      <c r="F291" s="38"/>
+      <c r="G291" s="38"/>
+      <c r="H291" s="38"/>
+      <c r="I291" s="38"/>
+    </row>
+    <row r="292" spans="1:9">
+      <c r="A292" s="30">
+        <v>288</v>
+      </c>
+      <c r="B292" s="38"/>
+      <c r="C292" s="38"/>
+      <c r="D292" s="38"/>
+      <c r="E292" s="38"/>
+      <c r="F292" s="38"/>
+      <c r="G292" s="38"/>
+      <c r="H292" s="38"/>
+      <c r="I292" s="38"/>
+    </row>
+    <row r="293" spans="1:9">
+      <c r="A293" s="30">
+        <v>289</v>
+      </c>
+      <c r="B293" s="38"/>
+      <c r="C293" s="38"/>
+      <c r="D293" s="38"/>
+      <c r="E293" s="38"/>
+      <c r="F293" s="38"/>
+      <c r="G293" s="38"/>
+      <c r="H293" s="38"/>
+      <c r="I293" s="38"/>
+    </row>
+    <row r="294" spans="1:9">
+      <c r="A294" s="30">
+        <v>290</v>
+      </c>
+      <c r="B294" s="38"/>
+      <c r="C294" s="38"/>
+      <c r="D294" s="38"/>
+      <c r="E294" s="38"/>
+      <c r="F294" s="38"/>
+      <c r="G294" s="38"/>
+      <c r="H294" s="38"/>
+      <c r="I294" s="38"/>
+    </row>
+    <row r="295" spans="1:9">
+      <c r="A295" s="30">
+        <v>291</v>
+      </c>
+      <c r="B295" s="38"/>
+      <c r="C295" s="38"/>
+      <c r="D295" s="38"/>
+      <c r="E295" s="38"/>
+      <c r="F295" s="38"/>
+      <c r="G295" s="38"/>
+      <c r="H295" s="38"/>
+      <c r="I295" s="38"/>
+    </row>
+    <row r="296" spans="1:9">
+      <c r="A296" s="30">
+        <v>292</v>
+      </c>
+      <c r="B296" s="38"/>
+      <c r="C296" s="38"/>
+      <c r="D296" s="38"/>
+      <c r="E296" s="38"/>
+      <c r="F296" s="38"/>
+      <c r="G296" s="38"/>
+      <c r="H296" s="38"/>
+      <c r="I296" s="38"/>
+    </row>
+    <row r="297" spans="1:9">
+      <c r="A297" s="30">
+        <v>293</v>
+      </c>
+      <c r="B297" s="38"/>
+      <c r="C297" s="38"/>
+      <c r="D297" s="38"/>
+      <c r="E297" s="38"/>
+      <c r="F297" s="38"/>
+      <c r="G297" s="38"/>
+      <c r="H297" s="38"/>
+      <c r="I297" s="38"/>
+    </row>
+    <row r="298" spans="1:9">
+      <c r="A298" s="30">
+        <v>294</v>
+      </c>
+      <c r="B298" s="38"/>
+      <c r="C298" s="38"/>
+      <c r="D298" s="38"/>
+      <c r="E298" s="38"/>
+      <c r="F298" s="38"/>
+      <c r="G298" s="38"/>
+      <c r="H298" s="38"/>
+      <c r="I298" s="38"/>
+    </row>
+    <row r="299" spans="1:9">
+      <c r="A299" s="30">
+        <v>295</v>
+      </c>
+      <c r="B299" s="38"/>
+      <c r="C299" s="38"/>
+      <c r="D299" s="38"/>
+      <c r="E299" s="38"/>
+      <c r="F299" s="38"/>
+      <c r="G299" s="38"/>
+      <c r="H299" s="38"/>
+      <c r="I299" s="38"/>
+    </row>
+    <row r="300" spans="1:9">
+      <c r="A300" s="30">
+        <v>296</v>
+      </c>
+      <c r="B300" s="38"/>
+      <c r="C300" s="38"/>
+      <c r="D300" s="38"/>
+      <c r="E300" s="38"/>
+      <c r="F300" s="38"/>
+      <c r="G300" s="38"/>
+      <c r="H300" s="38"/>
+      <c r="I300" s="38"/>
+    </row>
+    <row r="301" spans="1:9">
+      <c r="A301" s="30">
+        <v>297</v>
+      </c>
+      <c r="B301" s="38"/>
+      <c r="C301" s="38"/>
+      <c r="D301" s="38"/>
+      <c r="E301" s="38"/>
+      <c r="F301" s="38"/>
+      <c r="G301" s="38"/>
+      <c r="H301" s="38"/>
+      <c r="I301" s="38"/>
+    </row>
+    <row r="302" spans="1:9">
+      <c r="A302" s="30">
+        <v>298</v>
+      </c>
+      <c r="B302" s="38"/>
+      <c r="C302" s="38"/>
+      <c r="D302" s="38"/>
+      <c r="E302" s="38"/>
+      <c r="F302" s="38"/>
+      <c r="G302" s="38"/>
+      <c r="H302" s="38"/>
+      <c r="I302" s="38"/>
+    </row>
+    <row r="303" spans="1:9">
+      <c r="A303" s="30">
+        <v>299</v>
+      </c>
+      <c r="B303" s="38"/>
+      <c r="C303" s="38"/>
+      <c r="D303" s="38"/>
+      <c r="E303" s="38"/>
+      <c r="F303" s="38"/>
+      <c r="G303" s="38"/>
+      <c r="H303" s="38"/>
+      <c r="I303" s="38"/>
+    </row>
+    <row r="304" spans="1:9">
+      <c r="A304" s="30">
+        <v>300</v>
+      </c>
+      <c r="B304" s="38"/>
+      <c r="C304" s="38"/>
+      <c r="D304" s="38"/>
+      <c r="E304" s="38"/>
+      <c r="F304" s="38"/>
+      <c r="G304" s="38"/>
+      <c r="H304" s="38"/>
+      <c r="I304" s="38"/>
+    </row>
+  </sheetData>
+  <mergeCells count="2">
+    <mergeCell ref="A1:I1"/>
+    <mergeCell ref="A2:I2"/>
+  </mergeCells>
+  <dataValidations count="3">
+    <dataValidation type="list" allowBlank="1" sqref="D5:D304">
+      <formula1>"بكالوريوس علوم الحاسب,بكالوريوس علوم البيانات,ماجستير علوم البيانات,مشترك للبرامج الثلاثة"</formula1>
+    </dataValidation>
+    <dataValidation type="list" allowBlank="1" sqref="G5:G304">
+      <formula1>'الإعدادات واللجنة'!$B$12:$B$20</formula1>
+    </dataValidation>
+    <dataValidation type="date" operator="greaterThan" allowBlank="1" showErrorMessage="1" error="اكتب تاريخاً صحيحاً" sqref="H5:H304">
+      <formula1>45000</formula1>
+    </dataValidation>
+  </dataValidations>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
+</file>
+
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{9D5F76BD-1E17-DC4F-93F9-7A03DF44BB80}">
   <dimension ref="A1:F32"/>

</xml_diff>

<commit_message>
Quality documents: split course and field-training reports by semester
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Gat5tVsr5NWC6rDktNbfy6
</commit_message>
<xml_diff>
--- a/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
+++ b/خطة_الاعتماد_البرامجي_المرحلة_الأولى.xlsx
@@ -4030,11 +4030,11 @@
   <sheetPr>
     <tabColor rgb="FFC00000"/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H75"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="40" customWidth="1"/>
-    <col min="2" max="2" width="13" customWidth="1"/>
+    <col min="2" max="2" width="24" customWidth="1"/>
     <col min="3" max="4" width="10" customWidth="1"/>
     <col min="5" max="5" width="10" customWidth="1"/>
     <col min="6" max="6" width="14" customWidth="1"/>
@@ -4051,7 +4051,7 @@
     <row r="2" spans="1:8" ht="44" customHeight="1">
       <c r="A2" s="99" t="inlineStr">
         <is>
-          <t xml:space="preserve">اكتبي في «المطلوب» عدد الوثائق المطلوبة (مثل عدد المقررات)، وفي «تم» عدد المنجز منها، وضعي الرابط. اكتبي 0 في «المطلوب» إذا كانت الوثيقة لا تنطبق على البرنامج. النسبة والحالة تُحسبان تلقائياً.</t>
+          <t xml:space="preserve">اكتبي في «المطلوب» عدد الوثائق المطلوبة (مثل عدد المقررات في الفصل)، وفي «تم» عدد المنجز منها، وضعي الرابط. اكتبي 0 في «المطلوب» إذا كانت الوثيقة لا تنطبق على البرنامج. النسبة والحالة تُحسبان تلقائياً.</t>
         </is>
       </c>
     </row>
@@ -4065,7 +4065,7 @@
       <c r="C3" s="29"/>
       <c r="D3" s="29"/>
       <c r="E3" s="35">
-        <f>IFERROR(AVERAGE(E23,E43,E63),0)</f>
+        <f>IFERROR(AVERAGE(E27,E51,E75),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -4090,7 +4090,7 @@
       </c>
       <c r="B6" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">العام</t>
+          <t xml:space="preserve">العام / الفصل</t>
         </is>
       </c>
       <c r="C6" s="29" t="inlineStr">
@@ -4310,7 +4310,7 @@
       </c>
       <c r="B14" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-2025</t>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
         </is>
       </c>
       <c r="C14" s="38"/>
@@ -4334,7 +4334,7 @@
       </c>
       <c r="B15" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-2026</t>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
         </is>
       </c>
       <c r="C15" s="38"/>
@@ -4353,12 +4353,12 @@
     <row r="16" spans="1:8" ht="24" customHeight="1">
       <c r="A16" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
         </is>
       </c>
       <c r="B16" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-2025</t>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
         </is>
       </c>
       <c r="C16" s="38"/>
@@ -4377,12 +4377,12 @@
     <row r="17" spans="1:8" ht="24" customHeight="1">
       <c r="A17" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
         </is>
       </c>
       <c r="B17" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-2026</t>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
         </is>
       </c>
       <c r="C17" s="38"/>
@@ -4401,306 +4401,302 @@
     <row r="18" spans="1:8" ht="24" customHeight="1">
       <c r="A18" s="31" t="inlineStr">
         <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B18" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C18" s="38"/>
+      <c r="D18" s="38"/>
+      <c r="E18" s="35">
+        <f>IF(OR(C18="",C18=0),"",MIN(N(D18)/C18,1))</f>
+        <v/>
+      </c>
+      <c r="F18" s="30" t="str">
+        <f>IF(C18="","لم يُحدد",IF(C18=0,"لا ينطبق",IF(N(D18)&gt;=C18,"مكتمل",IF(N(D18)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G18" s="38"/>
+      <c r="H18" s="38"/>
+    </row>
+    <row r="19" spans="1:8" ht="24" customHeight="1">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B19" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C19" s="38"/>
+      <c r="D19" s="38"/>
+      <c r="E19" s="35">
+        <f>IF(OR(C19="",C19=0),"",MIN(N(D19)/C19,1))</f>
+        <v/>
+      </c>
+      <c r="F19" s="30" t="str">
+        <f>IF(C19="","لم يُحدد",IF(C19=0,"لا ينطبق",IF(N(D19)&gt;=C19,"مكتمل",IF(N(D19)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G19" s="38"/>
+      <c r="H19" s="38"/>
+    </row>
+    <row r="20" spans="1:8" ht="24" customHeight="1">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B20" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C20" s="38"/>
+      <c r="D20" s="38"/>
+      <c r="E20" s="35">
+        <f>IF(OR(C20="",C20=0),"",MIN(N(D20)/C20,1))</f>
+        <v/>
+      </c>
+      <c r="F20" s="30" t="str">
+        <f>IF(C20="","لم يُحدد",IF(C20=0,"لا ينطبق",IF(N(D20)&gt;=C20,"مكتمل",IF(N(D20)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G20" s="38"/>
+      <c r="H20" s="38"/>
+    </row>
+    <row r="21" spans="1:8" ht="24" customHeight="1">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B21" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C21" s="38"/>
+      <c r="D21" s="38"/>
+      <c r="E21" s="35">
+        <f>IF(OR(C21="",C21=0),"",MIN(N(D21)/C21,1))</f>
+        <v/>
+      </c>
+      <c r="F21" s="30" t="str">
+        <f>IF(C21="","لم يُحدد",IF(C21=0,"لا ينطبق",IF(N(D21)&gt;=C21,"مكتمل",IF(N(D21)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G21" s="38"/>
+      <c r="H21" s="38"/>
+    </row>
+    <row r="22" spans="1:8" ht="24" customHeight="1">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
           <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
         </is>
       </c>
-      <c r="B18" s="30" t="inlineStr">
+      <c r="B22" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C18" s="38">
+      <c r="C22" s="38">
         <v>1</v>
       </c>
-      <c r="D18" s="38"/>
-      <c r="E18" s="35">
-        <f>IF(OR(C18="",C18=0),"",MIN(N(D18)/C18,1))</f>
-        <v/>
-      </c>
-      <c r="F18" s="30" t="str">
-        <f>IF(C18="","لم يُحدد",IF(C18=0,"لا ينطبق",IF(N(D18)&gt;=C18,"مكتمل",IF(N(D18)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G18" s="38"/>
-      <c r="H18" s="38"/>
-    </row>
-    <row r="19" spans="1:8" ht="24" customHeight="1">
-      <c r="A19" s="31" t="inlineStr">
+      <c r="D22" s="38"/>
+      <c r="E22" s="35">
+        <f>IF(OR(C22="",C22=0),"",MIN(N(D22)/C22,1))</f>
+        <v/>
+      </c>
+      <c r="F22" s="30" t="str">
+        <f>IF(C22="","لم يُحدد",IF(C22=0,"لا ينطبق",IF(N(D22)&gt;=C22,"مكتمل",IF(N(D22)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G22" s="38"/>
+      <c r="H22" s="38"/>
+    </row>
+    <row r="23" spans="1:8" ht="24" customHeight="1">
+      <c r="A23" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
         </is>
       </c>
-      <c r="B19" s="30" t="inlineStr">
+      <c r="B23" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C19" s="38">
+      <c r="C23" s="38">
         <v>1</v>
       </c>
-      <c r="D19" s="38"/>
-      <c r="E19" s="35">
-        <f>IF(OR(C19="",C19=0),"",MIN(N(D19)/C19,1))</f>
-        <v/>
-      </c>
-      <c r="F19" s="30" t="str">
-        <f>IF(C19="","لم يُحدد",IF(C19=0,"لا ينطبق",IF(N(D19)&gt;=C19,"مكتمل",IF(N(D19)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G19" s="38"/>
-      <c r="H19" s="38"/>
-    </row>
-    <row r="20" spans="1:8" ht="24" customHeight="1">
-      <c r="A20" s="31" t="inlineStr">
+      <c r="D23" s="38"/>
+      <c r="E23" s="35">
+        <f>IF(OR(C23="",C23=0),"",MIN(N(D23)/C23,1))</f>
+        <v/>
+      </c>
+      <c r="F23" s="30" t="str">
+        <f>IF(C23="","لم يُحدد",IF(C23=0,"لا ينطبق",IF(N(D23)&gt;=C23,"مكتمل",IF(N(D23)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G23" s="38"/>
+      <c r="H23" s="38"/>
+    </row>
+    <row r="24" spans="1:8" ht="24" customHeight="1">
+      <c r="A24" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B20" s="30" t="inlineStr">
+      <c r="B24" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2023-2024</t>
         </is>
       </c>
-      <c r="C20" s="38">
+      <c r="C24" s="38">
         <v>1</v>
       </c>
-      <c r="D20" s="38"/>
-      <c r="E20" s="35">
-        <f>IF(OR(C20="",C20=0),"",MIN(N(D20)/C20,1))</f>
-        <v/>
-      </c>
-      <c r="F20" s="30" t="str">
-        <f>IF(C20="","لم يُحدد",IF(C20=0,"لا ينطبق",IF(N(D20)&gt;=C20,"مكتمل",IF(N(D20)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G20" s="38"/>
-      <c r="H20" s="38"/>
-    </row>
-    <row r="21" spans="1:8" ht="24" customHeight="1">
-      <c r="A21" s="31" t="inlineStr">
+      <c r="D24" s="38"/>
+      <c r="E24" s="35">
+        <f>IF(OR(C24="",C24=0),"",MIN(N(D24)/C24,1))</f>
+        <v/>
+      </c>
+      <c r="F24" s="30" t="str">
+        <f>IF(C24="","لم يُحدد",IF(C24=0,"لا ينطبق",IF(N(D24)&gt;=C24,"مكتمل",IF(N(D24)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G24" s="38"/>
+      <c r="H24" s="38"/>
+    </row>
+    <row r="25" spans="1:8" ht="24" customHeight="1">
+      <c r="A25" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B21" s="30" t="inlineStr">
+      <c r="B25" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C21" s="38">
+      <c r="C25" s="38">
         <v>1</v>
       </c>
-      <c r="D21" s="38"/>
-      <c r="E21" s="35">
-        <f>IF(OR(C21="",C21=0),"",MIN(N(D21)/C21,1))</f>
-        <v/>
-      </c>
-      <c r="F21" s="30" t="str">
-        <f>IF(C21="","لم يُحدد",IF(C21=0,"لا ينطبق",IF(N(D21)&gt;=C21,"مكتمل",IF(N(D21)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G21" s="38"/>
-      <c r="H21" s="38"/>
-    </row>
-    <row r="22" spans="1:8" ht="24" customHeight="1">
-      <c r="A22" s="31" t="inlineStr">
+      <c r="D25" s="38"/>
+      <c r="E25" s="35">
+        <f>IF(OR(C25="",C25=0),"",MIN(N(D25)/C25,1))</f>
+        <v/>
+      </c>
+      <c r="F25" s="30" t="str">
+        <f>IF(C25="","لم يُحدد",IF(C25=0,"لا ينطبق",IF(N(D25)&gt;=C25,"مكتمل",IF(N(D25)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G25" s="38"/>
+      <c r="H25" s="38"/>
+    </row>
+    <row r="26" spans="1:8" ht="24" customHeight="1">
+      <c r="A26" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B22" s="30" t="inlineStr">
+      <c r="B26" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C22" s="38">
+      <c r="C26" s="38">
         <v>1</v>
       </c>
-      <c r="D22" s="38"/>
-      <c r="E22" s="35">
-        <f>IF(OR(C22="",C22=0),"",MIN(N(D22)/C22,1))</f>
-        <v/>
-      </c>
-      <c r="F22" s="30" t="str">
-        <f>IF(C22="","لم يُحدد",IF(C22=0,"لا ينطبق",IF(N(D22)&gt;=C22,"مكتمل",IF(N(D22)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G22" s="38"/>
-      <c r="H22" s="38"/>
-    </row>
-    <row r="23" spans="1:8" ht="26" customHeight="1">
-      <c r="A23" s="29" t="inlineStr">
+      <c r="D26" s="38"/>
+      <c r="E26" s="35">
+        <f>IF(OR(C26="",C26=0),"",MIN(N(D26)/C26,1))</f>
+        <v/>
+      </c>
+      <c r="F26" s="30" t="str">
+        <f>IF(C26="","لم يُحدد",IF(C26=0,"لا ينطبق",IF(N(D26)&gt;=C26,"مكتمل",IF(N(D26)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G26" s="38"/>
+      <c r="H26" s="38"/>
+    </row>
+    <row r="27" spans="1:8" ht="26" customHeight="1">
+      <c r="A27" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">نسبة إنجاز البرنامج</t>
         </is>
       </c>
-      <c r="B23" s="29"/>
-      <c r="C23" s="29"/>
-      <c r="D23" s="29"/>
-      <c r="E23" s="35">
-        <f>IFERROR(AVERAGE(E7:E22),0)</f>
+      <c r="B27" s="29"/>
+      <c r="C27" s="29"/>
+      <c r="D27" s="29"/>
+      <c r="E27" s="35">
+        <f>IFERROR(AVERAGE(E7:E26),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="25" spans="1:8" ht="26" customHeight="1">
-      <c r="A25" s="97" t="str">
+    <row r="29" spans="1:8" ht="26" customHeight="1">
+      <c r="A29" s="97" t="str">
         <f>'الإعدادات واللجنة'!$B$6</f>
         <v/>
       </c>
-      <c r="B25" s="97"/>
-      <c r="C25" s="97"/>
-      <c r="D25" s="97"/>
-      <c r="E25" s="97"/>
-      <c r="F25" s="97"/>
-      <c r="G25" s="97"/>
-      <c r="H25" s="97"/>
-    </row>
-    <row r="26" spans="1:8" ht="28" customHeight="1">
-      <c r="A26" s="29" t="inlineStr">
+      <c r="B29" s="97"/>
+      <c r="C29" s="97"/>
+      <c r="D29" s="97"/>
+      <c r="E29" s="97"/>
+      <c r="F29" s="97"/>
+      <c r="G29" s="97"/>
+      <c r="H29" s="97"/>
+    </row>
+    <row r="30" spans="1:8" ht="28" customHeight="1">
+      <c r="A30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">الوثيقة</t>
         </is>
       </c>
-      <c r="B26" s="29" t="inlineStr">
+      <c r="B30" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">العام</t>
+          <t xml:space="preserve">العام / الفصل</t>
         </is>
       </c>
-      <c r="C26" s="29" t="inlineStr">
+      <c r="C30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">المطلوب</t>
         </is>
       </c>
-      <c r="D26" s="29" t="inlineStr">
+      <c r="D30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">تم</t>
         </is>
       </c>
-      <c r="E26" s="29" t="inlineStr">
+      <c r="E30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">النسبة</t>
         </is>
       </c>
-      <c r="F26" s="29" t="inlineStr">
+      <c r="F30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">الحالة</t>
         </is>
       </c>
-      <c r="G26" s="29" t="inlineStr">
+      <c r="G30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">رابط الوثيقة</t>
         </is>
       </c>
-      <c r="H26" s="29" t="inlineStr">
+      <c r="H30" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">ملاحظات</t>
         </is>
       </c>
     </row>
-    <row r="27" spans="1:8" ht="24" customHeight="1">
-      <c r="A27" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">توصيف البرنامج (TP-151)</t>
-        </is>
-      </c>
-      <c r="B27" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C27" s="38">
-        <v>1</v>
-      </c>
-      <c r="D27" s="38"/>
-      <c r="E27" s="35">
-        <f>IF(OR(C27="",C27=0),"",MIN(N(D27)/C27,1))</f>
-        <v/>
-      </c>
-      <c r="F27" s="30" t="str">
-        <f>IF(C27="","لم يُحدد",IF(C27=0,"لا ينطبق",IF(N(D27)&gt;=C27,"مكتمل",IF(N(D27)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G27" s="38"/>
-      <c r="H27" s="38"/>
-    </row>
-    <row r="28" spans="1:8" ht="24" customHeight="1">
-      <c r="A28" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">توصيفات المقررات (TP-153)</t>
-        </is>
-      </c>
-      <c r="B28" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C28" s="38"/>
-      <c r="D28" s="38"/>
-      <c r="E28" s="35">
-        <f>IF(OR(C28="",C28=0),"",MIN(N(D28)/C28,1))</f>
-        <v/>
-      </c>
-      <c r="F28" s="30" t="str">
-        <f>IF(C28="","لم يُحدد",IF(C28=0,"لا ينطبق",IF(N(D28)&gt;=C28,"مكتمل",IF(N(D28)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G28" s="38"/>
-      <c r="H28" s="38"/>
-    </row>
-    <row r="29" spans="1:8" ht="24" customHeight="1">
-      <c r="A29" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">توصيف التدريب العملي (TP-155)</t>
-        </is>
-      </c>
-      <c r="B29" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C29" s="38"/>
-      <c r="D29" s="38"/>
-      <c r="E29" s="35">
-        <f>IF(OR(C29="",C29=0),"",MIN(N(D29)/C29,1))</f>
-        <v/>
-      </c>
-      <c r="F29" s="30" t="str">
-        <f>IF(C29="","لم يُحدد",IF(C29=0,"لا ينطبق",IF(N(D29)&gt;=C29,"مكتمل",IF(N(D29)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G29" s="38"/>
-      <c r="H29" s="38"/>
-    </row>
-    <row r="30" spans="1:8" ht="24" customHeight="1">
-      <c r="A30" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تقرير الاتساق مع الإطار الوطني (TP-150)</t>
-        </is>
-      </c>
-      <c r="B30" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C30" s="38">
-        <v>1</v>
-      </c>
-      <c r="D30" s="38"/>
-      <c r="E30" s="35">
-        <f>IF(OR(C30="",C30=0),"",MIN(N(D30)/C30,1))</f>
-        <v/>
-      </c>
-      <c r="F30" s="30" t="str">
-        <f>IF(C30="","لم يُحدد",IF(C30=0,"لا ينطبق",IF(N(D30)&gt;=C30,"مكتمل",IF(N(D30)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G30" s="38"/>
-      <c r="H30" s="38"/>
-    </row>
     <row r="31" spans="1:8" ht="24" customHeight="1">
       <c r="A31" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">خطة تقييم نواتج التعلم</t>
+          <t xml:space="preserve">توصيف البرنامج (TP-151)</t>
         </is>
       </c>
       <c r="B31" s="30" t="inlineStr">
@@ -4726,17 +4722,15 @@
     <row r="32" spans="1:8" ht="24" customHeight="1">
       <c r="A32" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
+          <t xml:space="preserve">توصيفات المقررات (TP-153)</t>
         </is>
       </c>
       <c r="B32" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-2025</t>
+          <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
-      <c r="C32" s="38">
-        <v>1</v>
-      </c>
+      <c r="C32" s="38"/>
       <c r="D32" s="38"/>
       <c r="E32" s="35">
         <f>IF(OR(C32="",C32=0),"",MIN(N(D32)/C32,1))</f>
@@ -4752,17 +4746,15 @@
     <row r="33" spans="1:8" ht="24" customHeight="1">
       <c r="A33" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
+          <t xml:space="preserve">توصيف التدريب العملي (TP-155)</t>
         </is>
       </c>
       <c r="B33" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-2026</t>
+          <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
-      <c r="C33" s="38">
-        <v>1</v>
-      </c>
+      <c r="C33" s="38"/>
       <c r="D33" s="38"/>
       <c r="E33" s="35">
         <f>IF(OR(C33="",C33=0),"",MIN(N(D33)/C33,1))</f>
@@ -4778,15 +4770,17 @@
     <row r="34" spans="1:8" ht="24" customHeight="1">
       <c r="A34" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+          <t xml:space="preserve">تقرير الاتساق مع الإطار الوطني (TP-150)</t>
         </is>
       </c>
       <c r="B34" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2024-2025</t>
+          <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
-      <c r="C34" s="38"/>
+      <c r="C34" s="38">
+        <v>1</v>
+      </c>
       <c r="D34" s="38"/>
       <c r="E34" s="35">
         <f>IF(OR(C34="",C34=0),"",MIN(N(D34)/C34,1))</f>
@@ -4802,15 +4796,17 @@
     <row r="35" spans="1:8" ht="24" customHeight="1">
       <c r="A35" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+          <t xml:space="preserve">خطة تقييم نواتج التعلم</t>
         </is>
       </c>
       <c r="B35" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-2026</t>
+          <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
-      <c r="C35" s="38"/>
+      <c r="C35" s="38">
+        <v>1</v>
+      </c>
       <c r="D35" s="38"/>
       <c r="E35" s="35">
         <f>IF(OR(C35="",C35=0),"",MIN(N(D35)/C35,1))</f>
@@ -4826,7 +4822,7 @@
     <row r="36" spans="1:8" ht="24" customHeight="1">
       <c r="A36" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
         </is>
       </c>
       <c r="B36" s="30" t="inlineStr">
@@ -4834,7 +4830,9 @@
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C36" s="38"/>
+      <c r="C36" s="38">
+        <v>1</v>
+      </c>
       <c r="D36" s="38"/>
       <c r="E36" s="35">
         <f>IF(OR(C36="",C36=0),"",MIN(N(D36)/C36,1))</f>
@@ -4850,7 +4848,7 @@
     <row r="37" spans="1:8" ht="24" customHeight="1">
       <c r="A37" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
         </is>
       </c>
       <c r="B37" s="30" t="inlineStr">
@@ -4858,7 +4856,9 @@
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C37" s="38"/>
+      <c r="C37" s="38">
+        <v>1</v>
+      </c>
       <c r="D37" s="38"/>
       <c r="E37" s="35">
         <f>IF(OR(C37="",C37=0),"",MIN(N(D37)/C37,1))</f>
@@ -4874,437 +4874,429 @@
     <row r="38" spans="1:8" ht="24" customHeight="1">
       <c r="A38" s="31" t="inlineStr">
         <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B38" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C38" s="38"/>
+      <c r="D38" s="38"/>
+      <c r="E38" s="35">
+        <f>IF(OR(C38="",C38=0),"",MIN(N(D38)/C38,1))</f>
+        <v/>
+      </c>
+      <c r="F38" s="30" t="str">
+        <f>IF(C38="","لم يُحدد",IF(C38=0,"لا ينطبق",IF(N(D38)&gt;=C38,"مكتمل",IF(N(D38)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G38" s="38"/>
+      <c r="H38" s="38"/>
+    </row>
+    <row r="39" spans="1:8" ht="24" customHeight="1">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B39" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C39" s="38"/>
+      <c r="D39" s="38"/>
+      <c r="E39" s="35">
+        <f>IF(OR(C39="",C39=0),"",MIN(N(D39)/C39,1))</f>
+        <v/>
+      </c>
+      <c r="F39" s="30" t="str">
+        <f>IF(C39="","لم يُحدد",IF(C39=0,"لا ينطبق",IF(N(D39)&gt;=C39,"مكتمل",IF(N(D39)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G39" s="38"/>
+      <c r="H39" s="38"/>
+    </row>
+    <row r="40" spans="1:8" ht="24" customHeight="1">
+      <c r="A40" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B40" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C40" s="38"/>
+      <c r="D40" s="38"/>
+      <c r="E40" s="35">
+        <f>IF(OR(C40="",C40=0),"",MIN(N(D40)/C40,1))</f>
+        <v/>
+      </c>
+      <c r="F40" s="30" t="str">
+        <f>IF(C40="","لم يُحدد",IF(C40=0,"لا ينطبق",IF(N(D40)&gt;=C40,"مكتمل",IF(N(D40)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G40" s="38"/>
+      <c r="H40" s="38"/>
+    </row>
+    <row r="41" spans="1:8" ht="24" customHeight="1">
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B41" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C41" s="38"/>
+      <c r="D41" s="38"/>
+      <c r="E41" s="35">
+        <f>IF(OR(C41="",C41=0),"",MIN(N(D41)/C41,1))</f>
+        <v/>
+      </c>
+      <c r="F41" s="30" t="str">
+        <f>IF(C41="","لم يُحدد",IF(C41=0,"لا ينطبق",IF(N(D41)&gt;=C41,"مكتمل",IF(N(D41)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G41" s="38"/>
+      <c r="H41" s="38"/>
+    </row>
+    <row r="42" spans="1:8" ht="24" customHeight="1">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B42" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C42" s="38"/>
+      <c r="D42" s="38"/>
+      <c r="E42" s="35">
+        <f>IF(OR(C42="",C42=0),"",MIN(N(D42)/C42,1))</f>
+        <v/>
+      </c>
+      <c r="F42" s="30" t="str">
+        <f>IF(C42="","لم يُحدد",IF(C42=0,"لا ينطبق",IF(N(D42)&gt;=C42,"مكتمل",IF(N(D42)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G42" s="38"/>
+      <c r="H42" s="38"/>
+    </row>
+    <row r="43" spans="1:8" ht="24" customHeight="1">
+      <c r="A43" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B43" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C43" s="38"/>
+      <c r="D43" s="38"/>
+      <c r="E43" s="35">
+        <f>IF(OR(C43="",C43=0),"",MIN(N(D43)/C43,1))</f>
+        <v/>
+      </c>
+      <c r="F43" s="30" t="str">
+        <f>IF(C43="","لم يُحدد",IF(C43=0,"لا ينطبق",IF(N(D43)&gt;=C43,"مكتمل",IF(N(D43)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G43" s="38"/>
+      <c r="H43" s="38"/>
+    </row>
+    <row r="44" spans="1:8" ht="24" customHeight="1">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B44" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C44" s="38"/>
+      <c r="D44" s="38"/>
+      <c r="E44" s="35">
+        <f>IF(OR(C44="",C44=0),"",MIN(N(D44)/C44,1))</f>
+        <v/>
+      </c>
+      <c r="F44" s="30" t="str">
+        <f>IF(C44="","لم يُحدد",IF(C44=0,"لا ينطبق",IF(N(D44)&gt;=C44,"مكتمل",IF(N(D44)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G44" s="38"/>
+      <c r="H44" s="38"/>
+    </row>
+    <row r="45" spans="1:8" ht="24" customHeight="1">
+      <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B45" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C45" s="38"/>
+      <c r="D45" s="38"/>
+      <c r="E45" s="35">
+        <f>IF(OR(C45="",C45=0),"",MIN(N(D45)/C45,1))</f>
+        <v/>
+      </c>
+      <c r="F45" s="30" t="str">
+        <f>IF(C45="","لم يُحدد",IF(C45=0,"لا ينطبق",IF(N(D45)&gt;=C45,"مكتمل",IF(N(D45)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G45" s="38"/>
+      <c r="H45" s="38"/>
+    </row>
+    <row r="46" spans="1:8" ht="24" customHeight="1">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
           <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
         </is>
       </c>
-      <c r="B38" s="30" t="inlineStr">
+      <c r="B46" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C38" s="38">
+      <c r="C46" s="38">
         <v>1</v>
       </c>
-      <c r="D38" s="38"/>
-      <c r="E38" s="35">
-        <f>IF(OR(C38="",C38=0),"",MIN(N(D38)/C38,1))</f>
-        <v/>
-      </c>
-      <c r="F38" s="30" t="str">
-        <f>IF(C38="","لم يُحدد",IF(C38=0,"لا ينطبق",IF(N(D38)&gt;=C38,"مكتمل",IF(N(D38)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G38" s="38"/>
-      <c r="H38" s="38"/>
-    </row>
-    <row r="39" spans="1:8" ht="24" customHeight="1">
-      <c r="A39" s="31" t="inlineStr">
+      <c r="D46" s="38"/>
+      <c r="E46" s="35">
+        <f>IF(OR(C46="",C46=0),"",MIN(N(D46)/C46,1))</f>
+        <v/>
+      </c>
+      <c r="F46" s="30" t="str">
+        <f>IF(C46="","لم يُحدد",IF(C46=0,"لا ينطبق",IF(N(D46)&gt;=C46,"مكتمل",IF(N(D46)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G46" s="38"/>
+      <c r="H46" s="38"/>
+    </row>
+    <row r="47" spans="1:8" ht="24" customHeight="1">
+      <c r="A47" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
         </is>
       </c>
-      <c r="B39" s="30" t="inlineStr">
+      <c r="B47" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C39" s="38">
+      <c r="C47" s="38">
         <v>1</v>
       </c>
-      <c r="D39" s="38"/>
-      <c r="E39" s="35">
-        <f>IF(OR(C39="",C39=0),"",MIN(N(D39)/C39,1))</f>
-        <v/>
-      </c>
-      <c r="F39" s="30" t="str">
-        <f>IF(C39="","لم يُحدد",IF(C39=0,"لا ينطبق",IF(N(D39)&gt;=C39,"مكتمل",IF(N(D39)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G39" s="38"/>
-      <c r="H39" s="38"/>
-    </row>
-    <row r="40" spans="1:8" ht="24" customHeight="1">
-      <c r="A40" s="31" t="inlineStr">
+      <c r="D47" s="38"/>
+      <c r="E47" s="35">
+        <f>IF(OR(C47="",C47=0),"",MIN(N(D47)/C47,1))</f>
+        <v/>
+      </c>
+      <c r="F47" s="30" t="str">
+        <f>IF(C47="","لم يُحدد",IF(C47=0,"لا ينطبق",IF(N(D47)&gt;=C47,"مكتمل",IF(N(D47)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G47" s="38"/>
+      <c r="H47" s="38"/>
+    </row>
+    <row r="48" spans="1:8" ht="24" customHeight="1">
+      <c r="A48" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B40" s="30" t="inlineStr">
+      <c r="B48" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2023-2024</t>
         </is>
       </c>
-      <c r="C40" s="38">
+      <c r="C48" s="38">
         <v>1</v>
       </c>
-      <c r="D40" s="38"/>
-      <c r="E40" s="35">
-        <f>IF(OR(C40="",C40=0),"",MIN(N(D40)/C40,1))</f>
-        <v/>
-      </c>
-      <c r="F40" s="30" t="str">
-        <f>IF(C40="","لم يُحدد",IF(C40=0,"لا ينطبق",IF(N(D40)&gt;=C40,"مكتمل",IF(N(D40)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G40" s="38"/>
-      <c r="H40" s="38"/>
-    </row>
-    <row r="41" spans="1:8" ht="24" customHeight="1">
-      <c r="A41" s="31" t="inlineStr">
+      <c r="D48" s="38"/>
+      <c r="E48" s="35">
+        <f>IF(OR(C48="",C48=0),"",MIN(N(D48)/C48,1))</f>
+        <v/>
+      </c>
+      <c r="F48" s="30" t="str">
+        <f>IF(C48="","لم يُحدد",IF(C48=0,"لا ينطبق",IF(N(D48)&gt;=C48,"مكتمل",IF(N(D48)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G48" s="38"/>
+      <c r="H48" s="38"/>
+    </row>
+    <row r="49" spans="1:8" ht="24" customHeight="1">
+      <c r="A49" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B41" s="30" t="inlineStr">
+      <c r="B49" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C41" s="38">
+      <c r="C49" s="38">
         <v>1</v>
       </c>
-      <c r="D41" s="38"/>
-      <c r="E41" s="35">
-        <f>IF(OR(C41="",C41=0),"",MIN(N(D41)/C41,1))</f>
-        <v/>
-      </c>
-      <c r="F41" s="30" t="str">
-        <f>IF(C41="","لم يُحدد",IF(C41=0,"لا ينطبق",IF(N(D41)&gt;=C41,"مكتمل",IF(N(D41)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G41" s="38"/>
-      <c r="H41" s="38"/>
-    </row>
-    <row r="42" spans="1:8" ht="24" customHeight="1">
-      <c r="A42" s="31" t="inlineStr">
+      <c r="D49" s="38"/>
+      <c r="E49" s="35">
+        <f>IF(OR(C49="",C49=0),"",MIN(N(D49)/C49,1))</f>
+        <v/>
+      </c>
+      <c r="F49" s="30" t="str">
+        <f>IF(C49="","لم يُحدد",IF(C49=0,"لا ينطبق",IF(N(D49)&gt;=C49,"مكتمل",IF(N(D49)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G49" s="38"/>
+      <c r="H49" s="38"/>
+    </row>
+    <row r="50" spans="1:8" ht="24" customHeight="1">
+      <c r="A50" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B42" s="30" t="inlineStr">
+      <c r="B50" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C42" s="38">
+      <c r="C50" s="38">
         <v>1</v>
       </c>
-      <c r="D42" s="38"/>
-      <c r="E42" s="35">
-        <f>IF(OR(C42="",C42=0),"",MIN(N(D42)/C42,1))</f>
-        <v/>
-      </c>
-      <c r="F42" s="30" t="str">
-        <f>IF(C42="","لم يُحدد",IF(C42=0,"لا ينطبق",IF(N(D42)&gt;=C42,"مكتمل",IF(N(D42)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G42" s="38"/>
-      <c r="H42" s="38"/>
-    </row>
-    <row r="43" spans="1:8" ht="26" customHeight="1">
-      <c r="A43" s="29" t="inlineStr">
+      <c r="D50" s="38"/>
+      <c r="E50" s="35">
+        <f>IF(OR(C50="",C50=0),"",MIN(N(D50)/C50,1))</f>
+        <v/>
+      </c>
+      <c r="F50" s="30" t="str">
+        <f>IF(C50="","لم يُحدد",IF(C50=0,"لا ينطبق",IF(N(D50)&gt;=C50,"مكتمل",IF(N(D50)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G50" s="38"/>
+      <c r="H50" s="38"/>
+    </row>
+    <row r="51" spans="1:8" ht="26" customHeight="1">
+      <c r="A51" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">نسبة إنجاز البرنامج</t>
         </is>
       </c>
-      <c r="B43" s="29"/>
-      <c r="C43" s="29"/>
-      <c r="D43" s="29"/>
-      <c r="E43" s="35">
-        <f>IFERROR(AVERAGE(E27:E42),0)</f>
+      <c r="B51" s="29"/>
+      <c r="C51" s="29"/>
+      <c r="D51" s="29"/>
+      <c r="E51" s="35">
+        <f>IFERROR(AVERAGE(E31:E50),0)</f>
         <v>0</v>
       </c>
     </row>
-    <row r="45" spans="1:8" ht="26" customHeight="1">
-      <c r="A45" s="97" t="str">
+    <row r="53" spans="1:8" ht="26" customHeight="1">
+      <c r="A53" s="97" t="str">
         <f>'الإعدادات واللجنة'!$B$7</f>
         <v/>
       </c>
-      <c r="B45" s="97"/>
-      <c r="C45" s="97"/>
-      <c r="D45" s="97"/>
-      <c r="E45" s="97"/>
-      <c r="F45" s="97"/>
-      <c r="G45" s="97"/>
-      <c r="H45" s="97"/>
-    </row>
-    <row r="46" spans="1:8" ht="28" customHeight="1">
-      <c r="A46" s="29" t="inlineStr">
+      <c r="B53" s="97"/>
+      <c r="C53" s="97"/>
+      <c r="D53" s="97"/>
+      <c r="E53" s="97"/>
+      <c r="F53" s="97"/>
+      <c r="G53" s="97"/>
+      <c r="H53" s="97"/>
+    </row>
+    <row r="54" spans="1:8" ht="28" customHeight="1">
+      <c r="A54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">الوثيقة</t>
         </is>
       </c>
-      <c r="B46" s="29" t="inlineStr">
+      <c r="B54" s="29" t="inlineStr">
         <is>
-          <t xml:space="preserve">العام</t>
+          <t xml:space="preserve">العام / الفصل</t>
         </is>
       </c>
-      <c r="C46" s="29" t="inlineStr">
+      <c r="C54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">المطلوب</t>
         </is>
       </c>
-      <c r="D46" s="29" t="inlineStr">
+      <c r="D54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">تم</t>
         </is>
       </c>
-      <c r="E46" s="29" t="inlineStr">
+      <c r="E54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">النسبة</t>
         </is>
       </c>
-      <c r="F46" s="29" t="inlineStr">
+      <c r="F54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">الحالة</t>
         </is>
       </c>
-      <c r="G46" s="29" t="inlineStr">
+      <c r="G54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">رابط الوثيقة</t>
         </is>
       </c>
-      <c r="H46" s="29" t="inlineStr">
+      <c r="H54" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">ملاحظات</t>
         </is>
       </c>
     </row>
-    <row r="47" spans="1:8" ht="24" customHeight="1">
-      <c r="A47" s="31" t="inlineStr">
+    <row r="55" spans="1:8" ht="24" customHeight="1">
+      <c r="A55" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">توصيف البرنامج (TP-151)</t>
         </is>
       </c>
-      <c r="B47" s="30" t="inlineStr">
+      <c r="B55" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
-      <c r="C47" s="38">
+      <c r="C55" s="38">
         <v>1</v>
       </c>
-      <c r="D47" s="38"/>
-      <c r="E47" s="35">
-        <f>IF(OR(C47="",C47=0),"",MIN(N(D47)/C47,1))</f>
-        <v/>
-      </c>
-      <c r="F47" s="30" t="str">
-        <f>IF(C47="","لم يُحدد",IF(C47=0,"لا ينطبق",IF(N(D47)&gt;=C47,"مكتمل",IF(N(D47)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G47" s="38"/>
-      <c r="H47" s="38"/>
-    </row>
-    <row r="48" spans="1:8" ht="24" customHeight="1">
-      <c r="A48" s="31" t="inlineStr">
+      <c r="D55" s="38"/>
+      <c r="E55" s="35">
+        <f>IF(OR(C55="",C55=0),"",MIN(N(D55)/C55,1))</f>
+        <v/>
+      </c>
+      <c r="F55" s="30" t="str">
+        <f>IF(C55="","لم يُحدد",IF(C55=0,"لا ينطبق",IF(N(D55)&gt;=C55,"مكتمل",IF(N(D55)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G55" s="38"/>
+      <c r="H55" s="38"/>
+    </row>
+    <row r="56" spans="1:8" ht="24" customHeight="1">
+      <c r="A56" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">توصيفات المقررات (TP-153)</t>
         </is>
       </c>
-      <c r="B48" s="30" t="inlineStr">
+      <c r="B56" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C48" s="38"/>
-      <c r="D48" s="38"/>
-      <c r="E48" s="35">
-        <f>IF(OR(C48="",C48=0),"",MIN(N(D48)/C48,1))</f>
-        <v/>
-      </c>
-      <c r="F48" s="30" t="str">
-        <f>IF(C48="","لم يُحدد",IF(C48=0,"لا ينطبق",IF(N(D48)&gt;=C48,"مكتمل",IF(N(D48)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G48" s="38"/>
-      <c r="H48" s="38"/>
-    </row>
-    <row r="49" spans="1:8" ht="24" customHeight="1">
-      <c r="A49" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">توصيف التدريب العملي (TP-155)</t>
-        </is>
-      </c>
-      <c r="B49" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C49" s="38"/>
-      <c r="D49" s="38"/>
-      <c r="E49" s="35">
-        <f>IF(OR(C49="",C49=0),"",MIN(N(D49)/C49,1))</f>
-        <v/>
-      </c>
-      <c r="F49" s="30" t="str">
-        <f>IF(C49="","لم يُحدد",IF(C49=0,"لا ينطبق",IF(N(D49)&gt;=C49,"مكتمل",IF(N(D49)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G49" s="38"/>
-      <c r="H49" s="38"/>
-    </row>
-    <row r="50" spans="1:8" ht="24" customHeight="1">
-      <c r="A50" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تقرير الاتساق مع الإطار الوطني (TP-150)</t>
-        </is>
-      </c>
-      <c r="B50" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C50" s="38">
-        <v>1</v>
-      </c>
-      <c r="D50" s="38"/>
-      <c r="E50" s="35">
-        <f>IF(OR(C50="",C50=0),"",MIN(N(D50)/C50,1))</f>
-        <v/>
-      </c>
-      <c r="F50" s="30" t="str">
-        <f>IF(C50="","لم يُحدد",IF(C50=0,"لا ينطبق",IF(N(D50)&gt;=C50,"مكتمل",IF(N(D50)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G50" s="38"/>
-      <c r="H50" s="38"/>
-    </row>
-    <row r="51" spans="1:8" ht="24" customHeight="1">
-      <c r="A51" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">خطة تقييم نواتج التعلم</t>
-        </is>
-      </c>
-      <c r="B51" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">مرة واحدة</t>
-        </is>
-      </c>
-      <c r="C51" s="38">
-        <v>1</v>
-      </c>
-      <c r="D51" s="38"/>
-      <c r="E51" s="35">
-        <f>IF(OR(C51="",C51=0),"",MIN(N(D51)/C51,1))</f>
-        <v/>
-      </c>
-      <c r="F51" s="30" t="str">
-        <f>IF(C51="","لم يُحدد",IF(C51=0,"لا ينطبق",IF(N(D51)&gt;=C51,"مكتمل",IF(N(D51)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G51" s="38"/>
-      <c r="H51" s="38"/>
-    </row>
-    <row r="52" spans="1:8" ht="24" customHeight="1">
-      <c r="A52" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
-        </is>
-      </c>
-      <c r="B52" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2024-2025</t>
-        </is>
-      </c>
-      <c r="C52" s="38">
-        <v>1</v>
-      </c>
-      <c r="D52" s="38"/>
-      <c r="E52" s="35">
-        <f>IF(OR(C52="",C52=0),"",MIN(N(D52)/C52,1))</f>
-        <v/>
-      </c>
-      <c r="F52" s="30" t="str">
-        <f>IF(C52="","لم يُحدد",IF(C52=0,"لا ينطبق",IF(N(D52)&gt;=C52,"مكتمل",IF(N(D52)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G52" s="38"/>
-      <c r="H52" s="38"/>
-    </row>
-    <row r="53" spans="1:8" ht="24" customHeight="1">
-      <c r="A53" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
-        </is>
-      </c>
-      <c r="B53" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-2026</t>
-        </is>
-      </c>
-      <c r="C53" s="38">
-        <v>1</v>
-      </c>
-      <c r="D53" s="38"/>
-      <c r="E53" s="35">
-        <f>IF(OR(C53="",C53=0),"",MIN(N(D53)/C53,1))</f>
-        <v/>
-      </c>
-      <c r="F53" s="30" t="str">
-        <f>IF(C53="","لم يُحدد",IF(C53=0,"لا ينطبق",IF(N(D53)&gt;=C53,"مكتمل",IF(N(D53)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G53" s="38"/>
-      <c r="H53" s="38"/>
-    </row>
-    <row r="54" spans="1:8" ht="24" customHeight="1">
-      <c r="A54" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
-        </is>
-      </c>
-      <c r="B54" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2024-2025</t>
-        </is>
-      </c>
-      <c r="C54" s="38"/>
-      <c r="D54" s="38"/>
-      <c r="E54" s="35">
-        <f>IF(OR(C54="",C54=0),"",MIN(N(D54)/C54,1))</f>
-        <v/>
-      </c>
-      <c r="F54" s="30" t="str">
-        <f>IF(C54="","لم يُحدد",IF(C54=0,"لا ينطبق",IF(N(D54)&gt;=C54,"مكتمل",IF(N(D54)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G54" s="38"/>
-      <c r="H54" s="38"/>
-    </row>
-    <row r="55" spans="1:8" ht="24" customHeight="1">
-      <c r="A55" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
-        </is>
-      </c>
-      <c r="B55" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2025-2026</t>
-        </is>
-      </c>
-      <c r="C55" s="38"/>
-      <c r="D55" s="38"/>
-      <c r="E55" s="35">
-        <f>IF(OR(C55="",C55=0),"",MIN(N(D55)/C55,1))</f>
-        <v/>
-      </c>
-      <c r="F55" s="30" t="str">
-        <f>IF(C55="","لم يُحدد",IF(C55=0,"لا ينطبق",IF(N(D55)&gt;=C55,"مكتمل",IF(N(D55)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G55" s="38"/>
-      <c r="H55" s="38"/>
-    </row>
-    <row r="56" spans="1:8" ht="24" customHeight="1">
-      <c r="A56" s="31" t="inlineStr">
-        <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
-        </is>
-      </c>
-      <c r="B56" s="30" t="inlineStr">
-        <is>
-          <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
       <c r="C56" s="38"/>
@@ -5323,12 +5315,12 @@
     <row r="57" spans="1:8" ht="24" customHeight="1">
       <c r="A57" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+          <t xml:space="preserve">توصيف التدريب العملي (TP-155)</t>
         </is>
       </c>
       <c r="B57" s="30" t="inlineStr">
         <is>
-          <t xml:space="preserve">2025-2026</t>
+          <t xml:space="preserve">مرة واحدة</t>
         </is>
       </c>
       <c r="C57" s="38"/>
@@ -5347,144 +5339,440 @@
     <row r="58" spans="1:8" ht="24" customHeight="1">
       <c r="A58" s="31" t="inlineStr">
         <is>
-          <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
+          <t xml:space="preserve">تقرير الاتساق مع الإطار الوطني (TP-150)</t>
         </is>
       </c>
       <c r="B58" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مرة واحدة</t>
+        </is>
+      </c>
+      <c r="C58" s="38">
+        <v>1</v>
+      </c>
+      <c r="D58" s="38"/>
+      <c r="E58" s="35">
+        <f>IF(OR(C58="",C58=0),"",MIN(N(D58)/C58,1))</f>
+        <v/>
+      </c>
+      <c r="F58" s="30" t="str">
+        <f>IF(C58="","لم يُحدد",IF(C58=0,"لا ينطبق",IF(N(D58)&gt;=C58,"مكتمل",IF(N(D58)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G58" s="38"/>
+      <c r="H58" s="38"/>
+    </row>
+    <row r="59" spans="1:8" ht="24" customHeight="1">
+      <c r="A59" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">خطة تقييم نواتج التعلم</t>
+        </is>
+      </c>
+      <c r="B59" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">مرة واحدة</t>
+        </is>
+      </c>
+      <c r="C59" s="38">
+        <v>1</v>
+      </c>
+      <c r="D59" s="38"/>
+      <c r="E59" s="35">
+        <f>IF(OR(C59="",C59=0),"",MIN(N(D59)/C59,1))</f>
+        <v/>
+      </c>
+      <c r="F59" s="30" t="str">
+        <f>IF(C59="","لم يُحدد",IF(C59=0,"لا ينطبق",IF(N(D59)&gt;=C59,"مكتمل",IF(N(D59)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G59" s="38"/>
+      <c r="H59" s="38"/>
+    </row>
+    <row r="60" spans="1:8" ht="24" customHeight="1">
+      <c r="A60" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
+        </is>
+      </c>
+      <c r="B60" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C58" s="38">
+      <c r="C60" s="38">
         <v>1</v>
       </c>
-      <c r="D58" s="38"/>
-      <c r="E58" s="35">
-        <f>IF(OR(C58="",C58=0),"",MIN(N(D58)/C58,1))</f>
-        <v/>
-      </c>
-      <c r="F58" s="30" t="str">
-        <f>IF(C58="","لم يُحدد",IF(C58=0,"لا ينطبق",IF(N(D58)&gt;=C58,"مكتمل",IF(N(D58)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G58" s="38"/>
-      <c r="H58" s="38"/>
-    </row>
-    <row r="59" spans="1:8" ht="24" customHeight="1">
-      <c r="A59" s="31" t="inlineStr">
+      <c r="D60" s="38"/>
+      <c r="E60" s="35">
+        <f>IF(OR(C60="",C60=0),"",MIN(N(D60)/C60,1))</f>
+        <v/>
+      </c>
+      <c r="F60" s="30" t="str">
+        <f>IF(C60="","لم يُحدد",IF(C60=0,"لا ينطبق",IF(N(D60)&gt;=C60,"مكتمل",IF(N(D60)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G60" s="38"/>
+      <c r="H60" s="38"/>
+    </row>
+    <row r="61" spans="1:8" ht="24" customHeight="1">
+      <c r="A61" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">التقرير السنوي للبرنامج (TP-152)</t>
+        </is>
+      </c>
+      <c r="B61" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026</t>
+        </is>
+      </c>
+      <c r="C61" s="38">
+        <v>1</v>
+      </c>
+      <c r="D61" s="38"/>
+      <c r="E61" s="35">
+        <f>IF(OR(C61="",C61=0),"",MIN(N(D61)/C61,1))</f>
+        <v/>
+      </c>
+      <c r="F61" s="30" t="str">
+        <f>IF(C61="","لم يُحدد",IF(C61=0,"لا ينطبق",IF(N(D61)&gt;=C61,"مكتمل",IF(N(D61)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G61" s="38"/>
+      <c r="H61" s="38"/>
+    </row>
+    <row r="62" spans="1:8" ht="24" customHeight="1">
+      <c r="A62" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B62" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C62" s="38"/>
+      <c r="D62" s="38"/>
+      <c r="E62" s="35">
+        <f>IF(OR(C62="",C62=0),"",MIN(N(D62)/C62,1))</f>
+        <v/>
+      </c>
+      <c r="F62" s="30" t="str">
+        <f>IF(C62="","لم يُحدد",IF(C62=0,"لا ينطبق",IF(N(D62)&gt;=C62,"مكتمل",IF(N(D62)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G62" s="38"/>
+      <c r="H62" s="38"/>
+    </row>
+    <row r="63" spans="1:8" ht="24" customHeight="1">
+      <c r="A63" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B63" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C63" s="38"/>
+      <c r="D63" s="38"/>
+      <c r="E63" s="35">
+        <f>IF(OR(C63="",C63=0),"",MIN(N(D63)/C63,1))</f>
+        <v/>
+      </c>
+      <c r="F63" s="30" t="str">
+        <f>IF(C63="","لم يُحدد",IF(C63=0,"لا ينطبق",IF(N(D63)&gt;=C63,"مكتمل",IF(N(D63)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G63" s="38"/>
+      <c r="H63" s="38"/>
+    </row>
+    <row r="64" spans="1:8" ht="24" customHeight="1">
+      <c r="A64" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B64" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C64" s="38"/>
+      <c r="D64" s="38"/>
+      <c r="E64" s="35">
+        <f>IF(OR(C64="",C64=0),"",MIN(N(D64)/C64,1))</f>
+        <v/>
+      </c>
+      <c r="F64" s="30" t="str">
+        <f>IF(C64="","لم يُحدد",IF(C64=0,"لا ينطبق",IF(N(D64)&gt;=C64,"مكتمل",IF(N(D64)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G64" s="38"/>
+      <c r="H64" s="38"/>
+    </row>
+    <row r="65" spans="1:8" ht="24" customHeight="1">
+      <c r="A65" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقارير المقررات (TP-154)</t>
+        </is>
+      </c>
+      <c r="B65" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C65" s="38"/>
+      <c r="D65" s="38"/>
+      <c r="E65" s="35">
+        <f>IF(OR(C65="",C65=0),"",MIN(N(D65)/C65,1))</f>
+        <v/>
+      </c>
+      <c r="F65" s="30" t="str">
+        <f>IF(C65="","لم يُحدد",IF(C65=0,"لا ينطبق",IF(N(D65)&gt;=C65,"مكتمل",IF(N(D65)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G65" s="38"/>
+      <c r="H65" s="38"/>
+    </row>
+    <row r="66" spans="1:8" ht="24" customHeight="1">
+      <c r="A66" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B66" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C66" s="38"/>
+      <c r="D66" s="38"/>
+      <c r="E66" s="35">
+        <f>IF(OR(C66="",C66=0),"",MIN(N(D66)/C66,1))</f>
+        <v/>
+      </c>
+      <c r="F66" s="30" t="str">
+        <f>IF(C66="","لم يُحدد",IF(C66=0,"لا ينطبق",IF(N(D66)&gt;=C66,"مكتمل",IF(N(D66)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G66" s="38"/>
+      <c r="H66" s="38"/>
+    </row>
+    <row r="67" spans="1:8" ht="24" customHeight="1">
+      <c r="A67" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B67" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C67" s="38"/>
+      <c r="D67" s="38"/>
+      <c r="E67" s="35">
+        <f>IF(OR(C67="",C67=0),"",MIN(N(D67)/C67,1))</f>
+        <v/>
+      </c>
+      <c r="F67" s="30" t="str">
+        <f>IF(C67="","لم يُحدد",IF(C67=0,"لا ينطبق",IF(N(D67)&gt;=C67,"مكتمل",IF(N(D67)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G67" s="38"/>
+      <c r="H67" s="38"/>
+    </row>
+    <row r="68" spans="1:8" ht="24" customHeight="1">
+      <c r="A68" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B68" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الأول</t>
+        </is>
+      </c>
+      <c r="C68" s="38"/>
+      <c r="D68" s="38"/>
+      <c r="E68" s="35">
+        <f>IF(OR(C68="",C68=0),"",MIN(N(D68)/C68,1))</f>
+        <v/>
+      </c>
+      <c r="F68" s="30" t="str">
+        <f>IF(C68="","لم يُحدد",IF(C68=0,"لا ينطبق",IF(N(D68)&gt;=C68,"مكتمل",IF(N(D68)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G68" s="38"/>
+      <c r="H68" s="38"/>
+    </row>
+    <row r="69" spans="1:8" ht="24" customHeight="1">
+      <c r="A69" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير التدريب العملي (TP-156)</t>
+        </is>
+      </c>
+      <c r="B69" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2025-2026 – الفصل الثاني</t>
+        </is>
+      </c>
+      <c r="C69" s="38"/>
+      <c r="D69" s="38"/>
+      <c r="E69" s="35">
+        <f>IF(OR(C69="",C69=0),"",MIN(N(D69)/C69,1))</f>
+        <v/>
+      </c>
+      <c r="F69" s="30" t="str">
+        <f>IF(C69="","لم يُحدد",IF(C69=0,"لا ينطبق",IF(N(D69)&gt;=C69,"مكتمل",IF(N(D69)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G69" s="38"/>
+      <c r="H69" s="38"/>
+    </row>
+    <row r="70" spans="1:8" ht="24" customHeight="1">
+      <c r="A70" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
         </is>
       </c>
-      <c r="B59" s="30" t="inlineStr">
+      <c r="B70" s="30" t="inlineStr">
+        <is>
+          <t xml:space="preserve">2024-2025</t>
+        </is>
+      </c>
+      <c r="C70" s="38">
+        <v>1</v>
+      </c>
+      <c r="D70" s="38"/>
+      <c r="E70" s="35">
+        <f>IF(OR(C70="",C70=0),"",MIN(N(D70)/C70,1))</f>
+        <v/>
+      </c>
+      <c r="F70" s="30" t="str">
+        <f>IF(C70="","لم يُحدد",IF(C70=0,"لا ينطبق",IF(N(D70)&gt;=C70,"مكتمل",IF(N(D70)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G70" s="38"/>
+      <c r="H70" s="38"/>
+    </row>
+    <row r="71" spans="1:8" ht="24" customHeight="1">
+      <c r="A71" s="31" t="inlineStr">
+        <is>
+          <t xml:space="preserve">تقرير قياس نواتج التعلم</t>
+        </is>
+      </c>
+      <c r="B71" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C59" s="38">
+      <c r="C71" s="38">
         <v>1</v>
       </c>
-      <c r="D59" s="38"/>
-      <c r="E59" s="35">
-        <f>IF(OR(C59="",C59=0),"",MIN(N(D59)/C59,1))</f>
-        <v/>
-      </c>
-      <c r="F59" s="30" t="str">
-        <f>IF(C59="","لم يُحدد",IF(C59=0,"لا ينطبق",IF(N(D59)&gt;=C59,"مكتمل",IF(N(D59)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G59" s="38"/>
-      <c r="H59" s="38"/>
-    </row>
-    <row r="60" spans="1:8" ht="24" customHeight="1">
-      <c r="A60" s="31" t="inlineStr">
+      <c r="D71" s="38"/>
+      <c r="E71" s="35">
+        <f>IF(OR(C71="",C71=0),"",MIN(N(D71)/C71,1))</f>
+        <v/>
+      </c>
+      <c r="F71" s="30" t="str">
+        <f>IF(C71="","لم يُحدد",IF(C71=0,"لا ينطبق",IF(N(D71)&gt;=C71,"مكتمل",IF(N(D71)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G71" s="38"/>
+      <c r="H71" s="38"/>
+    </row>
+    <row r="72" spans="1:8" ht="24" customHeight="1">
+      <c r="A72" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B60" s="30" t="inlineStr">
+      <c r="B72" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2023-2024</t>
         </is>
       </c>
-      <c r="C60" s="38">
+      <c r="C72" s="38">
         <v>1</v>
       </c>
-      <c r="D60" s="38"/>
-      <c r="E60" s="35">
-        <f>IF(OR(C60="",C60=0),"",MIN(N(D60)/C60,1))</f>
-        <v/>
-      </c>
-      <c r="F60" s="30" t="str">
-        <f>IF(C60="","لم يُحدد",IF(C60=0,"لا ينطبق",IF(N(D60)&gt;=C60,"مكتمل",IF(N(D60)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G60" s="38"/>
-      <c r="H60" s="38"/>
-    </row>
-    <row r="61" spans="1:8" ht="24" customHeight="1">
-      <c r="A61" s="31" t="inlineStr">
+      <c r="D72" s="38"/>
+      <c r="E72" s="35">
+        <f>IF(OR(C72="",C72=0),"",MIN(N(D72)/C72,1))</f>
+        <v/>
+      </c>
+      <c r="F72" s="30" t="str">
+        <f>IF(C72="","لم يُحدد",IF(C72=0,"لا ينطبق",IF(N(D72)&gt;=C72,"مكتمل",IF(N(D72)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G72" s="38"/>
+      <c r="H72" s="38"/>
+    </row>
+    <row r="73" spans="1:8" ht="24" customHeight="1">
+      <c r="A73" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B61" s="30" t="inlineStr">
+      <c r="B73" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2024-2025</t>
         </is>
       </c>
-      <c r="C61" s="38">
+      <c r="C73" s="38">
         <v>1</v>
       </c>
-      <c r="D61" s="38"/>
-      <c r="E61" s="35">
-        <f>IF(OR(C61="",C61=0),"",MIN(N(D61)/C61,1))</f>
-        <v/>
-      </c>
-      <c r="F61" s="30" t="str">
-        <f>IF(C61="","لم يُحدد",IF(C61=0,"لا ينطبق",IF(N(D61)&gt;=C61,"مكتمل",IF(N(D61)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G61" s="38"/>
-      <c r="H61" s="38"/>
-    </row>
-    <row r="62" spans="1:8" ht="24" customHeight="1">
-      <c r="A62" s="31" t="inlineStr">
+      <c r="D73" s="38"/>
+      <c r="E73" s="35">
+        <f>IF(OR(C73="",C73=0),"",MIN(N(D73)/C73,1))</f>
+        <v/>
+      </c>
+      <c r="F73" s="30" t="str">
+        <f>IF(C73="","لم يُحدد",IF(C73=0,"لا ينطبق",IF(N(D73)&gt;=C73,"مكتمل",IF(N(D73)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G73" s="38"/>
+      <c r="H73" s="38"/>
+    </row>
+    <row r="74" spans="1:8" ht="24" customHeight="1">
+      <c r="A74" s="31" t="inlineStr">
         <is>
           <t xml:space="preserve">مؤشرات الأداء مع المقارنة المرجعية</t>
         </is>
       </c>
-      <c r="B62" s="30" t="inlineStr">
+      <c r="B74" s="30" t="inlineStr">
         <is>
           <t xml:space="preserve">2025-2026</t>
         </is>
       </c>
-      <c r="C62" s="38">
+      <c r="C74" s="38">
         <v>1</v>
       </c>
-      <c r="D62" s="38"/>
-      <c r="E62" s="35">
-        <f>IF(OR(C62="",C62=0),"",MIN(N(D62)/C62,1))</f>
-        <v/>
-      </c>
-      <c r="F62" s="30" t="str">
-        <f>IF(C62="","لم يُحدد",IF(C62=0,"لا ينطبق",IF(N(D62)&gt;=C62,"مكتمل",IF(N(D62)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
-        <v/>
-      </c>
-      <c r="G62" s="38"/>
-      <c r="H62" s="38"/>
-    </row>
-    <row r="63" spans="1:8" ht="26" customHeight="1">
-      <c r="A63" s="29" t="inlineStr">
+      <c r="D74" s="38"/>
+      <c r="E74" s="35">
+        <f>IF(OR(C74="",C74=0),"",MIN(N(D74)/C74,1))</f>
+        <v/>
+      </c>
+      <c r="F74" s="30" t="str">
+        <f>IF(C74="","لم يُحدد",IF(C74=0,"لا ينطبق",IF(N(D74)&gt;=C74,"مكتمل",IF(N(D74)&gt;0,"قيد التحديث","لم يبدأ"))))</f>
+        <v/>
+      </c>
+      <c r="G74" s="38"/>
+      <c r="H74" s="38"/>
+    </row>
+    <row r="75" spans="1:8" ht="26" customHeight="1">
+      <c r="A75" s="29" t="inlineStr">
         <is>
           <t xml:space="preserve">نسبة إنجاز البرنامج</t>
         </is>
       </c>
-      <c r="B63" s="29"/>
-      <c r="C63" s="29"/>
-      <c r="D63" s="29"/>
-      <c r="E63" s="35">
-        <f>IFERROR(AVERAGE(E47:E62),0)</f>
+      <c r="B75" s="29"/>
+      <c r="C75" s="29"/>
+      <c r="D75" s="29"/>
+      <c r="E75" s="35">
+        <f>IFERROR(AVERAGE(E55:E74),0)</f>
         <v>0</v>
       </c>
     </row>
@@ -5492,15 +5780,15 @@
   <mergeCells count="9">
     <mergeCell ref="A1:H1"/>
     <mergeCell ref="A2:H2"/>
+    <mergeCell ref="A3:D3"/>
     <mergeCell ref="A5:H5"/>
-    <mergeCell ref="A23:D23"/>
-    <mergeCell ref="A25:H25"/>
-    <mergeCell ref="A43:D43"/>
-    <mergeCell ref="A45:H45"/>
-    <mergeCell ref="A63:D63"/>
-    <mergeCell ref="A3:D3"/>
+    <mergeCell ref="A27:D27"/>
+    <mergeCell ref="A29:H29"/>
+    <mergeCell ref="A51:D51"/>
+    <mergeCell ref="A53:H53"/>
+    <mergeCell ref="A75:D75"/>
   </mergeCells>
-  <conditionalFormatting sqref="F7:F22">
+  <conditionalFormatting sqref="F7:F26">
     <cfRule type="cellIs" dxfId="26" priority="10" operator="equal">
       <formula>"مكتمل"</formula>
     </cfRule>
@@ -5511,7 +5799,7 @@
       <formula>"لم يبدأ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F27:F42">
+  <conditionalFormatting sqref="F31:F50">
     <cfRule type="cellIs" dxfId="26" priority="13" operator="equal">
       <formula>"مكتمل"</formula>
     </cfRule>
@@ -5522,7 +5810,7 @@
       <formula>"لم يبدأ"</formula>
     </cfRule>
   </conditionalFormatting>
-  <conditionalFormatting sqref="F47:F62">
+  <conditionalFormatting sqref="F55:F74">
     <cfRule type="cellIs" dxfId="26" priority="16" operator="equal">
       <formula>"مكتمل"</formula>
     </cfRule>
@@ -5534,7 +5822,7 @@
     </cfRule>
   </conditionalFormatting>
   <dataValidations count="1">
-    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="قيمة غير صحيحة" error="اكتبي رقماً (0 أو أكثر)" sqref="C7:D22 C27:D42 C47:D62">
+    <dataValidation type="decimal" operator="greaterThanOrEqual" allowBlank="1" showErrorMessage="1" errorTitle="قيمة غير صحيحة" error="اكتبي رقماً (0 أو أكثر)" sqref="C7:D26 C31:D50 C55:D74">
       <formula1>0</formula1>
     </dataValidation>
   </dataValidations>

</xml_diff>